<commit_message>
Atualiza preços de 2026-09-13
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G406"/>
+  <dimension ref="A1:G421"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9292,9 +9292,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D392" t="inlineStr"/>
-      <c r="E392" t="inlineStr"/>
-      <c r="F392" t="inlineStr"/>
       <c r="G392" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9317,9 +9314,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D393" t="inlineStr"/>
-      <c r="E393" t="inlineStr"/>
-      <c r="F393" t="inlineStr"/>
       <c r="G393" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9342,9 +9336,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D394" t="inlineStr"/>
-      <c r="E394" t="inlineStr"/>
-      <c r="F394" t="inlineStr"/>
       <c r="G394" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9367,9 +9358,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D395" t="inlineStr"/>
-      <c r="E395" t="inlineStr"/>
-      <c r="F395" t="inlineStr"/>
       <c r="G395" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9392,9 +9380,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D396" t="inlineStr"/>
-      <c r="E396" t="inlineStr"/>
-      <c r="F396" t="inlineStr"/>
       <c r="G396" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9417,9 +9402,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D397" t="inlineStr"/>
-      <c r="E397" t="inlineStr"/>
-      <c r="F397" t="inlineStr"/>
       <c r="G397" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9442,9 +9424,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D398" t="inlineStr"/>
-      <c r="E398" t="inlineStr"/>
-      <c r="F398" t="inlineStr"/>
       <c r="G398" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9467,9 +9446,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D399" t="inlineStr"/>
-      <c r="E399" t="inlineStr"/>
-      <c r="F399" t="inlineStr"/>
       <c r="G399" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9492,9 +9468,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D400" t="inlineStr"/>
-      <c r="E400" t="inlineStr"/>
-      <c r="F400" t="inlineStr"/>
       <c r="G400" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9517,9 +9490,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D401" t="inlineStr"/>
-      <c r="E401" t="inlineStr"/>
-      <c r="F401" t="inlineStr"/>
       <c r="G401" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9542,9 +9512,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D402" t="inlineStr"/>
-      <c r="E402" t="inlineStr"/>
-      <c r="F402" t="inlineStr"/>
       <c r="G402" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9567,9 +9534,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D403" t="inlineStr"/>
-      <c r="E403" t="inlineStr"/>
-      <c r="F403" t="inlineStr"/>
       <c r="G403" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9592,9 +9556,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D404" t="inlineStr"/>
-      <c r="E404" t="inlineStr"/>
-      <c r="F404" t="inlineStr"/>
       <c r="G404" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9617,9 +9578,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D405" t="inlineStr"/>
-      <c r="E405" t="inlineStr"/>
-      <c r="F405" t="inlineStr"/>
       <c r="G405" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9642,10 +9600,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D406" t="inlineStr"/>
-      <c r="E406" t="inlineStr"/>
-      <c r="F406" t="inlineStr"/>
       <c r="G406" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr"/>
+      <c r="E407" t="inlineStr"/>
+      <c r="F407" t="inlineStr"/>
+      <c r="G407" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr"/>
+      <c r="E408" t="inlineStr"/>
+      <c r="F408" t="inlineStr"/>
+      <c r="G408" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr"/>
+      <c r="E409" t="inlineStr"/>
+      <c r="F409" t="inlineStr"/>
+      <c r="G409" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr"/>
+      <c r="E410" t="inlineStr"/>
+      <c r="F410" t="inlineStr"/>
+      <c r="G410" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr"/>
+      <c r="E411" t="inlineStr"/>
+      <c r="F411" t="inlineStr"/>
+      <c r="G411" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr"/>
+      <c r="E412" t="inlineStr"/>
+      <c r="F412" t="inlineStr"/>
+      <c r="G412" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr"/>
+      <c r="E413" t="inlineStr"/>
+      <c r="F413" t="inlineStr"/>
+      <c r="G413" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr"/>
+      <c r="E414" t="inlineStr"/>
+      <c r="F414" t="inlineStr"/>
+      <c r="G414" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr"/>
+      <c r="E415" t="inlineStr"/>
+      <c r="F415" t="inlineStr"/>
+      <c r="G415" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr"/>
+      <c r="E416" t="inlineStr"/>
+      <c r="F416" t="inlineStr"/>
+      <c r="G416" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr"/>
+      <c r="E417" t="inlineStr"/>
+      <c r="F417" t="inlineStr"/>
+      <c r="G417" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr"/>
+      <c r="E418" t="inlineStr"/>
+      <c r="F418" t="inlineStr"/>
+      <c r="G418" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr"/>
+      <c r="E419" t="inlineStr"/>
+      <c r="F419" t="inlineStr"/>
+      <c r="G419" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr"/>
+      <c r="E420" t="inlineStr"/>
+      <c r="F420" t="inlineStr"/>
+      <c r="G420" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr"/>
+      <c r="E421" t="inlineStr"/>
+      <c r="F421" t="inlineStr"/>
+      <c r="G421" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-09-14
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G421"/>
+  <dimension ref="A1:G436"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9622,9 +9622,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D407" t="inlineStr"/>
-      <c r="E407" t="inlineStr"/>
-      <c r="F407" t="inlineStr"/>
       <c r="G407" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9647,9 +9644,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D408" t="inlineStr"/>
-      <c r="E408" t="inlineStr"/>
-      <c r="F408" t="inlineStr"/>
       <c r="G408" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9672,9 +9666,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D409" t="inlineStr"/>
-      <c r="E409" t="inlineStr"/>
-      <c r="F409" t="inlineStr"/>
       <c r="G409" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9697,9 +9688,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D410" t="inlineStr"/>
-      <c r="E410" t="inlineStr"/>
-      <c r="F410" t="inlineStr"/>
       <c r="G410" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9722,9 +9710,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D411" t="inlineStr"/>
-      <c r="E411" t="inlineStr"/>
-      <c r="F411" t="inlineStr"/>
       <c r="G411" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9747,9 +9732,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D412" t="inlineStr"/>
-      <c r="E412" t="inlineStr"/>
-      <c r="F412" t="inlineStr"/>
       <c r="G412" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9772,9 +9754,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D413" t="inlineStr"/>
-      <c r="E413" t="inlineStr"/>
-      <c r="F413" t="inlineStr"/>
       <c r="G413" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9797,9 +9776,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D414" t="inlineStr"/>
-      <c r="E414" t="inlineStr"/>
-      <c r="F414" t="inlineStr"/>
       <c r="G414" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9822,9 +9798,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D415" t="inlineStr"/>
-      <c r="E415" t="inlineStr"/>
-      <c r="F415" t="inlineStr"/>
       <c r="G415" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9847,9 +9820,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D416" t="inlineStr"/>
-      <c r="E416" t="inlineStr"/>
-      <c r="F416" t="inlineStr"/>
       <c r="G416" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9872,9 +9842,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D417" t="inlineStr"/>
-      <c r="E417" t="inlineStr"/>
-      <c r="F417" t="inlineStr"/>
       <c r="G417" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9897,9 +9864,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D418" t="inlineStr"/>
-      <c r="E418" t="inlineStr"/>
-      <c r="F418" t="inlineStr"/>
       <c r="G418" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9922,9 +9886,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D419" t="inlineStr"/>
-      <c r="E419" t="inlineStr"/>
-      <c r="F419" t="inlineStr"/>
       <c r="G419" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9947,9 +9908,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D420" t="inlineStr"/>
-      <c r="E420" t="inlineStr"/>
-      <c r="F420" t="inlineStr"/>
       <c r="G420" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9972,10 +9930,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D421" t="inlineStr"/>
-      <c r="E421" t="inlineStr"/>
-      <c r="F421" t="inlineStr"/>
       <c r="G421" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr"/>
+      <c r="E422" t="inlineStr"/>
+      <c r="F422" t="inlineStr"/>
+      <c r="G422" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr"/>
+      <c r="E423" t="inlineStr"/>
+      <c r="F423" t="inlineStr"/>
+      <c r="G423" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr"/>
+      <c r="E424" t="inlineStr"/>
+      <c r="F424" t="inlineStr"/>
+      <c r="G424" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr"/>
+      <c r="E425" t="inlineStr"/>
+      <c r="F425" t="inlineStr"/>
+      <c r="G425" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr"/>
+      <c r="E426" t="inlineStr"/>
+      <c r="F426" t="inlineStr"/>
+      <c r="G426" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr"/>
+      <c r="E427" t="inlineStr"/>
+      <c r="F427" t="inlineStr"/>
+      <c r="G427" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr"/>
+      <c r="E428" t="inlineStr"/>
+      <c r="F428" t="inlineStr"/>
+      <c r="G428" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr"/>
+      <c r="E429" t="inlineStr"/>
+      <c r="F429" t="inlineStr"/>
+      <c r="G429" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr"/>
+      <c r="E430" t="inlineStr"/>
+      <c r="F430" t="inlineStr"/>
+      <c r="G430" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr"/>
+      <c r="E431" t="inlineStr"/>
+      <c r="F431" t="inlineStr"/>
+      <c r="G431" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr"/>
+      <c r="E432" t="inlineStr"/>
+      <c r="F432" t="inlineStr"/>
+      <c r="G432" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr"/>
+      <c r="E433" t="inlineStr"/>
+      <c r="F433" t="inlineStr"/>
+      <c r="G433" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr"/>
+      <c r="E434" t="inlineStr"/>
+      <c r="F434" t="inlineStr"/>
+      <c r="G434" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr"/>
+      <c r="E435" t="inlineStr"/>
+      <c r="F435" t="inlineStr"/>
+      <c r="G435" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr"/>
+      <c r="E436" t="inlineStr"/>
+      <c r="F436" t="inlineStr"/>
+      <c r="G436" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-09-15
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G436"/>
+  <dimension ref="A1:G451"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9952,9 +9952,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D422" t="inlineStr"/>
-      <c r="E422" t="inlineStr"/>
-      <c r="F422" t="inlineStr"/>
       <c r="G422" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9977,9 +9974,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D423" t="inlineStr"/>
-      <c r="E423" t="inlineStr"/>
-      <c r="F423" t="inlineStr"/>
       <c r="G423" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10002,9 +9996,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D424" t="inlineStr"/>
-      <c r="E424" t="inlineStr"/>
-      <c r="F424" t="inlineStr"/>
       <c r="G424" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10027,9 +10018,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D425" t="inlineStr"/>
-      <c r="E425" t="inlineStr"/>
-      <c r="F425" t="inlineStr"/>
       <c r="G425" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10052,9 +10040,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D426" t="inlineStr"/>
-      <c r="E426" t="inlineStr"/>
-      <c r="F426" t="inlineStr"/>
       <c r="G426" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10077,9 +10062,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D427" t="inlineStr"/>
-      <c r="E427" t="inlineStr"/>
-      <c r="F427" t="inlineStr"/>
       <c r="G427" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10102,9 +10084,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D428" t="inlineStr"/>
-      <c r="E428" t="inlineStr"/>
-      <c r="F428" t="inlineStr"/>
       <c r="G428" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10127,9 +10106,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D429" t="inlineStr"/>
-      <c r="E429" t="inlineStr"/>
-      <c r="F429" t="inlineStr"/>
       <c r="G429" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10152,9 +10128,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D430" t="inlineStr"/>
-      <c r="E430" t="inlineStr"/>
-      <c r="F430" t="inlineStr"/>
       <c r="G430" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10177,9 +10150,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D431" t="inlineStr"/>
-      <c r="E431" t="inlineStr"/>
-      <c r="F431" t="inlineStr"/>
       <c r="G431" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10202,9 +10172,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D432" t="inlineStr"/>
-      <c r="E432" t="inlineStr"/>
-      <c r="F432" t="inlineStr"/>
       <c r="G432" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10227,9 +10194,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D433" t="inlineStr"/>
-      <c r="E433" t="inlineStr"/>
-      <c r="F433" t="inlineStr"/>
       <c r="G433" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10252,9 +10216,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D434" t="inlineStr"/>
-      <c r="E434" t="inlineStr"/>
-      <c r="F434" t="inlineStr"/>
       <c r="G434" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10277,9 +10238,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D435" t="inlineStr"/>
-      <c r="E435" t="inlineStr"/>
-      <c r="F435" t="inlineStr"/>
       <c r="G435" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10302,10 +10260,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D436" t="inlineStr"/>
-      <c r="E436" t="inlineStr"/>
-      <c r="F436" t="inlineStr"/>
       <c r="G436" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr"/>
+      <c r="E437" t="inlineStr"/>
+      <c r="F437" t="inlineStr"/>
+      <c r="G437" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr"/>
+      <c r="E438" t="inlineStr"/>
+      <c r="F438" t="inlineStr"/>
+      <c r="G438" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr"/>
+      <c r="E439" t="inlineStr"/>
+      <c r="F439" t="inlineStr"/>
+      <c r="G439" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr"/>
+      <c r="E440" t="inlineStr"/>
+      <c r="F440" t="inlineStr"/>
+      <c r="G440" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr"/>
+      <c r="E441" t="inlineStr"/>
+      <c r="F441" t="inlineStr"/>
+      <c r="G441" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr"/>
+      <c r="E442" t="inlineStr"/>
+      <c r="F442" t="inlineStr"/>
+      <c r="G442" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr"/>
+      <c r="E443" t="inlineStr"/>
+      <c r="F443" t="inlineStr"/>
+      <c r="G443" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr"/>
+      <c r="E444" t="inlineStr"/>
+      <c r="F444" t="inlineStr"/>
+      <c r="G444" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr"/>
+      <c r="E445" t="inlineStr"/>
+      <c r="F445" t="inlineStr"/>
+      <c r="G445" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr"/>
+      <c r="E446" t="inlineStr"/>
+      <c r="F446" t="inlineStr"/>
+      <c r="G446" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr"/>
+      <c r="E447" t="inlineStr"/>
+      <c r="F447" t="inlineStr"/>
+      <c r="G447" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr"/>
+      <c r="E448" t="inlineStr"/>
+      <c r="F448" t="inlineStr"/>
+      <c r="G448" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr"/>
+      <c r="E449" t="inlineStr"/>
+      <c r="F449" t="inlineStr"/>
+      <c r="G449" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr"/>
+      <c r="E450" t="inlineStr"/>
+      <c r="F450" t="inlineStr"/>
+      <c r="G450" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr"/>
+      <c r="E451" t="inlineStr"/>
+      <c r="F451" t="inlineStr"/>
+      <c r="G451" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-09-16
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G451"/>
+  <dimension ref="A1:G466"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10282,9 +10282,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D437" t="inlineStr"/>
-      <c r="E437" t="inlineStr"/>
-      <c r="F437" t="inlineStr"/>
       <c r="G437" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10307,9 +10304,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D438" t="inlineStr"/>
-      <c r="E438" t="inlineStr"/>
-      <c r="F438" t="inlineStr"/>
       <c r="G438" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10332,9 +10326,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D439" t="inlineStr"/>
-      <c r="E439" t="inlineStr"/>
-      <c r="F439" t="inlineStr"/>
       <c r="G439" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10357,9 +10348,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D440" t="inlineStr"/>
-      <c r="E440" t="inlineStr"/>
-      <c r="F440" t="inlineStr"/>
       <c r="G440" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10382,9 +10370,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D441" t="inlineStr"/>
-      <c r="E441" t="inlineStr"/>
-      <c r="F441" t="inlineStr"/>
       <c r="G441" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10407,9 +10392,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D442" t="inlineStr"/>
-      <c r="E442" t="inlineStr"/>
-      <c r="F442" t="inlineStr"/>
       <c r="G442" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10432,9 +10414,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D443" t="inlineStr"/>
-      <c r="E443" t="inlineStr"/>
-      <c r="F443" t="inlineStr"/>
       <c r="G443" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10457,9 +10436,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D444" t="inlineStr"/>
-      <c r="E444" t="inlineStr"/>
-      <c r="F444" t="inlineStr"/>
       <c r="G444" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10482,9 +10458,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D445" t="inlineStr"/>
-      <c r="E445" t="inlineStr"/>
-      <c r="F445" t="inlineStr"/>
       <c r="G445" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10507,9 +10480,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D446" t="inlineStr"/>
-      <c r="E446" t="inlineStr"/>
-      <c r="F446" t="inlineStr"/>
       <c r="G446" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10532,9 +10502,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D447" t="inlineStr"/>
-      <c r="E447" t="inlineStr"/>
-      <c r="F447" t="inlineStr"/>
       <c r="G447" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10557,9 +10524,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D448" t="inlineStr"/>
-      <c r="E448" t="inlineStr"/>
-      <c r="F448" t="inlineStr"/>
       <c r="G448" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10582,9 +10546,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D449" t="inlineStr"/>
-      <c r="E449" t="inlineStr"/>
-      <c r="F449" t="inlineStr"/>
       <c r="G449" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10607,9 +10568,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D450" t="inlineStr"/>
-      <c r="E450" t="inlineStr"/>
-      <c r="F450" t="inlineStr"/>
       <c r="G450" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10632,10 +10590,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D451" t="inlineStr"/>
-      <c r="E451" t="inlineStr"/>
-      <c r="F451" t="inlineStr"/>
       <c r="G451" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr"/>
+      <c r="E452" t="inlineStr"/>
+      <c r="F452" t="inlineStr"/>
+      <c r="G452" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr"/>
+      <c r="E453" t="inlineStr"/>
+      <c r="F453" t="inlineStr"/>
+      <c r="G453" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr"/>
+      <c r="E454" t="inlineStr"/>
+      <c r="F454" t="inlineStr"/>
+      <c r="G454" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr"/>
+      <c r="E455" t="inlineStr"/>
+      <c r="F455" t="inlineStr"/>
+      <c r="G455" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr"/>
+      <c r="E456" t="inlineStr"/>
+      <c r="F456" t="inlineStr"/>
+      <c r="G456" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr"/>
+      <c r="E457" t="inlineStr"/>
+      <c r="F457" t="inlineStr"/>
+      <c r="G457" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D458" t="inlineStr"/>
+      <c r="E458" t="inlineStr"/>
+      <c r="F458" t="inlineStr"/>
+      <c r="G458" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr"/>
+      <c r="E459" t="inlineStr"/>
+      <c r="F459" t="inlineStr"/>
+      <c r="G459" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr"/>
+      <c r="E460" t="inlineStr"/>
+      <c r="F460" t="inlineStr"/>
+      <c r="G460" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr"/>
+      <c r="E461" t="inlineStr"/>
+      <c r="F461" t="inlineStr"/>
+      <c r="G461" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr"/>
+      <c r="E462" t="inlineStr"/>
+      <c r="F462" t="inlineStr"/>
+      <c r="G462" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr"/>
+      <c r="E463" t="inlineStr"/>
+      <c r="F463" t="inlineStr"/>
+      <c r="G463" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr"/>
+      <c r="E464" t="inlineStr"/>
+      <c r="F464" t="inlineStr"/>
+      <c r="G464" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr"/>
+      <c r="E465" t="inlineStr"/>
+      <c r="F465" t="inlineStr"/>
+      <c r="G465" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr"/>
+      <c r="E466" t="inlineStr"/>
+      <c r="F466" t="inlineStr"/>
+      <c r="G466" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-09-17
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G466"/>
+  <dimension ref="A1:G481"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10612,9 +10612,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D452" t="inlineStr"/>
-      <c r="E452" t="inlineStr"/>
-      <c r="F452" t="inlineStr"/>
       <c r="G452" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10637,9 +10634,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D453" t="inlineStr"/>
-      <c r="E453" t="inlineStr"/>
-      <c r="F453" t="inlineStr"/>
       <c r="G453" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10662,9 +10656,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D454" t="inlineStr"/>
-      <c r="E454" t="inlineStr"/>
-      <c r="F454" t="inlineStr"/>
       <c r="G454" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10687,9 +10678,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D455" t="inlineStr"/>
-      <c r="E455" t="inlineStr"/>
-      <c r="F455" t="inlineStr"/>
       <c r="G455" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10712,9 +10700,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D456" t="inlineStr"/>
-      <c r="E456" t="inlineStr"/>
-      <c r="F456" t="inlineStr"/>
       <c r="G456" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10737,9 +10722,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D457" t="inlineStr"/>
-      <c r="E457" t="inlineStr"/>
-      <c r="F457" t="inlineStr"/>
       <c r="G457" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10762,9 +10744,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D458" t="inlineStr"/>
-      <c r="E458" t="inlineStr"/>
-      <c r="F458" t="inlineStr"/>
       <c r="G458" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10787,9 +10766,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D459" t="inlineStr"/>
-      <c r="E459" t="inlineStr"/>
-      <c r="F459" t="inlineStr"/>
       <c r="G459" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10812,9 +10788,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D460" t="inlineStr"/>
-      <c r="E460" t="inlineStr"/>
-      <c r="F460" t="inlineStr"/>
       <c r="G460" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10837,9 +10810,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D461" t="inlineStr"/>
-      <c r="E461" t="inlineStr"/>
-      <c r="F461" t="inlineStr"/>
       <c r="G461" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10862,9 +10832,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D462" t="inlineStr"/>
-      <c r="E462" t="inlineStr"/>
-      <c r="F462" t="inlineStr"/>
       <c r="G462" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10887,9 +10854,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D463" t="inlineStr"/>
-      <c r="E463" t="inlineStr"/>
-      <c r="F463" t="inlineStr"/>
       <c r="G463" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10912,9 +10876,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D464" t="inlineStr"/>
-      <c r="E464" t="inlineStr"/>
-      <c r="F464" t="inlineStr"/>
       <c r="G464" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10937,9 +10898,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D465" t="inlineStr"/>
-      <c r="E465" t="inlineStr"/>
-      <c r="F465" t="inlineStr"/>
       <c r="G465" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10962,10 +10920,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D466" t="inlineStr"/>
-      <c r="E466" t="inlineStr"/>
-      <c r="F466" t="inlineStr"/>
       <c r="G466" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr"/>
+      <c r="E467" t="inlineStr"/>
+      <c r="F467" t="inlineStr"/>
+      <c r="G467" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr"/>
+      <c r="E468" t="inlineStr"/>
+      <c r="F468" t="inlineStr"/>
+      <c r="G468" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr"/>
+      <c r="E469" t="inlineStr"/>
+      <c r="F469" t="inlineStr"/>
+      <c r="G469" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr"/>
+      <c r="E470" t="inlineStr"/>
+      <c r="F470" t="inlineStr"/>
+      <c r="G470" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr"/>
+      <c r="E471" t="inlineStr"/>
+      <c r="F471" t="inlineStr"/>
+      <c r="G471" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr"/>
+      <c r="E472" t="inlineStr"/>
+      <c r="F472" t="inlineStr"/>
+      <c r="G472" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr"/>
+      <c r="E473" t="inlineStr"/>
+      <c r="F473" t="inlineStr"/>
+      <c r="G473" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr"/>
+      <c r="E474" t="inlineStr"/>
+      <c r="F474" t="inlineStr"/>
+      <c r="G474" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr"/>
+      <c r="E475" t="inlineStr"/>
+      <c r="F475" t="inlineStr"/>
+      <c r="G475" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr"/>
+      <c r="E476" t="inlineStr"/>
+      <c r="F476" t="inlineStr"/>
+      <c r="G476" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr"/>
+      <c r="E477" t="inlineStr"/>
+      <c r="F477" t="inlineStr"/>
+      <c r="G477" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr"/>
+      <c r="E478" t="inlineStr"/>
+      <c r="F478" t="inlineStr"/>
+      <c r="G478" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr"/>
+      <c r="E479" t="inlineStr"/>
+      <c r="F479" t="inlineStr"/>
+      <c r="G479" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr"/>
+      <c r="E480" t="inlineStr"/>
+      <c r="F480" t="inlineStr"/>
+      <c r="G480" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr"/>
+      <c r="E481" t="inlineStr"/>
+      <c r="F481" t="inlineStr"/>
+      <c r="G481" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-09-18
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G481"/>
+  <dimension ref="A1:G496"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10942,9 +10942,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D467" t="inlineStr"/>
-      <c r="E467" t="inlineStr"/>
-      <c r="F467" t="inlineStr"/>
       <c r="G467" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10967,9 +10964,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D468" t="inlineStr"/>
-      <c r="E468" t="inlineStr"/>
-      <c r="F468" t="inlineStr"/>
       <c r="G468" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -10992,9 +10986,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D469" t="inlineStr"/>
-      <c r="E469" t="inlineStr"/>
-      <c r="F469" t="inlineStr"/>
       <c r="G469" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11017,9 +11008,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D470" t="inlineStr"/>
-      <c r="E470" t="inlineStr"/>
-      <c r="F470" t="inlineStr"/>
       <c r="G470" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11042,9 +11030,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D471" t="inlineStr"/>
-      <c r="E471" t="inlineStr"/>
-      <c r="F471" t="inlineStr"/>
       <c r="G471" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11067,9 +11052,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D472" t="inlineStr"/>
-      <c r="E472" t="inlineStr"/>
-      <c r="F472" t="inlineStr"/>
       <c r="G472" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11092,9 +11074,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D473" t="inlineStr"/>
-      <c r="E473" t="inlineStr"/>
-      <c r="F473" t="inlineStr"/>
       <c r="G473" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11117,9 +11096,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D474" t="inlineStr"/>
-      <c r="E474" t="inlineStr"/>
-      <c r="F474" t="inlineStr"/>
       <c r="G474" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11142,9 +11118,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D475" t="inlineStr"/>
-      <c r="E475" t="inlineStr"/>
-      <c r="F475" t="inlineStr"/>
       <c r="G475" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11167,9 +11140,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D476" t="inlineStr"/>
-      <c r="E476" t="inlineStr"/>
-      <c r="F476" t="inlineStr"/>
       <c r="G476" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11192,9 +11162,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D477" t="inlineStr"/>
-      <c r="E477" t="inlineStr"/>
-      <c r="F477" t="inlineStr"/>
       <c r="G477" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11217,9 +11184,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D478" t="inlineStr"/>
-      <c r="E478" t="inlineStr"/>
-      <c r="F478" t="inlineStr"/>
       <c r="G478" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11242,9 +11206,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D479" t="inlineStr"/>
-      <c r="E479" t="inlineStr"/>
-      <c r="F479" t="inlineStr"/>
       <c r="G479" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11267,9 +11228,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D480" t="inlineStr"/>
-      <c r="E480" t="inlineStr"/>
-      <c r="F480" t="inlineStr"/>
       <c r="G480" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11292,10 +11250,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D481" t="inlineStr"/>
-      <c r="E481" t="inlineStr"/>
-      <c r="F481" t="inlineStr"/>
       <c r="G481" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr"/>
+      <c r="E482" t="inlineStr"/>
+      <c r="F482" t="inlineStr"/>
+      <c r="G482" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr"/>
+      <c r="E483" t="inlineStr"/>
+      <c r="F483" t="inlineStr"/>
+      <c r="G483" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr"/>
+      <c r="E484" t="inlineStr"/>
+      <c r="F484" t="inlineStr"/>
+      <c r="G484" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr"/>
+      <c r="E485" t="inlineStr"/>
+      <c r="F485" t="inlineStr"/>
+      <c r="G485" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr"/>
+      <c r="E486" t="inlineStr"/>
+      <c r="F486" t="inlineStr"/>
+      <c r="G486" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr"/>
+      <c r="E487" t="inlineStr"/>
+      <c r="F487" t="inlineStr"/>
+      <c r="G487" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr"/>
+      <c r="E488" t="inlineStr"/>
+      <c r="F488" t="inlineStr"/>
+      <c r="G488" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr"/>
+      <c r="E489" t="inlineStr"/>
+      <c r="F489" t="inlineStr"/>
+      <c r="G489" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D490" t="inlineStr"/>
+      <c r="E490" t="inlineStr"/>
+      <c r="F490" t="inlineStr"/>
+      <c r="G490" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr"/>
+      <c r="E491" t="inlineStr"/>
+      <c r="F491" t="inlineStr"/>
+      <c r="G491" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr"/>
+      <c r="E492" t="inlineStr"/>
+      <c r="F492" t="inlineStr"/>
+      <c r="G492" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr"/>
+      <c r="E493" t="inlineStr"/>
+      <c r="F493" t="inlineStr"/>
+      <c r="G493" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr"/>
+      <c r="E494" t="inlineStr"/>
+      <c r="F494" t="inlineStr"/>
+      <c r="G494" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr"/>
+      <c r="E495" t="inlineStr"/>
+      <c r="F495" t="inlineStr"/>
+      <c r="G495" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr"/>
+      <c r="E496" t="inlineStr"/>
+      <c r="F496" t="inlineStr"/>
+      <c r="G496" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-09-19
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G496"/>
+  <dimension ref="A1:G511"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11272,9 +11272,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D482" t="inlineStr"/>
-      <c r="E482" t="inlineStr"/>
-      <c r="F482" t="inlineStr"/>
       <c r="G482" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11297,9 +11294,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D483" t="inlineStr"/>
-      <c r="E483" t="inlineStr"/>
-      <c r="F483" t="inlineStr"/>
       <c r="G483" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11322,9 +11316,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D484" t="inlineStr"/>
-      <c r="E484" t="inlineStr"/>
-      <c r="F484" t="inlineStr"/>
       <c r="G484" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11347,9 +11338,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D485" t="inlineStr"/>
-      <c r="E485" t="inlineStr"/>
-      <c r="F485" t="inlineStr"/>
       <c r="G485" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11372,9 +11360,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D486" t="inlineStr"/>
-      <c r="E486" t="inlineStr"/>
-      <c r="F486" t="inlineStr"/>
       <c r="G486" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11397,9 +11382,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D487" t="inlineStr"/>
-      <c r="E487" t="inlineStr"/>
-      <c r="F487" t="inlineStr"/>
       <c r="G487" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11422,9 +11404,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D488" t="inlineStr"/>
-      <c r="E488" t="inlineStr"/>
-      <c r="F488" t="inlineStr"/>
       <c r="G488" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11447,9 +11426,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D489" t="inlineStr"/>
-      <c r="E489" t="inlineStr"/>
-      <c r="F489" t="inlineStr"/>
       <c r="G489" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11472,9 +11448,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D490" t="inlineStr"/>
-      <c r="E490" t="inlineStr"/>
-      <c r="F490" t="inlineStr"/>
       <c r="G490" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11497,9 +11470,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D491" t="inlineStr"/>
-      <c r="E491" t="inlineStr"/>
-      <c r="F491" t="inlineStr"/>
       <c r="G491" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11522,9 +11492,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D492" t="inlineStr"/>
-      <c r="E492" t="inlineStr"/>
-      <c r="F492" t="inlineStr"/>
       <c r="G492" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11547,9 +11514,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D493" t="inlineStr"/>
-      <c r="E493" t="inlineStr"/>
-      <c r="F493" t="inlineStr"/>
       <c r="G493" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11572,9 +11536,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D494" t="inlineStr"/>
-      <c r="E494" t="inlineStr"/>
-      <c r="F494" t="inlineStr"/>
       <c r="G494" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11597,9 +11558,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D495" t="inlineStr"/>
-      <c r="E495" t="inlineStr"/>
-      <c r="F495" t="inlineStr"/>
       <c r="G495" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11622,10 +11580,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D496" t="inlineStr"/>
-      <c r="E496" t="inlineStr"/>
-      <c r="F496" t="inlineStr"/>
       <c r="G496" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr"/>
+      <c r="E497" t="inlineStr"/>
+      <c r="F497" t="inlineStr"/>
+      <c r="G497" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr"/>
+      <c r="E498" t="inlineStr"/>
+      <c r="F498" t="inlineStr"/>
+      <c r="G498" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr"/>
+      <c r="E499" t="inlineStr"/>
+      <c r="F499" t="inlineStr"/>
+      <c r="G499" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr"/>
+      <c r="E500" t="inlineStr"/>
+      <c r="F500" t="inlineStr"/>
+      <c r="G500" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr"/>
+      <c r="E501" t="inlineStr"/>
+      <c r="F501" t="inlineStr"/>
+      <c r="G501" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr"/>
+      <c r="E502" t="inlineStr"/>
+      <c r="F502" t="inlineStr"/>
+      <c r="G502" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr"/>
+      <c r="E503" t="inlineStr"/>
+      <c r="F503" t="inlineStr"/>
+      <c r="G503" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr"/>
+      <c r="E504" t="inlineStr"/>
+      <c r="F504" t="inlineStr"/>
+      <c r="G504" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr"/>
+      <c r="E505" t="inlineStr"/>
+      <c r="F505" t="inlineStr"/>
+      <c r="G505" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D506" t="inlineStr"/>
+      <c r="E506" t="inlineStr"/>
+      <c r="F506" t="inlineStr"/>
+      <c r="G506" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D507" t="inlineStr"/>
+      <c r="E507" t="inlineStr"/>
+      <c r="F507" t="inlineStr"/>
+      <c r="G507" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D508" t="inlineStr"/>
+      <c r="E508" t="inlineStr"/>
+      <c r="F508" t="inlineStr"/>
+      <c r="G508" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D509" t="inlineStr"/>
+      <c r="E509" t="inlineStr"/>
+      <c r="F509" t="inlineStr"/>
+      <c r="G509" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D510" t="inlineStr"/>
+      <c r="E510" t="inlineStr"/>
+      <c r="F510" t="inlineStr"/>
+      <c r="G510" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D511" t="inlineStr"/>
+      <c r="E511" t="inlineStr"/>
+      <c r="F511" t="inlineStr"/>
+      <c r="G511" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-09-20
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G511"/>
+  <dimension ref="A1:G526"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11602,9 +11602,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D497" t="inlineStr"/>
-      <c r="E497" t="inlineStr"/>
-      <c r="F497" t="inlineStr"/>
       <c r="G497" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11627,9 +11624,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D498" t="inlineStr"/>
-      <c r="E498" t="inlineStr"/>
-      <c r="F498" t="inlineStr"/>
       <c r="G498" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11652,9 +11646,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D499" t="inlineStr"/>
-      <c r="E499" t="inlineStr"/>
-      <c r="F499" t="inlineStr"/>
       <c r="G499" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11677,9 +11668,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D500" t="inlineStr"/>
-      <c r="E500" t="inlineStr"/>
-      <c r="F500" t="inlineStr"/>
       <c r="G500" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11702,9 +11690,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D501" t="inlineStr"/>
-      <c r="E501" t="inlineStr"/>
-      <c r="F501" t="inlineStr"/>
       <c r="G501" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11727,9 +11712,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D502" t="inlineStr"/>
-      <c r="E502" t="inlineStr"/>
-      <c r="F502" t="inlineStr"/>
       <c r="G502" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11752,9 +11734,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D503" t="inlineStr"/>
-      <c r="E503" t="inlineStr"/>
-      <c r="F503" t="inlineStr"/>
       <c r="G503" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11777,9 +11756,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D504" t="inlineStr"/>
-      <c r="E504" t="inlineStr"/>
-      <c r="F504" t="inlineStr"/>
       <c r="G504" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11802,9 +11778,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D505" t="inlineStr"/>
-      <c r="E505" t="inlineStr"/>
-      <c r="F505" t="inlineStr"/>
       <c r="G505" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11827,9 +11800,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D506" t="inlineStr"/>
-      <c r="E506" t="inlineStr"/>
-      <c r="F506" t="inlineStr"/>
       <c r="G506" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11852,9 +11822,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D507" t="inlineStr"/>
-      <c r="E507" t="inlineStr"/>
-      <c r="F507" t="inlineStr"/>
       <c r="G507" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11877,9 +11844,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D508" t="inlineStr"/>
-      <c r="E508" t="inlineStr"/>
-      <c r="F508" t="inlineStr"/>
       <c r="G508" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11902,9 +11866,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D509" t="inlineStr"/>
-      <c r="E509" t="inlineStr"/>
-      <c r="F509" t="inlineStr"/>
       <c r="G509" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11927,9 +11888,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D510" t="inlineStr"/>
-      <c r="E510" t="inlineStr"/>
-      <c r="F510" t="inlineStr"/>
       <c r="G510" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11952,10 +11910,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D511" t="inlineStr"/>
-      <c r="E511" t="inlineStr"/>
-      <c r="F511" t="inlineStr"/>
       <c r="G511" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr"/>
+      <c r="E512" t="inlineStr"/>
+      <c r="F512" t="inlineStr"/>
+      <c r="G512" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr"/>
+      <c r="E513" t="inlineStr"/>
+      <c r="F513" t="inlineStr"/>
+      <c r="G513" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D514" t="inlineStr"/>
+      <c r="E514" t="inlineStr"/>
+      <c r="F514" t="inlineStr"/>
+      <c r="G514" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr"/>
+      <c r="E515" t="inlineStr"/>
+      <c r="F515" t="inlineStr"/>
+      <c r="G515" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D516" t="inlineStr"/>
+      <c r="E516" t="inlineStr"/>
+      <c r="F516" t="inlineStr"/>
+      <c r="G516" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr"/>
+      <c r="E517" t="inlineStr"/>
+      <c r="F517" t="inlineStr"/>
+      <c r="G517" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr"/>
+      <c r="E518" t="inlineStr"/>
+      <c r="F518" t="inlineStr"/>
+      <c r="G518" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D519" t="inlineStr"/>
+      <c r="E519" t="inlineStr"/>
+      <c r="F519" t="inlineStr"/>
+      <c r="G519" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D520" t="inlineStr"/>
+      <c r="E520" t="inlineStr"/>
+      <c r="F520" t="inlineStr"/>
+      <c r="G520" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D521" t="inlineStr"/>
+      <c r="E521" t="inlineStr"/>
+      <c r="F521" t="inlineStr"/>
+      <c r="G521" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D522" t="inlineStr"/>
+      <c r="E522" t="inlineStr"/>
+      <c r="F522" t="inlineStr"/>
+      <c r="G522" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D523" t="inlineStr"/>
+      <c r="E523" t="inlineStr"/>
+      <c r="F523" t="inlineStr"/>
+      <c r="G523" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D524" t="inlineStr"/>
+      <c r="E524" t="inlineStr"/>
+      <c r="F524" t="inlineStr"/>
+      <c r="G524" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D525" t="inlineStr"/>
+      <c r="E525" t="inlineStr"/>
+      <c r="F525" t="inlineStr"/>
+      <c r="G525" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D526" t="inlineStr"/>
+      <c r="E526" t="inlineStr"/>
+      <c r="F526" t="inlineStr"/>
+      <c r="G526" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-09-21
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G526"/>
+  <dimension ref="A1:G541"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11932,9 +11932,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D512" t="inlineStr"/>
-      <c r="E512" t="inlineStr"/>
-      <c r="F512" t="inlineStr"/>
       <c r="G512" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11957,9 +11954,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D513" t="inlineStr"/>
-      <c r="E513" t="inlineStr"/>
-      <c r="F513" t="inlineStr"/>
       <c r="G513" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -11982,9 +11976,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D514" t="inlineStr"/>
-      <c r="E514" t="inlineStr"/>
-      <c r="F514" t="inlineStr"/>
       <c r="G514" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12007,9 +11998,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D515" t="inlineStr"/>
-      <c r="E515" t="inlineStr"/>
-      <c r="F515" t="inlineStr"/>
       <c r="G515" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12032,9 +12020,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D516" t="inlineStr"/>
-      <c r="E516" t="inlineStr"/>
-      <c r="F516" t="inlineStr"/>
       <c r="G516" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12057,9 +12042,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D517" t="inlineStr"/>
-      <c r="E517" t="inlineStr"/>
-      <c r="F517" t="inlineStr"/>
       <c r="G517" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12082,9 +12064,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D518" t="inlineStr"/>
-      <c r="E518" t="inlineStr"/>
-      <c r="F518" t="inlineStr"/>
       <c r="G518" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12107,9 +12086,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D519" t="inlineStr"/>
-      <c r="E519" t="inlineStr"/>
-      <c r="F519" t="inlineStr"/>
       <c r="G519" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12132,9 +12108,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D520" t="inlineStr"/>
-      <c r="E520" t="inlineStr"/>
-      <c r="F520" t="inlineStr"/>
       <c r="G520" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12157,9 +12130,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D521" t="inlineStr"/>
-      <c r="E521" t="inlineStr"/>
-      <c r="F521" t="inlineStr"/>
       <c r="G521" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12182,9 +12152,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D522" t="inlineStr"/>
-      <c r="E522" t="inlineStr"/>
-      <c r="F522" t="inlineStr"/>
       <c r="G522" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12207,9 +12174,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D523" t="inlineStr"/>
-      <c r="E523" t="inlineStr"/>
-      <c r="F523" t="inlineStr"/>
       <c r="G523" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12232,9 +12196,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D524" t="inlineStr"/>
-      <c r="E524" t="inlineStr"/>
-      <c r="F524" t="inlineStr"/>
       <c r="G524" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12257,9 +12218,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D525" t="inlineStr"/>
-      <c r="E525" t="inlineStr"/>
-      <c r="F525" t="inlineStr"/>
       <c r="G525" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12282,10 +12240,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D526" t="inlineStr"/>
-      <c r="E526" t="inlineStr"/>
-      <c r="F526" t="inlineStr"/>
       <c r="G526" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D527" t="inlineStr"/>
+      <c r="E527" t="inlineStr"/>
+      <c r="F527" t="inlineStr"/>
+      <c r="G527" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D528" t="inlineStr"/>
+      <c r="E528" t="inlineStr"/>
+      <c r="F528" t="inlineStr"/>
+      <c r="G528" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D529" t="inlineStr"/>
+      <c r="E529" t="inlineStr"/>
+      <c r="F529" t="inlineStr"/>
+      <c r="G529" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D530" t="inlineStr"/>
+      <c r="E530" t="inlineStr"/>
+      <c r="F530" t="inlineStr"/>
+      <c r="G530" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D531" t="inlineStr"/>
+      <c r="E531" t="inlineStr"/>
+      <c r="F531" t="inlineStr"/>
+      <c r="G531" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D532" t="inlineStr"/>
+      <c r="E532" t="inlineStr"/>
+      <c r="F532" t="inlineStr"/>
+      <c r="G532" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D533" t="inlineStr"/>
+      <c r="E533" t="inlineStr"/>
+      <c r="F533" t="inlineStr"/>
+      <c r="G533" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D534" t="inlineStr"/>
+      <c r="E534" t="inlineStr"/>
+      <c r="F534" t="inlineStr"/>
+      <c r="G534" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D535" t="inlineStr"/>
+      <c r="E535" t="inlineStr"/>
+      <c r="F535" t="inlineStr"/>
+      <c r="G535" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D536" t="inlineStr"/>
+      <c r="E536" t="inlineStr"/>
+      <c r="F536" t="inlineStr"/>
+      <c r="G536" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D537" t="inlineStr"/>
+      <c r="E537" t="inlineStr"/>
+      <c r="F537" t="inlineStr"/>
+      <c r="G537" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D538" t="inlineStr"/>
+      <c r="E538" t="inlineStr"/>
+      <c r="F538" t="inlineStr"/>
+      <c r="G538" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D539" t="inlineStr"/>
+      <c r="E539" t="inlineStr"/>
+      <c r="F539" t="inlineStr"/>
+      <c r="G539" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D540" t="inlineStr"/>
+      <c r="E540" t="inlineStr"/>
+      <c r="F540" t="inlineStr"/>
+      <c r="G540" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D541" t="inlineStr"/>
+      <c r="E541" t="inlineStr"/>
+      <c r="F541" t="inlineStr"/>
+      <c r="G541" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-09-22
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G541"/>
+  <dimension ref="A1:G556"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12262,9 +12262,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D527" t="inlineStr"/>
-      <c r="E527" t="inlineStr"/>
-      <c r="F527" t="inlineStr"/>
       <c r="G527" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12287,9 +12284,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D528" t="inlineStr"/>
-      <c r="E528" t="inlineStr"/>
-      <c r="F528" t="inlineStr"/>
       <c r="G528" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12312,9 +12306,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D529" t="inlineStr"/>
-      <c r="E529" t="inlineStr"/>
-      <c r="F529" t="inlineStr"/>
       <c r="G529" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12337,9 +12328,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D530" t="inlineStr"/>
-      <c r="E530" t="inlineStr"/>
-      <c r="F530" t="inlineStr"/>
       <c r="G530" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12362,9 +12350,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D531" t="inlineStr"/>
-      <c r="E531" t="inlineStr"/>
-      <c r="F531" t="inlineStr"/>
       <c r="G531" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12387,9 +12372,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D532" t="inlineStr"/>
-      <c r="E532" t="inlineStr"/>
-      <c r="F532" t="inlineStr"/>
       <c r="G532" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12412,9 +12394,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D533" t="inlineStr"/>
-      <c r="E533" t="inlineStr"/>
-      <c r="F533" t="inlineStr"/>
       <c r="G533" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12437,9 +12416,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D534" t="inlineStr"/>
-      <c r="E534" t="inlineStr"/>
-      <c r="F534" t="inlineStr"/>
       <c r="G534" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12462,9 +12438,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D535" t="inlineStr"/>
-      <c r="E535" t="inlineStr"/>
-      <c r="F535" t="inlineStr"/>
       <c r="G535" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12487,9 +12460,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D536" t="inlineStr"/>
-      <c r="E536" t="inlineStr"/>
-      <c r="F536" t="inlineStr"/>
       <c r="G536" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12512,9 +12482,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D537" t="inlineStr"/>
-      <c r="E537" t="inlineStr"/>
-      <c r="F537" t="inlineStr"/>
       <c r="G537" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12537,9 +12504,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D538" t="inlineStr"/>
-      <c r="E538" t="inlineStr"/>
-      <c r="F538" t="inlineStr"/>
       <c r="G538" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12562,9 +12526,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D539" t="inlineStr"/>
-      <c r="E539" t="inlineStr"/>
-      <c r="F539" t="inlineStr"/>
       <c r="G539" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12587,9 +12548,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D540" t="inlineStr"/>
-      <c r="E540" t="inlineStr"/>
-      <c r="F540" t="inlineStr"/>
       <c r="G540" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12612,10 +12570,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D541" t="inlineStr"/>
-      <c r="E541" t="inlineStr"/>
-      <c r="F541" t="inlineStr"/>
       <c r="G541" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D542" t="inlineStr"/>
+      <c r="E542" t="inlineStr"/>
+      <c r="F542" t="inlineStr"/>
+      <c r="G542" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D543" t="inlineStr"/>
+      <c r="E543" t="inlineStr"/>
+      <c r="F543" t="inlineStr"/>
+      <c r="G543" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D544" t="inlineStr"/>
+      <c r="E544" t="inlineStr"/>
+      <c r="F544" t="inlineStr"/>
+      <c r="G544" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D545" t="inlineStr"/>
+      <c r="E545" t="inlineStr"/>
+      <c r="F545" t="inlineStr"/>
+      <c r="G545" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D546" t="inlineStr"/>
+      <c r="E546" t="inlineStr"/>
+      <c r="F546" t="inlineStr"/>
+      <c r="G546" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D547" t="inlineStr"/>
+      <c r="E547" t="inlineStr"/>
+      <c r="F547" t="inlineStr"/>
+      <c r="G547" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D548" t="inlineStr"/>
+      <c r="E548" t="inlineStr"/>
+      <c r="F548" t="inlineStr"/>
+      <c r="G548" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D549" t="inlineStr"/>
+      <c r="E549" t="inlineStr"/>
+      <c r="F549" t="inlineStr"/>
+      <c r="G549" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D550" t="inlineStr"/>
+      <c r="E550" t="inlineStr"/>
+      <c r="F550" t="inlineStr"/>
+      <c r="G550" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D551" t="inlineStr"/>
+      <c r="E551" t="inlineStr"/>
+      <c r="F551" t="inlineStr"/>
+      <c r="G551" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D552" t="inlineStr"/>
+      <c r="E552" t="inlineStr"/>
+      <c r="F552" t="inlineStr"/>
+      <c r="G552" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D553" t="inlineStr"/>
+      <c r="E553" t="inlineStr"/>
+      <c r="F553" t="inlineStr"/>
+      <c r="G553" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D554" t="inlineStr"/>
+      <c r="E554" t="inlineStr"/>
+      <c r="F554" t="inlineStr"/>
+      <c r="G554" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D555" t="inlineStr"/>
+      <c r="E555" t="inlineStr"/>
+      <c r="F555" t="inlineStr"/>
+      <c r="G555" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D556" t="inlineStr"/>
+      <c r="E556" t="inlineStr"/>
+      <c r="F556" t="inlineStr"/>
+      <c r="G556" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-09-23
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G556"/>
+  <dimension ref="A1:G571"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12592,9 +12592,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D542" t="inlineStr"/>
-      <c r="E542" t="inlineStr"/>
-      <c r="F542" t="inlineStr"/>
       <c r="G542" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12617,9 +12614,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D543" t="inlineStr"/>
-      <c r="E543" t="inlineStr"/>
-      <c r="F543" t="inlineStr"/>
       <c r="G543" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12642,9 +12636,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D544" t="inlineStr"/>
-      <c r="E544" t="inlineStr"/>
-      <c r="F544" t="inlineStr"/>
       <c r="G544" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12667,9 +12658,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D545" t="inlineStr"/>
-      <c r="E545" t="inlineStr"/>
-      <c r="F545" t="inlineStr"/>
       <c r="G545" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12692,9 +12680,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D546" t="inlineStr"/>
-      <c r="E546" t="inlineStr"/>
-      <c r="F546" t="inlineStr"/>
       <c r="G546" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12717,9 +12702,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D547" t="inlineStr"/>
-      <c r="E547" t="inlineStr"/>
-      <c r="F547" t="inlineStr"/>
       <c r="G547" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12742,9 +12724,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D548" t="inlineStr"/>
-      <c r="E548" t="inlineStr"/>
-      <c r="F548" t="inlineStr"/>
       <c r="G548" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12767,9 +12746,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D549" t="inlineStr"/>
-      <c r="E549" t="inlineStr"/>
-      <c r="F549" t="inlineStr"/>
       <c r="G549" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12792,9 +12768,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D550" t="inlineStr"/>
-      <c r="E550" t="inlineStr"/>
-      <c r="F550" t="inlineStr"/>
       <c r="G550" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12817,9 +12790,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D551" t="inlineStr"/>
-      <c r="E551" t="inlineStr"/>
-      <c r="F551" t="inlineStr"/>
       <c r="G551" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12842,9 +12812,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D552" t="inlineStr"/>
-      <c r="E552" t="inlineStr"/>
-      <c r="F552" t="inlineStr"/>
       <c r="G552" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12867,9 +12834,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D553" t="inlineStr"/>
-      <c r="E553" t="inlineStr"/>
-      <c r="F553" t="inlineStr"/>
       <c r="G553" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12892,9 +12856,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D554" t="inlineStr"/>
-      <c r="E554" t="inlineStr"/>
-      <c r="F554" t="inlineStr"/>
       <c r="G554" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12917,9 +12878,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D555" t="inlineStr"/>
-      <c r="E555" t="inlineStr"/>
-      <c r="F555" t="inlineStr"/>
       <c r="G555" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12942,10 +12900,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D556" t="inlineStr"/>
-      <c r="E556" t="inlineStr"/>
-      <c r="F556" t="inlineStr"/>
       <c r="G556" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D557" t="inlineStr"/>
+      <c r="E557" t="inlineStr"/>
+      <c r="F557" t="inlineStr"/>
+      <c r="G557" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D558" t="inlineStr"/>
+      <c r="E558" t="inlineStr"/>
+      <c r="F558" t="inlineStr"/>
+      <c r="G558" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D559" t="inlineStr"/>
+      <c r="E559" t="inlineStr"/>
+      <c r="F559" t="inlineStr"/>
+      <c r="G559" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D560" t="inlineStr"/>
+      <c r="E560" t="inlineStr"/>
+      <c r="F560" t="inlineStr"/>
+      <c r="G560" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D561" t="inlineStr"/>
+      <c r="E561" t="inlineStr"/>
+      <c r="F561" t="inlineStr"/>
+      <c r="G561" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D562" t="inlineStr"/>
+      <c r="E562" t="inlineStr"/>
+      <c r="F562" t="inlineStr"/>
+      <c r="G562" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D563" t="inlineStr"/>
+      <c r="E563" t="inlineStr"/>
+      <c r="F563" t="inlineStr"/>
+      <c r="G563" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D564" t="inlineStr"/>
+      <c r="E564" t="inlineStr"/>
+      <c r="F564" t="inlineStr"/>
+      <c r="G564" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D565" t="inlineStr"/>
+      <c r="E565" t="inlineStr"/>
+      <c r="F565" t="inlineStr"/>
+      <c r="G565" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D566" t="inlineStr"/>
+      <c r="E566" t="inlineStr"/>
+      <c r="F566" t="inlineStr"/>
+      <c r="G566" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D567" t="inlineStr"/>
+      <c r="E567" t="inlineStr"/>
+      <c r="F567" t="inlineStr"/>
+      <c r="G567" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D568" t="inlineStr"/>
+      <c r="E568" t="inlineStr"/>
+      <c r="F568" t="inlineStr"/>
+      <c r="G568" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D569" t="inlineStr"/>
+      <c r="E569" t="inlineStr"/>
+      <c r="F569" t="inlineStr"/>
+      <c r="G569" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D570" t="inlineStr"/>
+      <c r="E570" t="inlineStr"/>
+      <c r="F570" t="inlineStr"/>
+      <c r="G570" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D571" t="inlineStr"/>
+      <c r="E571" t="inlineStr"/>
+      <c r="F571" t="inlineStr"/>
+      <c r="G571" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-09-24
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G571"/>
+  <dimension ref="A1:G592"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12922,9 +12922,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D557" t="inlineStr"/>
-      <c r="E557" t="inlineStr"/>
-      <c r="F557" t="inlineStr"/>
       <c r="G557" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12947,9 +12944,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D558" t="inlineStr"/>
-      <c r="E558" t="inlineStr"/>
-      <c r="F558" t="inlineStr"/>
       <c r="G558" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12972,9 +12966,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D559" t="inlineStr"/>
-      <c r="E559" t="inlineStr"/>
-      <c r="F559" t="inlineStr"/>
       <c r="G559" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -12997,9 +12988,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D560" t="inlineStr"/>
-      <c r="E560" t="inlineStr"/>
-      <c r="F560" t="inlineStr"/>
       <c r="G560" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -13022,9 +13010,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D561" t="inlineStr"/>
-      <c r="E561" t="inlineStr"/>
-      <c r="F561" t="inlineStr"/>
       <c r="G561" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -13047,9 +13032,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D562" t="inlineStr"/>
-      <c r="E562" t="inlineStr"/>
-      <c r="F562" t="inlineStr"/>
       <c r="G562" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -13072,9 +13054,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D563" t="inlineStr"/>
-      <c r="E563" t="inlineStr"/>
-      <c r="F563" t="inlineStr"/>
       <c r="G563" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -13097,9 +13076,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D564" t="inlineStr"/>
-      <c r="E564" t="inlineStr"/>
-      <c r="F564" t="inlineStr"/>
       <c r="G564" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -13122,9 +13098,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D565" t="inlineStr"/>
-      <c r="E565" t="inlineStr"/>
-      <c r="F565" t="inlineStr"/>
       <c r="G565" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -13147,9 +13120,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D566" t="inlineStr"/>
-      <c r="E566" t="inlineStr"/>
-      <c r="F566" t="inlineStr"/>
       <c r="G566" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -13172,9 +13142,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D567" t="inlineStr"/>
-      <c r="E567" t="inlineStr"/>
-      <c r="F567" t="inlineStr"/>
       <c r="G567" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -13197,9 +13164,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D568" t="inlineStr"/>
-      <c r="E568" t="inlineStr"/>
-      <c r="F568" t="inlineStr"/>
       <c r="G568" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -13222,9 +13186,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D569" t="inlineStr"/>
-      <c r="E569" t="inlineStr"/>
-      <c r="F569" t="inlineStr"/>
       <c r="G569" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -13247,9 +13208,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D570" t="inlineStr"/>
-      <c r="E570" t="inlineStr"/>
-      <c r="F570" t="inlineStr"/>
       <c r="G570" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -13272,14 +13230,545 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D571" t="inlineStr"/>
-      <c r="E571" t="inlineStr"/>
-      <c r="F571" t="inlineStr"/>
       <c r="G571" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>
       </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D572" t="inlineStr"/>
+      <c r="E572" t="inlineStr"/>
+      <c r="F572" t="inlineStr"/>
+      <c r="G572" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D573" t="inlineStr"/>
+      <c r="E573" t="inlineStr"/>
+      <c r="F573" t="inlineStr"/>
+      <c r="G573" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D574" t="inlineStr"/>
+      <c r="E574" t="inlineStr"/>
+      <c r="F574" t="inlineStr"/>
+      <c r="G574" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D575" t="inlineStr"/>
+      <c r="E575" t="inlineStr"/>
+      <c r="F575" t="inlineStr"/>
+      <c r="G575" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E576" t="n">
+        <v>2799</v>
+      </c>
+      <c r="F576" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Duplex-litros-Branca/dp/B07FXZ8TR6/ref=sr_1_5</t>
+        </is>
+      </c>
+      <c r="G576" t="inlineStr"/>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E577" t="n">
+        <v>3039.05</v>
+      </c>
+      <c r="F577" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-BRM46MK-Duplex-Extrafrio-Brastemp/dp/B0GL3Q3PTG/ref=sr_1_6</t>
+        </is>
+      </c>
+      <c r="G577" t="inlineStr"/>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E578" t="n">
+        <v>3048.61</v>
+      </c>
+      <c r="F578" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWVJ8LR/ref=sr_1_7</t>
+        </is>
+      </c>
+      <c r="G578" t="inlineStr"/>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D579" t="inlineStr"/>
+      <c r="E579" t="inlineStr"/>
+      <c r="F579" t="inlineStr"/>
+      <c r="G579" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D580" t="inlineStr"/>
+      <c r="E580" t="inlineStr"/>
+      <c r="F580" t="inlineStr"/>
+      <c r="G580" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D581" t="inlineStr"/>
+      <c r="E581" t="inlineStr"/>
+      <c r="F581" t="inlineStr"/>
+      <c r="G581" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D582" t="inlineStr"/>
+      <c r="E582" t="inlineStr"/>
+      <c r="F582" t="inlineStr"/>
+      <c r="G582" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E583" t="n">
+        <v>529.9</v>
+      </c>
+      <c r="F583" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Tira-Odor-MT30S/dp/B079Y3MLSP/ref=sr_1_1</t>
+        </is>
+      </c>
+      <c r="G583" t="inlineStr"/>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E584" t="n">
+        <v>490.1</v>
+      </c>
+      <c r="F584" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P2FLSR/ref=sr_1_2</t>
+        </is>
+      </c>
+      <c r="G584" t="inlineStr"/>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E585" t="n">
+        <v>483.55</v>
+      </c>
+      <c r="F585" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Electrolux-MTO30-Fun%C3%A7%C3%A3o-Tira/dp/B083ZFFC5Q/ref=sr_1_3</t>
+        </is>
+      </c>
+      <c r="G585" t="inlineStr"/>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D586" t="inlineStr"/>
+      <c r="E586" t="inlineStr"/>
+      <c r="F586" t="inlineStr"/>
+      <c r="G586" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D587" t="inlineStr"/>
+      <c r="E587" t="inlineStr"/>
+      <c r="F587" t="inlineStr"/>
+      <c r="G587" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D588" t="inlineStr"/>
+      <c r="E588" t="inlineStr"/>
+      <c r="F588" t="inlineStr"/>
+      <c r="G588" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D589" t="inlineStr"/>
+      <c r="E589" t="inlineStr"/>
+      <c r="F589" t="inlineStr"/>
+      <c r="G589" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E590" t="n">
+        <v>1099</v>
+      </c>
+      <c r="F590" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-04-Bocas-FS-CF04NABUNA/dp/B07JPZN51P/ref=sr_1_5</t>
+        </is>
+      </c>
+      <c r="G590" t="inlineStr"/>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E591" t="n">
+        <v>1258.75</v>
+      </c>
+      <c r="F591" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-Consul-Bocas-CFO4NARUNA-Bivolt/dp/B07HM9JL5K/ref=sr_1_6</t>
+        </is>
+      </c>
+      <c r="G591" t="inlineStr"/>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E592" t="n">
+        <v>1519.05</v>
+      </c>
+      <c r="F592" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-Bocas-Consul-Vidro-Bivolt/dp/B076BC7769/ref=sr_1_7</t>
+        </is>
+      </c>
+      <c r="G592" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Atualiza preços de 2026-09-25
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G592"/>
+  <dimension ref="A1:G613"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13252,9 +13252,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D572" t="inlineStr"/>
-      <c r="E572" t="inlineStr"/>
-      <c r="F572" t="inlineStr"/>
       <c r="G572" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -13277,9 +13274,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D573" t="inlineStr"/>
-      <c r="E573" t="inlineStr"/>
-      <c r="F573" t="inlineStr"/>
       <c r="G573" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -13302,9 +13296,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D574" t="inlineStr"/>
-      <c r="E574" t="inlineStr"/>
-      <c r="F574" t="inlineStr"/>
       <c r="G574" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -13327,9 +13318,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D575" t="inlineStr"/>
-      <c r="E575" t="inlineStr"/>
-      <c r="F575" t="inlineStr"/>
       <c r="G575" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -13360,7 +13348,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Duplex-litros-Branca/dp/B07FXZ8TR6/ref=sr_1_5</t>
         </is>
       </c>
-      <c r="G576" t="inlineStr"/>
     </row>
     <row r="577">
       <c r="A577" t="inlineStr">
@@ -13386,7 +13373,6 @@
           <t>https://www.amazon.com.br/Geladeira-BRM46MK-Duplex-Extrafrio-Brastemp/dp/B0GL3Q3PTG/ref=sr_1_6</t>
         </is>
       </c>
-      <c r="G577" t="inlineStr"/>
     </row>
     <row r="578">
       <c r="A578" t="inlineStr">
@@ -13412,7 +13398,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWVJ8LR/ref=sr_1_7</t>
         </is>
       </c>
-      <c r="G578" t="inlineStr"/>
     </row>
     <row r="579">
       <c r="A579" t="inlineStr">
@@ -13430,9 +13415,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D579" t="inlineStr"/>
-      <c r="E579" t="inlineStr"/>
-      <c r="F579" t="inlineStr"/>
       <c r="G579" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -13455,9 +13437,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D580" t="inlineStr"/>
-      <c r="E580" t="inlineStr"/>
-      <c r="F580" t="inlineStr"/>
       <c r="G580" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -13480,9 +13459,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D581" t="inlineStr"/>
-      <c r="E581" t="inlineStr"/>
-      <c r="F581" t="inlineStr"/>
       <c r="G581" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -13505,9 +13481,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D582" t="inlineStr"/>
-      <c r="E582" t="inlineStr"/>
-      <c r="F582" t="inlineStr"/>
       <c r="G582" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -13538,7 +13511,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Tira-Odor-MT30S/dp/B079Y3MLSP/ref=sr_1_1</t>
         </is>
       </c>
-      <c r="G583" t="inlineStr"/>
     </row>
     <row r="584">
       <c r="A584" t="inlineStr">
@@ -13564,7 +13536,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P2FLSR/ref=sr_1_2</t>
         </is>
       </c>
-      <c r="G584" t="inlineStr"/>
     </row>
     <row r="585">
       <c r="A585" t="inlineStr">
@@ -13590,7 +13561,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Electrolux-MTO30-Fun%C3%A7%C3%A3o-Tira/dp/B083ZFFC5Q/ref=sr_1_3</t>
         </is>
       </c>
-      <c r="G585" t="inlineStr"/>
     </row>
     <row r="586">
       <c r="A586" t="inlineStr">
@@ -13608,9 +13578,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D586" t="inlineStr"/>
-      <c r="E586" t="inlineStr"/>
-      <c r="F586" t="inlineStr"/>
       <c r="G586" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -13633,9 +13600,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D587" t="inlineStr"/>
-      <c r="E587" t="inlineStr"/>
-      <c r="F587" t="inlineStr"/>
       <c r="G587" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -13658,9 +13622,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D588" t="inlineStr"/>
-      <c r="E588" t="inlineStr"/>
-      <c r="F588" t="inlineStr"/>
       <c r="G588" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -13683,9 +13644,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D589" t="inlineStr"/>
-      <c r="E589" t="inlineStr"/>
-      <c r="F589" t="inlineStr"/>
       <c r="G589" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -13716,7 +13674,6 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-04-Bocas-FS-CF04NABUNA/dp/B07JPZN51P/ref=sr_1_5</t>
         </is>
       </c>
-      <c r="G590" t="inlineStr"/>
     </row>
     <row r="591">
       <c r="A591" t="inlineStr">
@@ -13742,7 +13699,6 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-Consul-Bocas-CFO4NARUNA-Bivolt/dp/B07HM9JL5K/ref=sr_1_6</t>
         </is>
       </c>
-      <c r="G591" t="inlineStr"/>
     </row>
     <row r="592">
       <c r="A592" t="inlineStr">
@@ -13768,7 +13724,540 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-Bocas-Consul-Vidro-Bivolt/dp/B076BC7769/ref=sr_1_7</t>
         </is>
       </c>
-      <c r="G592" t="inlineStr"/>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D593" t="inlineStr"/>
+      <c r="E593" t="inlineStr"/>
+      <c r="F593" t="inlineStr"/>
+      <c r="G593" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D594" t="inlineStr"/>
+      <c r="E594" t="inlineStr"/>
+      <c r="F594" t="inlineStr"/>
+      <c r="G594" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D595" t="inlineStr"/>
+      <c r="E595" t="inlineStr"/>
+      <c r="F595" t="inlineStr"/>
+      <c r="G595" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D596" t="inlineStr"/>
+      <c r="E596" t="inlineStr"/>
+      <c r="F596" t="inlineStr"/>
+      <c r="G596" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E597" t="n">
+        <v>2735.13</v>
+      </c>
+      <c r="F597" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-BRM46MK-Duplex-Extrafrio-Brastemp/dp/B0GL3Q3PTG/ref=sr_1_3</t>
+        </is>
+      </c>
+      <c r="G597" t="inlineStr"/>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E598" t="n">
+        <v>2799</v>
+      </c>
+      <c r="F598" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Duplex-litros-Branca/dp/B07FXZ8TR6/ref=sr_1_4</t>
+        </is>
+      </c>
+      <c r="G598" t="inlineStr"/>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E599" t="n">
+        <v>3134.05</v>
+      </c>
+      <c r="F599" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWSXQGL/ref=sr_1_5</t>
+        </is>
+      </c>
+      <c r="G599" t="inlineStr"/>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D600" t="inlineStr"/>
+      <c r="E600" t="inlineStr"/>
+      <c r="F600" t="inlineStr"/>
+      <c r="G600" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D601" t="inlineStr"/>
+      <c r="E601" t="inlineStr"/>
+      <c r="F601" t="inlineStr"/>
+      <c r="G601" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D602" t="inlineStr"/>
+      <c r="E602" t="inlineStr"/>
+      <c r="F602" t="inlineStr"/>
+      <c r="G602" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D603" t="inlineStr"/>
+      <c r="E603" t="inlineStr"/>
+      <c r="F603" t="inlineStr"/>
+      <c r="G603" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E604" t="n">
+        <v>529.9</v>
+      </c>
+      <c r="F604" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Tira-Odor-MT30S/dp/B079Y3MLSP/ref=sr_1_1</t>
+        </is>
+      </c>
+      <c r="G604" t="inlineStr"/>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E605" t="n">
+        <v>483.55</v>
+      </c>
+      <c r="F605" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Electrolux-MTO30-Fun%C3%A7%C3%A3o-Tira/dp/B083ZFFC5Q/ref=sr_1_2</t>
+        </is>
+      </c>
+      <c r="G605" t="inlineStr"/>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E606" t="n">
+        <v>499.01</v>
+      </c>
+      <c r="F606" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Efficient-23L-ME23B/dp/B0B8KWNK12/ref=sr_1_3</t>
+        </is>
+      </c>
+      <c r="G606" t="inlineStr"/>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D607" t="inlineStr"/>
+      <c r="E607" t="inlineStr"/>
+      <c r="F607" t="inlineStr"/>
+      <c r="G607" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D608" t="inlineStr"/>
+      <c r="E608" t="inlineStr"/>
+      <c r="F608" t="inlineStr"/>
+      <c r="G608" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D609" t="inlineStr"/>
+      <c r="E609" t="inlineStr"/>
+      <c r="F609" t="inlineStr"/>
+      <c r="G609" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D610" t="inlineStr"/>
+      <c r="E610" t="inlineStr"/>
+      <c r="F610" t="inlineStr"/>
+      <c r="G610" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E611" t="n">
+        <v>1099</v>
+      </c>
+      <c r="F611" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-04-Bocas-FS-CF04NABUNA/dp/B07JPZN51P/ref=sr_1_5</t>
+        </is>
+      </c>
+      <c r="G611" t="inlineStr"/>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E612" t="n">
+        <v>1132.87</v>
+      </c>
+      <c r="F612" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-Consul-Bocas-CFO4NARUNA-Bivolt/dp/B07HM9JL5K/ref=sr_1_6</t>
+        </is>
+      </c>
+      <c r="G612" t="inlineStr"/>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E613" t="n">
+        <v>1258.75</v>
+      </c>
+      <c r="F613" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-Bocas-Consul-Vidro-Bivolt/dp/B076BC7769/ref=sr_1_7</t>
+        </is>
+      </c>
+      <c r="G613" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Atualiza preços de 2026-09-26
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G613"/>
+  <dimension ref="A1:G634"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13741,9 +13741,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D593" t="inlineStr"/>
-      <c r="E593" t="inlineStr"/>
-      <c r="F593" t="inlineStr"/>
       <c r="G593" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -13766,9 +13763,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D594" t="inlineStr"/>
-      <c r="E594" t="inlineStr"/>
-      <c r="F594" t="inlineStr"/>
       <c r="G594" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -13791,9 +13785,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D595" t="inlineStr"/>
-      <c r="E595" t="inlineStr"/>
-      <c r="F595" t="inlineStr"/>
       <c r="G595" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -13816,9 +13807,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D596" t="inlineStr"/>
-      <c r="E596" t="inlineStr"/>
-      <c r="F596" t="inlineStr"/>
       <c r="G596" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -13849,7 +13837,6 @@
           <t>https://www.amazon.com.br/Geladeira-BRM46MK-Duplex-Extrafrio-Brastemp/dp/B0GL3Q3PTG/ref=sr_1_3</t>
         </is>
       </c>
-      <c r="G597" t="inlineStr"/>
     </row>
     <row r="598">
       <c r="A598" t="inlineStr">
@@ -13875,7 +13862,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Duplex-litros-Branca/dp/B07FXZ8TR6/ref=sr_1_4</t>
         </is>
       </c>
-      <c r="G598" t="inlineStr"/>
     </row>
     <row r="599">
       <c r="A599" t="inlineStr">
@@ -13901,7 +13887,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWSXQGL/ref=sr_1_5</t>
         </is>
       </c>
-      <c r="G599" t="inlineStr"/>
     </row>
     <row r="600">
       <c r="A600" t="inlineStr">
@@ -13919,9 +13904,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D600" t="inlineStr"/>
-      <c r="E600" t="inlineStr"/>
-      <c r="F600" t="inlineStr"/>
       <c r="G600" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -13944,9 +13926,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D601" t="inlineStr"/>
-      <c r="E601" t="inlineStr"/>
-      <c r="F601" t="inlineStr"/>
       <c r="G601" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -13969,9 +13948,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D602" t="inlineStr"/>
-      <c r="E602" t="inlineStr"/>
-      <c r="F602" t="inlineStr"/>
       <c r="G602" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -13994,9 +13970,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D603" t="inlineStr"/>
-      <c r="E603" t="inlineStr"/>
-      <c r="F603" t="inlineStr"/>
       <c r="G603" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -14027,7 +14000,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Tira-Odor-MT30S/dp/B079Y3MLSP/ref=sr_1_1</t>
         </is>
       </c>
-      <c r="G604" t="inlineStr"/>
     </row>
     <row r="605">
       <c r="A605" t="inlineStr">
@@ -14053,7 +14025,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Electrolux-MTO30-Fun%C3%A7%C3%A3o-Tira/dp/B083ZFFC5Q/ref=sr_1_2</t>
         </is>
       </c>
-      <c r="G605" t="inlineStr"/>
     </row>
     <row r="606">
       <c r="A606" t="inlineStr">
@@ -14079,7 +14050,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Efficient-23L-ME23B/dp/B0B8KWNK12/ref=sr_1_3</t>
         </is>
       </c>
-      <c r="G606" t="inlineStr"/>
     </row>
     <row r="607">
       <c r="A607" t="inlineStr">
@@ -14097,9 +14067,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D607" t="inlineStr"/>
-      <c r="E607" t="inlineStr"/>
-      <c r="F607" t="inlineStr"/>
       <c r="G607" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -14122,9 +14089,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D608" t="inlineStr"/>
-      <c r="E608" t="inlineStr"/>
-      <c r="F608" t="inlineStr"/>
       <c r="G608" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -14147,9 +14111,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D609" t="inlineStr"/>
-      <c r="E609" t="inlineStr"/>
-      <c r="F609" t="inlineStr"/>
       <c r="G609" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -14172,9 +14133,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D610" t="inlineStr"/>
-      <c r="E610" t="inlineStr"/>
-      <c r="F610" t="inlineStr"/>
       <c r="G610" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -14205,7 +14163,6 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-04-Bocas-FS-CF04NABUNA/dp/B07JPZN51P/ref=sr_1_5</t>
         </is>
       </c>
-      <c r="G611" t="inlineStr"/>
     </row>
     <row r="612">
       <c r="A612" t="inlineStr">
@@ -14231,7 +14188,6 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-Consul-Bocas-CFO4NARUNA-Bivolt/dp/B07HM9JL5K/ref=sr_1_6</t>
         </is>
       </c>
-      <c r="G612" t="inlineStr"/>
     </row>
     <row r="613">
       <c r="A613" t="inlineStr">
@@ -14257,7 +14213,540 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-Bocas-Consul-Vidro-Bivolt/dp/B076BC7769/ref=sr_1_7</t>
         </is>
       </c>
-      <c r="G613" t="inlineStr"/>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D614" t="inlineStr"/>
+      <c r="E614" t="inlineStr"/>
+      <c r="F614" t="inlineStr"/>
+      <c r="G614" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D615" t="inlineStr"/>
+      <c r="E615" t="inlineStr"/>
+      <c r="F615" t="inlineStr"/>
+      <c r="G615" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D616" t="inlineStr"/>
+      <c r="E616" t="inlineStr"/>
+      <c r="F616" t="inlineStr"/>
+      <c r="G616" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D617" t="inlineStr"/>
+      <c r="E617" t="inlineStr"/>
+      <c r="F617" t="inlineStr"/>
+      <c r="G617" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E618" t="n">
+        <v>2899.9</v>
+      </c>
+      <c r="F618" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Duplex-litros-Branca/dp/B07FXZ8TR6/ref=sr_1_1</t>
+        </is>
+      </c>
+      <c r="G618" t="inlineStr"/>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E619" t="n">
+        <v>3048.61</v>
+      </c>
+      <c r="F619" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWVJ8LR/ref=sr_1_2</t>
+        </is>
+      </c>
+      <c r="G619" t="inlineStr"/>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E620" t="n">
+        <v>2820.65</v>
+      </c>
+      <c r="F620" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-BRM46MK-Duplex-Extrafrio-Brastemp/dp/B0GL3Q3PTG/ref=sr_1_3</t>
+        </is>
+      </c>
+      <c r="G620" t="inlineStr"/>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D621" t="inlineStr"/>
+      <c r="E621" t="inlineStr"/>
+      <c r="F621" t="inlineStr"/>
+      <c r="G621" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D622" t="inlineStr"/>
+      <c r="E622" t="inlineStr"/>
+      <c r="F622" t="inlineStr"/>
+      <c r="G622" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D623" t="inlineStr"/>
+      <c r="E623" t="inlineStr"/>
+      <c r="F623" t="inlineStr"/>
+      <c r="G623" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D624" t="inlineStr"/>
+      <c r="E624" t="inlineStr"/>
+      <c r="F624" t="inlineStr"/>
+      <c r="G624" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E625" t="n">
+        <v>476.1</v>
+      </c>
+      <c r="F625" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Tira-Odor-MT30S/dp/B079Y3MLSP/ref=sr_1_3</t>
+        </is>
+      </c>
+      <c r="G625" t="inlineStr"/>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E626" t="n">
+        <v>476.1</v>
+      </c>
+      <c r="F626" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Tira-Odor-MT30S/dp/B079Y3MLSP/ref=sr_1_3_so_MICROWAVE_OVEN</t>
+        </is>
+      </c>
+      <c r="G626" t="inlineStr"/>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E627" t="n">
+        <v>509</v>
+      </c>
+      <c r="F627" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Electrolux-MTO30-Fun%C3%A7%C3%A3o-Tira/dp/B083ZFFC5Q/ref=sr_1_4</t>
+        </is>
+      </c>
+      <c r="G627" t="inlineStr"/>
+    </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D628" t="inlineStr"/>
+      <c r="E628" t="inlineStr"/>
+      <c r="F628" t="inlineStr"/>
+      <c r="G628" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D629" t="inlineStr"/>
+      <c r="E629" t="inlineStr"/>
+      <c r="F629" t="inlineStr"/>
+      <c r="G629" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D630" t="inlineStr"/>
+      <c r="E630" t="inlineStr"/>
+      <c r="F630" t="inlineStr"/>
+      <c r="G630" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D631" t="inlineStr"/>
+      <c r="E631" t="inlineStr"/>
+      <c r="F631" t="inlineStr"/>
+      <c r="G631" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E632" t="n">
+        <v>1195.81</v>
+      </c>
+      <c r="F632" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-Consul-Bocas-CFO4NARUNA-Bivolt/dp/B07HM9JL5K/ref=sr_1_1</t>
+        </is>
+      </c>
+      <c r="G632" t="inlineStr"/>
+    </row>
+    <row r="633">
+      <c r="A633" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E633" t="n">
+        <v>1218.5</v>
+      </c>
+      <c r="F633" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-04-Bocas-FS-CF04NABUNA/dp/B07JPZN51P/ref=sr_1_2</t>
+        </is>
+      </c>
+      <c r="G633" t="inlineStr"/>
+    </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E634" t="n">
+        <v>1443.09</v>
+      </c>
+      <c r="F634" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-Bocas-Consul-Vidro-Bivolt/dp/B076BC7769/ref=sr_1_3</t>
+        </is>
+      </c>
+      <c r="G634" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Atualiza preços de 2026-09-27
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G634"/>
+  <dimension ref="A1:G655"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14230,9 +14230,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D614" t="inlineStr"/>
-      <c r="E614" t="inlineStr"/>
-      <c r="F614" t="inlineStr"/>
       <c r="G614" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -14255,9 +14252,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D615" t="inlineStr"/>
-      <c r="E615" t="inlineStr"/>
-      <c r="F615" t="inlineStr"/>
       <c r="G615" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -14280,9 +14274,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D616" t="inlineStr"/>
-      <c r="E616" t="inlineStr"/>
-      <c r="F616" t="inlineStr"/>
       <c r="G616" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -14305,9 +14296,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D617" t="inlineStr"/>
-      <c r="E617" t="inlineStr"/>
-      <c r="F617" t="inlineStr"/>
       <c r="G617" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -14338,7 +14326,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Duplex-litros-Branca/dp/B07FXZ8TR6/ref=sr_1_1</t>
         </is>
       </c>
-      <c r="G618" t="inlineStr"/>
     </row>
     <row r="619">
       <c r="A619" t="inlineStr">
@@ -14364,7 +14351,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWVJ8LR/ref=sr_1_2</t>
         </is>
       </c>
-      <c r="G619" t="inlineStr"/>
     </row>
     <row r="620">
       <c r="A620" t="inlineStr">
@@ -14390,7 +14376,6 @@
           <t>https://www.amazon.com.br/Geladeira-BRM46MK-Duplex-Extrafrio-Brastemp/dp/B0GL3Q3PTG/ref=sr_1_3</t>
         </is>
       </c>
-      <c r="G620" t="inlineStr"/>
     </row>
     <row r="621">
       <c r="A621" t="inlineStr">
@@ -14408,9 +14393,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D621" t="inlineStr"/>
-      <c r="E621" t="inlineStr"/>
-      <c r="F621" t="inlineStr"/>
       <c r="G621" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -14433,9 +14415,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D622" t="inlineStr"/>
-      <c r="E622" t="inlineStr"/>
-      <c r="F622" t="inlineStr"/>
       <c r="G622" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -14458,9 +14437,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D623" t="inlineStr"/>
-      <c r="E623" t="inlineStr"/>
-      <c r="F623" t="inlineStr"/>
       <c r="G623" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -14483,9 +14459,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D624" t="inlineStr"/>
-      <c r="E624" t="inlineStr"/>
-      <c r="F624" t="inlineStr"/>
       <c r="G624" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -14516,7 +14489,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Tira-Odor-MT30S/dp/B079Y3MLSP/ref=sr_1_3</t>
         </is>
       </c>
-      <c r="G625" t="inlineStr"/>
     </row>
     <row r="626">
       <c r="A626" t="inlineStr">
@@ -14542,7 +14514,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Tira-Odor-MT30S/dp/B079Y3MLSP/ref=sr_1_3_so_MICROWAVE_OVEN</t>
         </is>
       </c>
-      <c r="G626" t="inlineStr"/>
     </row>
     <row r="627">
       <c r="A627" t="inlineStr">
@@ -14568,7 +14539,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Electrolux-MTO30-Fun%C3%A7%C3%A3o-Tira/dp/B083ZFFC5Q/ref=sr_1_4</t>
         </is>
       </c>
-      <c r="G627" t="inlineStr"/>
     </row>
     <row r="628">
       <c r="A628" t="inlineStr">
@@ -14586,9 +14556,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D628" t="inlineStr"/>
-      <c r="E628" t="inlineStr"/>
-      <c r="F628" t="inlineStr"/>
       <c r="G628" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -14611,9 +14578,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D629" t="inlineStr"/>
-      <c r="E629" t="inlineStr"/>
-      <c r="F629" t="inlineStr"/>
       <c r="G629" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -14636,9 +14600,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D630" t="inlineStr"/>
-      <c r="E630" t="inlineStr"/>
-      <c r="F630" t="inlineStr"/>
       <c r="G630" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -14661,9 +14622,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D631" t="inlineStr"/>
-      <c r="E631" t="inlineStr"/>
-      <c r="F631" t="inlineStr"/>
       <c r="G631" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -14694,7 +14652,6 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-Consul-Bocas-CFO4NARUNA-Bivolt/dp/B07HM9JL5K/ref=sr_1_1</t>
         </is>
       </c>
-      <c r="G632" t="inlineStr"/>
     </row>
     <row r="633">
       <c r="A633" t="inlineStr">
@@ -14720,7 +14677,6 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-04-Bocas-FS-CF04NABUNA/dp/B07JPZN51P/ref=sr_1_2</t>
         </is>
       </c>
-      <c r="G633" t="inlineStr"/>
     </row>
     <row r="634">
       <c r="A634" t="inlineStr">
@@ -14746,7 +14702,540 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-Bocas-Consul-Vidro-Bivolt/dp/B076BC7769/ref=sr_1_3</t>
         </is>
       </c>
-      <c r="G634" t="inlineStr"/>
+    </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D635" t="inlineStr"/>
+      <c r="E635" t="inlineStr"/>
+      <c r="F635" t="inlineStr"/>
+      <c r="G635" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D636" t="inlineStr"/>
+      <c r="E636" t="inlineStr"/>
+      <c r="F636" t="inlineStr"/>
+      <c r="G636" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D637" t="inlineStr"/>
+      <c r="E637" t="inlineStr"/>
+      <c r="F637" t="inlineStr"/>
+      <c r="G637" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D638" t="inlineStr"/>
+      <c r="E638" t="inlineStr"/>
+      <c r="F638" t="inlineStr"/>
+      <c r="G638" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E639" t="n">
+        <v>2799</v>
+      </c>
+      <c r="F639" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Duplex-litros-Branca/dp/B07FXZ8TR6/ref=sr_1_1</t>
+        </is>
+      </c>
+      <c r="G639" t="inlineStr"/>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E640" t="n">
+        <v>3048.61</v>
+      </c>
+      <c r="F640" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWVJ8LR/ref=sr_1_2</t>
+        </is>
+      </c>
+      <c r="G640" t="inlineStr"/>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E641" t="n">
+        <v>2849.99</v>
+      </c>
+      <c r="F641" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-BRM46MK-Duplex-Extrafrio-Brastemp/dp/B0GL3Q3PTG/ref=sr_1_3</t>
+        </is>
+      </c>
+      <c r="G641" t="inlineStr"/>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D642" t="inlineStr"/>
+      <c r="E642" t="inlineStr"/>
+      <c r="F642" t="inlineStr"/>
+      <c r="G642" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D643" t="inlineStr"/>
+      <c r="E643" t="inlineStr"/>
+      <c r="F643" t="inlineStr"/>
+      <c r="G643" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D644" t="inlineStr"/>
+      <c r="E644" t="inlineStr"/>
+      <c r="F644" t="inlineStr"/>
+      <c r="G644" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D645" t="inlineStr"/>
+      <c r="E645" t="inlineStr"/>
+      <c r="F645" t="inlineStr"/>
+      <c r="G645" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E646" t="n">
+        <v>739</v>
+      </c>
+      <c r="F646" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Tira-Odor-MT30S/dp/B079Y3MLSP/ref=sr_1_4</t>
+        </is>
+      </c>
+      <c r="G646" t="inlineStr"/>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E647" t="n">
+        <v>490.1</v>
+      </c>
+      <c r="F647" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P2FLSR/ref=sr_1_5</t>
+        </is>
+      </c>
+      <c r="G647" t="inlineStr"/>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E648" t="n">
+        <v>483.55</v>
+      </c>
+      <c r="F648" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Electrolux-MTO30-Fun%C3%A7%C3%A3o-Tira/dp/B083ZFFC5Q/ref=sr_1_6</t>
+        </is>
+      </c>
+      <c r="G648" t="inlineStr"/>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D649" t="inlineStr"/>
+      <c r="E649" t="inlineStr"/>
+      <c r="F649" t="inlineStr"/>
+      <c r="G649" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D650" t="inlineStr"/>
+      <c r="E650" t="inlineStr"/>
+      <c r="F650" t="inlineStr"/>
+      <c r="G650" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D651" t="inlineStr"/>
+      <c r="E651" t="inlineStr"/>
+      <c r="F651" t="inlineStr"/>
+      <c r="G651" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D652" t="inlineStr"/>
+      <c r="E652" t="inlineStr"/>
+      <c r="F652" t="inlineStr"/>
+      <c r="G652" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E653" t="n">
+        <v>1258.75</v>
+      </c>
+      <c r="F653" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-Consul-Bocas-CFO4NARUNA-Bivolt/dp/B07HM9JL5K/ref=sr_1_5</t>
+        </is>
+      </c>
+      <c r="G653" t="inlineStr"/>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E654" t="n">
+        <v>1099</v>
+      </c>
+      <c r="F654" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-04-Bocas-FS-CF04NABUNA/dp/B07JPZN51P/ref=sr_1_6</t>
+        </is>
+      </c>
+      <c r="G654" t="inlineStr"/>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E655" t="n">
+        <v>1519.05</v>
+      </c>
+      <c r="F655" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-Bocas-Consul-Vidro-Bivolt/dp/B076BC7769/ref=sr_1_7</t>
+        </is>
+      </c>
+      <c r="G655" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Atualiza preços de 2026-09-28
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G655"/>
+  <dimension ref="A1:G670"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14719,9 +14719,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D635" t="inlineStr"/>
-      <c r="E635" t="inlineStr"/>
-      <c r="F635" t="inlineStr"/>
       <c r="G635" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -14744,9 +14741,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D636" t="inlineStr"/>
-      <c r="E636" t="inlineStr"/>
-      <c r="F636" t="inlineStr"/>
       <c r="G636" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -14769,9 +14763,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D637" t="inlineStr"/>
-      <c r="E637" t="inlineStr"/>
-      <c r="F637" t="inlineStr"/>
       <c r="G637" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -14794,9 +14785,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D638" t="inlineStr"/>
-      <c r="E638" t="inlineStr"/>
-      <c r="F638" t="inlineStr"/>
       <c r="G638" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -14827,7 +14815,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Duplex-litros-Branca/dp/B07FXZ8TR6/ref=sr_1_1</t>
         </is>
       </c>
-      <c r="G639" t="inlineStr"/>
     </row>
     <row r="640">
       <c r="A640" t="inlineStr">
@@ -14853,7 +14840,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWVJ8LR/ref=sr_1_2</t>
         </is>
       </c>
-      <c r="G640" t="inlineStr"/>
     </row>
     <row r="641">
       <c r="A641" t="inlineStr">
@@ -14879,7 +14865,6 @@
           <t>https://www.amazon.com.br/Geladeira-BRM46MK-Duplex-Extrafrio-Brastemp/dp/B0GL3Q3PTG/ref=sr_1_3</t>
         </is>
       </c>
-      <c r="G641" t="inlineStr"/>
     </row>
     <row r="642">
       <c r="A642" t="inlineStr">
@@ -14897,9 +14882,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D642" t="inlineStr"/>
-      <c r="E642" t="inlineStr"/>
-      <c r="F642" t="inlineStr"/>
       <c r="G642" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -14922,9 +14904,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D643" t="inlineStr"/>
-      <c r="E643" t="inlineStr"/>
-      <c r="F643" t="inlineStr"/>
       <c r="G643" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -14947,9 +14926,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D644" t="inlineStr"/>
-      <c r="E644" t="inlineStr"/>
-      <c r="F644" t="inlineStr"/>
       <c r="G644" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -14972,9 +14948,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D645" t="inlineStr"/>
-      <c r="E645" t="inlineStr"/>
-      <c r="F645" t="inlineStr"/>
       <c r="G645" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -15005,7 +14978,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Tira-Odor-MT30S/dp/B079Y3MLSP/ref=sr_1_4</t>
         </is>
       </c>
-      <c r="G646" t="inlineStr"/>
     </row>
     <row r="647">
       <c r="A647" t="inlineStr">
@@ -15031,7 +15003,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P2FLSR/ref=sr_1_5</t>
         </is>
       </c>
-      <c r="G647" t="inlineStr"/>
     </row>
     <row r="648">
       <c r="A648" t="inlineStr">
@@ -15057,7 +15028,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Electrolux-MTO30-Fun%C3%A7%C3%A3o-Tira/dp/B083ZFFC5Q/ref=sr_1_6</t>
         </is>
       </c>
-      <c r="G648" t="inlineStr"/>
     </row>
     <row r="649">
       <c r="A649" t="inlineStr">
@@ -15075,9 +15045,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D649" t="inlineStr"/>
-      <c r="E649" t="inlineStr"/>
-      <c r="F649" t="inlineStr"/>
       <c r="G649" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -15100,9 +15067,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D650" t="inlineStr"/>
-      <c r="E650" t="inlineStr"/>
-      <c r="F650" t="inlineStr"/>
       <c r="G650" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -15125,9 +15089,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D651" t="inlineStr"/>
-      <c r="E651" t="inlineStr"/>
-      <c r="F651" t="inlineStr"/>
       <c r="G651" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -15150,9 +15111,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D652" t="inlineStr"/>
-      <c r="E652" t="inlineStr"/>
-      <c r="F652" t="inlineStr"/>
       <c r="G652" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -15183,7 +15141,6 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-Consul-Bocas-CFO4NARUNA-Bivolt/dp/B07HM9JL5K/ref=sr_1_5</t>
         </is>
       </c>
-      <c r="G653" t="inlineStr"/>
     </row>
     <row r="654">
       <c r="A654" t="inlineStr">
@@ -15209,7 +15166,6 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-04-Bocas-FS-CF04NABUNA/dp/B07JPZN51P/ref=sr_1_6</t>
         </is>
       </c>
-      <c r="G654" t="inlineStr"/>
     </row>
     <row r="655">
       <c r="A655" t="inlineStr">
@@ -15235,7 +15191,381 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-Bocas-Consul-Vidro-Bivolt/dp/B076BC7769/ref=sr_1_7</t>
         </is>
       </c>
-      <c r="G655" t="inlineStr"/>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D656" t="inlineStr"/>
+      <c r="E656" t="inlineStr"/>
+      <c r="F656" t="inlineStr"/>
+      <c r="G656" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D657" t="inlineStr"/>
+      <c r="E657" t="inlineStr"/>
+      <c r="F657" t="inlineStr"/>
+      <c r="G657" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D658" t="inlineStr"/>
+      <c r="E658" t="inlineStr"/>
+      <c r="F658" t="inlineStr"/>
+      <c r="G658" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D659" t="inlineStr"/>
+      <c r="E659" t="inlineStr"/>
+      <c r="F659" t="inlineStr"/>
+      <c r="G659" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D660" t="inlineStr"/>
+      <c r="E660" t="inlineStr"/>
+      <c r="F660" t="inlineStr"/>
+      <c r="G660" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D661" t="inlineStr"/>
+      <c r="E661" t="inlineStr"/>
+      <c r="F661" t="inlineStr"/>
+      <c r="G661" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D662" t="inlineStr"/>
+      <c r="E662" t="inlineStr"/>
+      <c r="F662" t="inlineStr"/>
+      <c r="G662" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D663" t="inlineStr"/>
+      <c r="E663" t="inlineStr"/>
+      <c r="F663" t="inlineStr"/>
+      <c r="G663" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D664" t="inlineStr"/>
+      <c r="E664" t="inlineStr"/>
+      <c r="F664" t="inlineStr"/>
+      <c r="G664" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D665" t="inlineStr"/>
+      <c r="E665" t="inlineStr"/>
+      <c r="F665" t="inlineStr"/>
+      <c r="G665" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D666" t="inlineStr"/>
+      <c r="E666" t="inlineStr"/>
+      <c r="F666" t="inlineStr"/>
+      <c r="G666" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D667" t="inlineStr"/>
+      <c r="E667" t="inlineStr"/>
+      <c r="F667" t="inlineStr"/>
+      <c r="G667" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D668" t="inlineStr"/>
+      <c r="E668" t="inlineStr"/>
+      <c r="F668" t="inlineStr"/>
+      <c r="G668" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D669" t="inlineStr"/>
+      <c r="E669" t="inlineStr"/>
+      <c r="F669" t="inlineStr"/>
+      <c r="G669" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D670" t="inlineStr"/>
+      <c r="E670" t="inlineStr"/>
+      <c r="F670" t="inlineStr"/>
+      <c r="G670" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Atualiza preços de 2026-09-29
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G670"/>
+  <dimension ref="A1:G685"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15208,9 +15208,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D656" t="inlineStr"/>
-      <c r="E656" t="inlineStr"/>
-      <c r="F656" t="inlineStr"/>
       <c r="G656" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -15233,9 +15230,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D657" t="inlineStr"/>
-      <c r="E657" t="inlineStr"/>
-      <c r="F657" t="inlineStr"/>
       <c r="G657" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -15258,9 +15252,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D658" t="inlineStr"/>
-      <c r="E658" t="inlineStr"/>
-      <c r="F658" t="inlineStr"/>
       <c r="G658" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -15283,9 +15274,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D659" t="inlineStr"/>
-      <c r="E659" t="inlineStr"/>
-      <c r="F659" t="inlineStr"/>
       <c r="G659" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -15308,9 +15296,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D660" t="inlineStr"/>
-      <c r="E660" t="inlineStr"/>
-      <c r="F660" t="inlineStr"/>
       <c r="G660" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -15333,9 +15318,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D661" t="inlineStr"/>
-      <c r="E661" t="inlineStr"/>
-      <c r="F661" t="inlineStr"/>
       <c r="G661" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -15358,9 +15340,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D662" t="inlineStr"/>
-      <c r="E662" t="inlineStr"/>
-      <c r="F662" t="inlineStr"/>
       <c r="G662" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -15383,9 +15362,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D663" t="inlineStr"/>
-      <c r="E663" t="inlineStr"/>
-      <c r="F663" t="inlineStr"/>
       <c r="G663" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -15408,9 +15384,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D664" t="inlineStr"/>
-      <c r="E664" t="inlineStr"/>
-      <c r="F664" t="inlineStr"/>
       <c r="G664" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -15433,9 +15406,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D665" t="inlineStr"/>
-      <c r="E665" t="inlineStr"/>
-      <c r="F665" t="inlineStr"/>
       <c r="G665" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -15458,9 +15428,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D666" t="inlineStr"/>
-      <c r="E666" t="inlineStr"/>
-      <c r="F666" t="inlineStr"/>
       <c r="G666" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -15483,9 +15450,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D667" t="inlineStr"/>
-      <c r="E667" t="inlineStr"/>
-      <c r="F667" t="inlineStr"/>
       <c r="G667" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -15508,9 +15472,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D668" t="inlineStr"/>
-      <c r="E668" t="inlineStr"/>
-      <c r="F668" t="inlineStr"/>
       <c r="G668" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -15533,9 +15494,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D669" t="inlineStr"/>
-      <c r="E669" t="inlineStr"/>
-      <c r="F669" t="inlineStr"/>
       <c r="G669" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -15558,10 +15516,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D670" t="inlineStr"/>
-      <c r="E670" t="inlineStr"/>
-      <c r="F670" t="inlineStr"/>
       <c r="G670" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D671" t="inlineStr"/>
+      <c r="E671" t="inlineStr"/>
+      <c r="F671" t="inlineStr"/>
+      <c r="G671" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D672" t="inlineStr"/>
+      <c r="E672" t="inlineStr"/>
+      <c r="F672" t="inlineStr"/>
+      <c r="G672" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D673" t="inlineStr"/>
+      <c r="E673" t="inlineStr"/>
+      <c r="F673" t="inlineStr"/>
+      <c r="G673" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D674" t="inlineStr"/>
+      <c r="E674" t="inlineStr"/>
+      <c r="F674" t="inlineStr"/>
+      <c r="G674" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D675" t="inlineStr"/>
+      <c r="E675" t="inlineStr"/>
+      <c r="F675" t="inlineStr"/>
+      <c r="G675" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D676" t="inlineStr"/>
+      <c r="E676" t="inlineStr"/>
+      <c r="F676" t="inlineStr"/>
+      <c r="G676" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D677" t="inlineStr"/>
+      <c r="E677" t="inlineStr"/>
+      <c r="F677" t="inlineStr"/>
+      <c r="G677" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D678" t="inlineStr"/>
+      <c r="E678" t="inlineStr"/>
+      <c r="F678" t="inlineStr"/>
+      <c r="G678" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D679" t="inlineStr"/>
+      <c r="E679" t="inlineStr"/>
+      <c r="F679" t="inlineStr"/>
+      <c r="G679" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D680" t="inlineStr"/>
+      <c r="E680" t="inlineStr"/>
+      <c r="F680" t="inlineStr"/>
+      <c r="G680" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D681" t="inlineStr"/>
+      <c r="E681" t="inlineStr"/>
+      <c r="F681" t="inlineStr"/>
+      <c r="G681" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D682" t="inlineStr"/>
+      <c r="E682" t="inlineStr"/>
+      <c r="F682" t="inlineStr"/>
+      <c r="G682" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D683" t="inlineStr"/>
+      <c r="E683" t="inlineStr"/>
+      <c r="F683" t="inlineStr"/>
+      <c r="G683" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D684" t="inlineStr"/>
+      <c r="E684" t="inlineStr"/>
+      <c r="F684" t="inlineStr"/>
+      <c r="G684" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D685" t="inlineStr"/>
+      <c r="E685" t="inlineStr"/>
+      <c r="F685" t="inlineStr"/>
+      <c r="G685" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-09-30
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G685"/>
+  <dimension ref="A1:G700"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15538,9 +15538,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D671" t="inlineStr"/>
-      <c r="E671" t="inlineStr"/>
-      <c r="F671" t="inlineStr"/>
       <c r="G671" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -15563,9 +15560,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D672" t="inlineStr"/>
-      <c r="E672" t="inlineStr"/>
-      <c r="F672" t="inlineStr"/>
       <c r="G672" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -15588,9 +15582,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D673" t="inlineStr"/>
-      <c r="E673" t="inlineStr"/>
-      <c r="F673" t="inlineStr"/>
       <c r="G673" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -15613,9 +15604,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D674" t="inlineStr"/>
-      <c r="E674" t="inlineStr"/>
-      <c r="F674" t="inlineStr"/>
       <c r="G674" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -15638,9 +15626,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D675" t="inlineStr"/>
-      <c r="E675" t="inlineStr"/>
-      <c r="F675" t="inlineStr"/>
       <c r="G675" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -15663,9 +15648,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D676" t="inlineStr"/>
-      <c r="E676" t="inlineStr"/>
-      <c r="F676" t="inlineStr"/>
       <c r="G676" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -15688,9 +15670,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D677" t="inlineStr"/>
-      <c r="E677" t="inlineStr"/>
-      <c r="F677" t="inlineStr"/>
       <c r="G677" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -15713,9 +15692,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D678" t="inlineStr"/>
-      <c r="E678" t="inlineStr"/>
-      <c r="F678" t="inlineStr"/>
       <c r="G678" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -15738,9 +15714,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D679" t="inlineStr"/>
-      <c r="E679" t="inlineStr"/>
-      <c r="F679" t="inlineStr"/>
       <c r="G679" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -15763,9 +15736,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D680" t="inlineStr"/>
-      <c r="E680" t="inlineStr"/>
-      <c r="F680" t="inlineStr"/>
       <c r="G680" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -15788,9 +15758,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D681" t="inlineStr"/>
-      <c r="E681" t="inlineStr"/>
-      <c r="F681" t="inlineStr"/>
       <c r="G681" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -15813,9 +15780,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D682" t="inlineStr"/>
-      <c r="E682" t="inlineStr"/>
-      <c r="F682" t="inlineStr"/>
       <c r="G682" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -15838,9 +15802,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D683" t="inlineStr"/>
-      <c r="E683" t="inlineStr"/>
-      <c r="F683" t="inlineStr"/>
       <c r="G683" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -15863,9 +15824,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D684" t="inlineStr"/>
-      <c r="E684" t="inlineStr"/>
-      <c r="F684" t="inlineStr"/>
       <c r="G684" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -15888,10 +15846,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D685" t="inlineStr"/>
-      <c r="E685" t="inlineStr"/>
-      <c r="F685" t="inlineStr"/>
       <c r="G685" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D686" t="inlineStr"/>
+      <c r="E686" t="inlineStr"/>
+      <c r="F686" t="inlineStr"/>
+      <c r="G686" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D687" t="inlineStr"/>
+      <c r="E687" t="inlineStr"/>
+      <c r="F687" t="inlineStr"/>
+      <c r="G687" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D688" t="inlineStr"/>
+      <c r="E688" t="inlineStr"/>
+      <c r="F688" t="inlineStr"/>
+      <c r="G688" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D689" t="inlineStr"/>
+      <c r="E689" t="inlineStr"/>
+      <c r="F689" t="inlineStr"/>
+      <c r="G689" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D690" t="inlineStr"/>
+      <c r="E690" t="inlineStr"/>
+      <c r="F690" t="inlineStr"/>
+      <c r="G690" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D691" t="inlineStr"/>
+      <c r="E691" t="inlineStr"/>
+      <c r="F691" t="inlineStr"/>
+      <c r="G691" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D692" t="inlineStr"/>
+      <c r="E692" t="inlineStr"/>
+      <c r="F692" t="inlineStr"/>
+      <c r="G692" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D693" t="inlineStr"/>
+      <c r="E693" t="inlineStr"/>
+      <c r="F693" t="inlineStr"/>
+      <c r="G693" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D694" t="inlineStr"/>
+      <c r="E694" t="inlineStr"/>
+      <c r="F694" t="inlineStr"/>
+      <c r="G694" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D695" t="inlineStr"/>
+      <c r="E695" t="inlineStr"/>
+      <c r="F695" t="inlineStr"/>
+      <c r="G695" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D696" t="inlineStr"/>
+      <c r="E696" t="inlineStr"/>
+      <c r="F696" t="inlineStr"/>
+      <c r="G696" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D697" t="inlineStr"/>
+      <c r="E697" t="inlineStr"/>
+      <c r="F697" t="inlineStr"/>
+      <c r="G697" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D698" t="inlineStr"/>
+      <c r="E698" t="inlineStr"/>
+      <c r="F698" t="inlineStr"/>
+      <c r="G698" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D699" t="inlineStr"/>
+      <c r="E699" t="inlineStr"/>
+      <c r="F699" t="inlineStr"/>
+      <c r="G699" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D700" t="inlineStr"/>
+      <c r="E700" t="inlineStr"/>
+      <c r="F700" t="inlineStr"/>
+      <c r="G700" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-10-01
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G700"/>
+  <dimension ref="A1:G715"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15868,9 +15868,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D686" t="inlineStr"/>
-      <c r="E686" t="inlineStr"/>
-      <c r="F686" t="inlineStr"/>
       <c r="G686" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -15893,9 +15890,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D687" t="inlineStr"/>
-      <c r="E687" t="inlineStr"/>
-      <c r="F687" t="inlineStr"/>
       <c r="G687" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -15918,9 +15912,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D688" t="inlineStr"/>
-      <c r="E688" t="inlineStr"/>
-      <c r="F688" t="inlineStr"/>
       <c r="G688" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -15943,9 +15934,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D689" t="inlineStr"/>
-      <c r="E689" t="inlineStr"/>
-      <c r="F689" t="inlineStr"/>
       <c r="G689" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -15968,9 +15956,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D690" t="inlineStr"/>
-      <c r="E690" t="inlineStr"/>
-      <c r="F690" t="inlineStr"/>
       <c r="G690" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -15993,9 +15978,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D691" t="inlineStr"/>
-      <c r="E691" t="inlineStr"/>
-      <c r="F691" t="inlineStr"/>
       <c r="G691" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16018,9 +16000,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D692" t="inlineStr"/>
-      <c r="E692" t="inlineStr"/>
-      <c r="F692" t="inlineStr"/>
       <c r="G692" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16043,9 +16022,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D693" t="inlineStr"/>
-      <c r="E693" t="inlineStr"/>
-      <c r="F693" t="inlineStr"/>
       <c r="G693" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16068,9 +16044,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D694" t="inlineStr"/>
-      <c r="E694" t="inlineStr"/>
-      <c r="F694" t="inlineStr"/>
       <c r="G694" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16093,9 +16066,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D695" t="inlineStr"/>
-      <c r="E695" t="inlineStr"/>
-      <c r="F695" t="inlineStr"/>
       <c r="G695" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16118,9 +16088,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D696" t="inlineStr"/>
-      <c r="E696" t="inlineStr"/>
-      <c r="F696" t="inlineStr"/>
       <c r="G696" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16143,9 +16110,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D697" t="inlineStr"/>
-      <c r="E697" t="inlineStr"/>
-      <c r="F697" t="inlineStr"/>
       <c r="G697" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16168,9 +16132,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D698" t="inlineStr"/>
-      <c r="E698" t="inlineStr"/>
-      <c r="F698" t="inlineStr"/>
       <c r="G698" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16193,9 +16154,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D699" t="inlineStr"/>
-      <c r="E699" t="inlineStr"/>
-      <c r="F699" t="inlineStr"/>
       <c r="G699" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16218,10 +16176,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D700" t="inlineStr"/>
-      <c r="E700" t="inlineStr"/>
-      <c r="F700" t="inlineStr"/>
       <c r="G700" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D701" t="inlineStr"/>
+      <c r="E701" t="inlineStr"/>
+      <c r="F701" t="inlineStr"/>
+      <c r="G701" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D702" t="inlineStr"/>
+      <c r="E702" t="inlineStr"/>
+      <c r="F702" t="inlineStr"/>
+      <c r="G702" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D703" t="inlineStr"/>
+      <c r="E703" t="inlineStr"/>
+      <c r="F703" t="inlineStr"/>
+      <c r="G703" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D704" t="inlineStr"/>
+      <c r="E704" t="inlineStr"/>
+      <c r="F704" t="inlineStr"/>
+      <c r="G704" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D705" t="inlineStr"/>
+      <c r="E705" t="inlineStr"/>
+      <c r="F705" t="inlineStr"/>
+      <c r="G705" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C706" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D706" t="inlineStr"/>
+      <c r="E706" t="inlineStr"/>
+      <c r="F706" t="inlineStr"/>
+      <c r="G706" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D707" t="inlineStr"/>
+      <c r="E707" t="inlineStr"/>
+      <c r="F707" t="inlineStr"/>
+      <c r="G707" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D708" t="inlineStr"/>
+      <c r="E708" t="inlineStr"/>
+      <c r="F708" t="inlineStr"/>
+      <c r="G708" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B709" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C709" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D709" t="inlineStr"/>
+      <c r="E709" t="inlineStr"/>
+      <c r="F709" t="inlineStr"/>
+      <c r="G709" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C710" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D710" t="inlineStr"/>
+      <c r="E710" t="inlineStr"/>
+      <c r="F710" t="inlineStr"/>
+      <c r="G710" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C711" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D711" t="inlineStr"/>
+      <c r="E711" t="inlineStr"/>
+      <c r="F711" t="inlineStr"/>
+      <c r="G711" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C712" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D712" t="inlineStr"/>
+      <c r="E712" t="inlineStr"/>
+      <c r="F712" t="inlineStr"/>
+      <c r="G712" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D713" t="inlineStr"/>
+      <c r="E713" t="inlineStr"/>
+      <c r="F713" t="inlineStr"/>
+      <c r="G713" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C714" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D714" t="inlineStr"/>
+      <c r="E714" t="inlineStr"/>
+      <c r="F714" t="inlineStr"/>
+      <c r="G714" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C715" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D715" t="inlineStr"/>
+      <c r="E715" t="inlineStr"/>
+      <c r="F715" t="inlineStr"/>
+      <c r="G715" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-10-02
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G715"/>
+  <dimension ref="A1:G730"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16198,9 +16198,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D701" t="inlineStr"/>
-      <c r="E701" t="inlineStr"/>
-      <c r="F701" t="inlineStr"/>
       <c r="G701" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16223,9 +16220,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D702" t="inlineStr"/>
-      <c r="E702" t="inlineStr"/>
-      <c r="F702" t="inlineStr"/>
       <c r="G702" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16248,9 +16242,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D703" t="inlineStr"/>
-      <c r="E703" t="inlineStr"/>
-      <c r="F703" t="inlineStr"/>
       <c r="G703" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16273,9 +16264,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D704" t="inlineStr"/>
-      <c r="E704" t="inlineStr"/>
-      <c r="F704" t="inlineStr"/>
       <c r="G704" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16298,9 +16286,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D705" t="inlineStr"/>
-      <c r="E705" t="inlineStr"/>
-      <c r="F705" t="inlineStr"/>
       <c r="G705" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16323,9 +16308,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D706" t="inlineStr"/>
-      <c r="E706" t="inlineStr"/>
-      <c r="F706" t="inlineStr"/>
       <c r="G706" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16348,9 +16330,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D707" t="inlineStr"/>
-      <c r="E707" t="inlineStr"/>
-      <c r="F707" t="inlineStr"/>
       <c r="G707" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16373,9 +16352,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D708" t="inlineStr"/>
-      <c r="E708" t="inlineStr"/>
-      <c r="F708" t="inlineStr"/>
       <c r="G708" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16398,9 +16374,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D709" t="inlineStr"/>
-      <c r="E709" t="inlineStr"/>
-      <c r="F709" t="inlineStr"/>
       <c r="G709" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16423,9 +16396,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D710" t="inlineStr"/>
-      <c r="E710" t="inlineStr"/>
-      <c r="F710" t="inlineStr"/>
       <c r="G710" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16448,9 +16418,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D711" t="inlineStr"/>
-      <c r="E711" t="inlineStr"/>
-      <c r="F711" t="inlineStr"/>
       <c r="G711" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16473,9 +16440,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D712" t="inlineStr"/>
-      <c r="E712" t="inlineStr"/>
-      <c r="F712" t="inlineStr"/>
       <c r="G712" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16498,9 +16462,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D713" t="inlineStr"/>
-      <c r="E713" t="inlineStr"/>
-      <c r="F713" t="inlineStr"/>
       <c r="G713" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16523,9 +16484,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D714" t="inlineStr"/>
-      <c r="E714" t="inlineStr"/>
-      <c r="F714" t="inlineStr"/>
       <c r="G714" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16548,10 +16506,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D715" t="inlineStr"/>
-      <c r="E715" t="inlineStr"/>
-      <c r="F715" t="inlineStr"/>
       <c r="G715" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B716" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C716" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D716" t="inlineStr"/>
+      <c r="E716" t="inlineStr"/>
+      <c r="F716" t="inlineStr"/>
+      <c r="G716" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C717" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D717" t="inlineStr"/>
+      <c r="E717" t="inlineStr"/>
+      <c r="F717" t="inlineStr"/>
+      <c r="G717" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C718" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D718" t="inlineStr"/>
+      <c r="E718" t="inlineStr"/>
+      <c r="F718" t="inlineStr"/>
+      <c r="G718" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B719" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C719" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D719" t="inlineStr"/>
+      <c r="E719" t="inlineStr"/>
+      <c r="F719" t="inlineStr"/>
+      <c r="G719" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C720" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D720" t="inlineStr"/>
+      <c r="E720" t="inlineStr"/>
+      <c r="F720" t="inlineStr"/>
+      <c r="G720" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C721" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D721" t="inlineStr"/>
+      <c r="E721" t="inlineStr"/>
+      <c r="F721" t="inlineStr"/>
+      <c r="G721" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C722" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D722" t="inlineStr"/>
+      <c r="E722" t="inlineStr"/>
+      <c r="F722" t="inlineStr"/>
+      <c r="G722" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C723" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D723" t="inlineStr"/>
+      <c r="E723" t="inlineStr"/>
+      <c r="F723" t="inlineStr"/>
+      <c r="G723" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C724" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D724" t="inlineStr"/>
+      <c r="E724" t="inlineStr"/>
+      <c r="F724" t="inlineStr"/>
+      <c r="G724" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B725" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C725" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D725" t="inlineStr"/>
+      <c r="E725" t="inlineStr"/>
+      <c r="F725" t="inlineStr"/>
+      <c r="G725" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C726" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D726" t="inlineStr"/>
+      <c r="E726" t="inlineStr"/>
+      <c r="F726" t="inlineStr"/>
+      <c r="G726" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B727" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C727" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D727" t="inlineStr"/>
+      <c r="E727" t="inlineStr"/>
+      <c r="F727" t="inlineStr"/>
+      <c r="G727" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C728" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D728" t="inlineStr"/>
+      <c r="E728" t="inlineStr"/>
+      <c r="F728" t="inlineStr"/>
+      <c r="G728" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B729" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C729" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D729" t="inlineStr"/>
+      <c r="E729" t="inlineStr"/>
+      <c r="F729" t="inlineStr"/>
+      <c r="G729" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C730" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D730" t="inlineStr"/>
+      <c r="E730" t="inlineStr"/>
+      <c r="F730" t="inlineStr"/>
+      <c r="G730" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-10-03
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G730"/>
+  <dimension ref="A1:G745"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16528,9 +16528,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D716" t="inlineStr"/>
-      <c r="E716" t="inlineStr"/>
-      <c r="F716" t="inlineStr"/>
       <c r="G716" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16553,9 +16550,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D717" t="inlineStr"/>
-      <c r="E717" t="inlineStr"/>
-      <c r="F717" t="inlineStr"/>
       <c r="G717" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16578,9 +16572,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D718" t="inlineStr"/>
-      <c r="E718" t="inlineStr"/>
-      <c r="F718" t="inlineStr"/>
       <c r="G718" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16603,9 +16594,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D719" t="inlineStr"/>
-      <c r="E719" t="inlineStr"/>
-      <c r="F719" t="inlineStr"/>
       <c r="G719" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16628,9 +16616,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D720" t="inlineStr"/>
-      <c r="E720" t="inlineStr"/>
-      <c r="F720" t="inlineStr"/>
       <c r="G720" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16653,9 +16638,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D721" t="inlineStr"/>
-      <c r="E721" t="inlineStr"/>
-      <c r="F721" t="inlineStr"/>
       <c r="G721" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16678,9 +16660,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D722" t="inlineStr"/>
-      <c r="E722" t="inlineStr"/>
-      <c r="F722" t="inlineStr"/>
       <c r="G722" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16703,9 +16682,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D723" t="inlineStr"/>
-      <c r="E723" t="inlineStr"/>
-      <c r="F723" t="inlineStr"/>
       <c r="G723" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16728,9 +16704,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D724" t="inlineStr"/>
-      <c r="E724" t="inlineStr"/>
-      <c r="F724" t="inlineStr"/>
       <c r="G724" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16753,9 +16726,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D725" t="inlineStr"/>
-      <c r="E725" t="inlineStr"/>
-      <c r="F725" t="inlineStr"/>
       <c r="G725" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16778,9 +16748,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D726" t="inlineStr"/>
-      <c r="E726" t="inlineStr"/>
-      <c r="F726" t="inlineStr"/>
       <c r="G726" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16803,9 +16770,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D727" t="inlineStr"/>
-      <c r="E727" t="inlineStr"/>
-      <c r="F727" t="inlineStr"/>
       <c r="G727" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16828,9 +16792,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D728" t="inlineStr"/>
-      <c r="E728" t="inlineStr"/>
-      <c r="F728" t="inlineStr"/>
       <c r="G728" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16853,9 +16814,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D729" t="inlineStr"/>
-      <c r="E729" t="inlineStr"/>
-      <c r="F729" t="inlineStr"/>
       <c r="G729" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16878,10 +16836,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D730" t="inlineStr"/>
-      <c r="E730" t="inlineStr"/>
-      <c r="F730" t="inlineStr"/>
       <c r="G730" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C731" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D731" t="inlineStr"/>
+      <c r="E731" t="inlineStr"/>
+      <c r="F731" t="inlineStr"/>
+      <c r="G731" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C732" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D732" t="inlineStr"/>
+      <c r="E732" t="inlineStr"/>
+      <c r="F732" t="inlineStr"/>
+      <c r="G732" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D733" t="inlineStr"/>
+      <c r="E733" t="inlineStr"/>
+      <c r="F733" t="inlineStr"/>
+      <c r="G733" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D734" t="inlineStr"/>
+      <c r="E734" t="inlineStr"/>
+      <c r="F734" t="inlineStr"/>
+      <c r="G734" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D735" t="inlineStr"/>
+      <c r="E735" t="inlineStr"/>
+      <c r="F735" t="inlineStr"/>
+      <c r="G735" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C736" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D736" t="inlineStr"/>
+      <c r="E736" t="inlineStr"/>
+      <c r="F736" t="inlineStr"/>
+      <c r="G736" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D737" t="inlineStr"/>
+      <c r="E737" t="inlineStr"/>
+      <c r="F737" t="inlineStr"/>
+      <c r="G737" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C738" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D738" t="inlineStr"/>
+      <c r="E738" t="inlineStr"/>
+      <c r="F738" t="inlineStr"/>
+      <c r="G738" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B739" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C739" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D739" t="inlineStr"/>
+      <c r="E739" t="inlineStr"/>
+      <c r="F739" t="inlineStr"/>
+      <c r="G739" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C740" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D740" t="inlineStr"/>
+      <c r="E740" t="inlineStr"/>
+      <c r="F740" t="inlineStr"/>
+      <c r="G740" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B741" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C741" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D741" t="inlineStr"/>
+      <c r="E741" t="inlineStr"/>
+      <c r="F741" t="inlineStr"/>
+      <c r="G741" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C742" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D742" t="inlineStr"/>
+      <c r="E742" t="inlineStr"/>
+      <c r="F742" t="inlineStr"/>
+      <c r="G742" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C743" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D743" t="inlineStr"/>
+      <c r="E743" t="inlineStr"/>
+      <c r="F743" t="inlineStr"/>
+      <c r="G743" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B744" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C744" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D744" t="inlineStr"/>
+      <c r="E744" t="inlineStr"/>
+      <c r="F744" t="inlineStr"/>
+      <c r="G744" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C745" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D745" t="inlineStr"/>
+      <c r="E745" t="inlineStr"/>
+      <c r="F745" t="inlineStr"/>
+      <c r="G745" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-10-04
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G745"/>
+  <dimension ref="A1:G760"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16858,9 +16858,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D731" t="inlineStr"/>
-      <c r="E731" t="inlineStr"/>
-      <c r="F731" t="inlineStr"/>
       <c r="G731" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16883,9 +16880,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D732" t="inlineStr"/>
-      <c r="E732" t="inlineStr"/>
-      <c r="F732" t="inlineStr"/>
       <c r="G732" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16908,9 +16902,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D733" t="inlineStr"/>
-      <c r="E733" t="inlineStr"/>
-      <c r="F733" t="inlineStr"/>
       <c r="G733" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16933,9 +16924,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D734" t="inlineStr"/>
-      <c r="E734" t="inlineStr"/>
-      <c r="F734" t="inlineStr"/>
       <c r="G734" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16958,9 +16946,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D735" t="inlineStr"/>
-      <c r="E735" t="inlineStr"/>
-      <c r="F735" t="inlineStr"/>
       <c r="G735" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -16983,9 +16968,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D736" t="inlineStr"/>
-      <c r="E736" t="inlineStr"/>
-      <c r="F736" t="inlineStr"/>
       <c r="G736" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17008,9 +16990,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D737" t="inlineStr"/>
-      <c r="E737" t="inlineStr"/>
-      <c r="F737" t="inlineStr"/>
       <c r="G737" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17033,9 +17012,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D738" t="inlineStr"/>
-      <c r="E738" t="inlineStr"/>
-      <c r="F738" t="inlineStr"/>
       <c r="G738" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17058,9 +17034,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D739" t="inlineStr"/>
-      <c r="E739" t="inlineStr"/>
-      <c r="F739" t="inlineStr"/>
       <c r="G739" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17083,9 +17056,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D740" t="inlineStr"/>
-      <c r="E740" t="inlineStr"/>
-      <c r="F740" t="inlineStr"/>
       <c r="G740" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17108,9 +17078,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D741" t="inlineStr"/>
-      <c r="E741" t="inlineStr"/>
-      <c r="F741" t="inlineStr"/>
       <c r="G741" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17133,9 +17100,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D742" t="inlineStr"/>
-      <c r="E742" t="inlineStr"/>
-      <c r="F742" t="inlineStr"/>
       <c r="G742" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17158,9 +17122,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D743" t="inlineStr"/>
-      <c r="E743" t="inlineStr"/>
-      <c r="F743" t="inlineStr"/>
       <c r="G743" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17183,9 +17144,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D744" t="inlineStr"/>
-      <c r="E744" t="inlineStr"/>
-      <c r="F744" t="inlineStr"/>
       <c r="G744" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17208,10 +17166,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D745" t="inlineStr"/>
-      <c r="E745" t="inlineStr"/>
-      <c r="F745" t="inlineStr"/>
       <c r="G745" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B746" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C746" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D746" t="inlineStr"/>
+      <c r="E746" t="inlineStr"/>
+      <c r="F746" t="inlineStr"/>
+      <c r="G746" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C747" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D747" t="inlineStr"/>
+      <c r="E747" t="inlineStr"/>
+      <c r="F747" t="inlineStr"/>
+      <c r="G747" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D748" t="inlineStr"/>
+      <c r="E748" t="inlineStr"/>
+      <c r="F748" t="inlineStr"/>
+      <c r="G748" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C749" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D749" t="inlineStr"/>
+      <c r="E749" t="inlineStr"/>
+      <c r="F749" t="inlineStr"/>
+      <c r="G749" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B750" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C750" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D750" t="inlineStr"/>
+      <c r="E750" t="inlineStr"/>
+      <c r="F750" t="inlineStr"/>
+      <c r="G750" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B751" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C751" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D751" t="inlineStr"/>
+      <c r="E751" t="inlineStr"/>
+      <c r="F751" t="inlineStr"/>
+      <c r="G751" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D752" t="inlineStr"/>
+      <c r="E752" t="inlineStr"/>
+      <c r="F752" t="inlineStr"/>
+      <c r="G752" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B753" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C753" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D753" t="inlineStr"/>
+      <c r="E753" t="inlineStr"/>
+      <c r="F753" t="inlineStr"/>
+      <c r="G753" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C754" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D754" t="inlineStr"/>
+      <c r="E754" t="inlineStr"/>
+      <c r="F754" t="inlineStr"/>
+      <c r="G754" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C755" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D755" t="inlineStr"/>
+      <c r="E755" t="inlineStr"/>
+      <c r="F755" t="inlineStr"/>
+      <c r="G755" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B756" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C756" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D756" t="inlineStr"/>
+      <c r="E756" t="inlineStr"/>
+      <c r="F756" t="inlineStr"/>
+      <c r="G756" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B757" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C757" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D757" t="inlineStr"/>
+      <c r="E757" t="inlineStr"/>
+      <c r="F757" t="inlineStr"/>
+      <c r="G757" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B758" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C758" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D758" t="inlineStr"/>
+      <c r="E758" t="inlineStr"/>
+      <c r="F758" t="inlineStr"/>
+      <c r="G758" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B759" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C759" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D759" t="inlineStr"/>
+      <c r="E759" t="inlineStr"/>
+      <c r="F759" t="inlineStr"/>
+      <c r="G759" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B760" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C760" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D760" t="inlineStr"/>
+      <c r="E760" t="inlineStr"/>
+      <c r="F760" t="inlineStr"/>
+      <c r="G760" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-10-06
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G760"/>
+  <dimension ref="A1:G775"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17188,9 +17188,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D746" t="inlineStr"/>
-      <c r="E746" t="inlineStr"/>
-      <c r="F746" t="inlineStr"/>
       <c r="G746" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17213,9 +17210,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D747" t="inlineStr"/>
-      <c r="E747" t="inlineStr"/>
-      <c r="F747" t="inlineStr"/>
       <c r="G747" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17238,9 +17232,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D748" t="inlineStr"/>
-      <c r="E748" t="inlineStr"/>
-      <c r="F748" t="inlineStr"/>
       <c r="G748" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17263,9 +17254,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D749" t="inlineStr"/>
-      <c r="E749" t="inlineStr"/>
-      <c r="F749" t="inlineStr"/>
       <c r="G749" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17288,9 +17276,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D750" t="inlineStr"/>
-      <c r="E750" t="inlineStr"/>
-      <c r="F750" t="inlineStr"/>
       <c r="G750" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17313,9 +17298,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D751" t="inlineStr"/>
-      <c r="E751" t="inlineStr"/>
-      <c r="F751" t="inlineStr"/>
       <c r="G751" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17338,9 +17320,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D752" t="inlineStr"/>
-      <c r="E752" t="inlineStr"/>
-      <c r="F752" t="inlineStr"/>
       <c r="G752" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17363,9 +17342,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D753" t="inlineStr"/>
-      <c r="E753" t="inlineStr"/>
-      <c r="F753" t="inlineStr"/>
       <c r="G753" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17388,9 +17364,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D754" t="inlineStr"/>
-      <c r="E754" t="inlineStr"/>
-      <c r="F754" t="inlineStr"/>
       <c r="G754" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17413,9 +17386,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D755" t="inlineStr"/>
-      <c r="E755" t="inlineStr"/>
-      <c r="F755" t="inlineStr"/>
       <c r="G755" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17438,9 +17408,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D756" t="inlineStr"/>
-      <c r="E756" t="inlineStr"/>
-      <c r="F756" t="inlineStr"/>
       <c r="G756" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17463,9 +17430,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D757" t="inlineStr"/>
-      <c r="E757" t="inlineStr"/>
-      <c r="F757" t="inlineStr"/>
       <c r="G757" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17488,9 +17452,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D758" t="inlineStr"/>
-      <c r="E758" t="inlineStr"/>
-      <c r="F758" t="inlineStr"/>
       <c r="G758" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17513,9 +17474,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D759" t="inlineStr"/>
-      <c r="E759" t="inlineStr"/>
-      <c r="F759" t="inlineStr"/>
       <c r="G759" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17538,10 +17496,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D760" t="inlineStr"/>
-      <c r="E760" t="inlineStr"/>
-      <c r="F760" t="inlineStr"/>
       <c r="G760" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B761" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C761" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D761" t="inlineStr"/>
+      <c r="E761" t="inlineStr"/>
+      <c r="F761" t="inlineStr"/>
+      <c r="G761" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B762" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C762" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D762" t="inlineStr"/>
+      <c r="E762" t="inlineStr"/>
+      <c r="F762" t="inlineStr"/>
+      <c r="G762" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B763" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C763" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D763" t="inlineStr"/>
+      <c r="E763" t="inlineStr"/>
+      <c r="F763" t="inlineStr"/>
+      <c r="G763" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B764" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C764" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D764" t="inlineStr"/>
+      <c r="E764" t="inlineStr"/>
+      <c r="F764" t="inlineStr"/>
+      <c r="G764" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B765" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C765" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D765" t="inlineStr"/>
+      <c r="E765" t="inlineStr"/>
+      <c r="F765" t="inlineStr"/>
+      <c r="G765" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B766" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C766" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D766" t="inlineStr"/>
+      <c r="E766" t="inlineStr"/>
+      <c r="F766" t="inlineStr"/>
+      <c r="G766" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B767" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C767" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D767" t="inlineStr"/>
+      <c r="E767" t="inlineStr"/>
+      <c r="F767" t="inlineStr"/>
+      <c r="G767" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B768" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C768" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D768" t="inlineStr"/>
+      <c r="E768" t="inlineStr"/>
+      <c r="F768" t="inlineStr"/>
+      <c r="G768" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B769" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C769" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D769" t="inlineStr"/>
+      <c r="E769" t="inlineStr"/>
+      <c r="F769" t="inlineStr"/>
+      <c r="G769" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B770" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C770" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D770" t="inlineStr"/>
+      <c r="E770" t="inlineStr"/>
+      <c r="F770" t="inlineStr"/>
+      <c r="G770" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B771" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C771" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D771" t="inlineStr"/>
+      <c r="E771" t="inlineStr"/>
+      <c r="F771" t="inlineStr"/>
+      <c r="G771" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B772" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C772" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D772" t="inlineStr"/>
+      <c r="E772" t="inlineStr"/>
+      <c r="F772" t="inlineStr"/>
+      <c r="G772" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B773" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C773" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D773" t="inlineStr"/>
+      <c r="E773" t="inlineStr"/>
+      <c r="F773" t="inlineStr"/>
+      <c r="G773" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B774" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C774" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D774" t="inlineStr"/>
+      <c r="E774" t="inlineStr"/>
+      <c r="F774" t="inlineStr"/>
+      <c r="G774" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B775" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C775" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D775" t="inlineStr"/>
+      <c r="E775" t="inlineStr"/>
+      <c r="F775" t="inlineStr"/>
+      <c r="G775" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-10-07
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G775"/>
+  <dimension ref="A1:G790"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17518,9 +17518,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D761" t="inlineStr"/>
-      <c r="E761" t="inlineStr"/>
-      <c r="F761" t="inlineStr"/>
       <c r="G761" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17543,9 +17540,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D762" t="inlineStr"/>
-      <c r="E762" t="inlineStr"/>
-      <c r="F762" t="inlineStr"/>
       <c r="G762" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17568,9 +17562,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D763" t="inlineStr"/>
-      <c r="E763" t="inlineStr"/>
-      <c r="F763" t="inlineStr"/>
       <c r="G763" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17593,9 +17584,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D764" t="inlineStr"/>
-      <c r="E764" t="inlineStr"/>
-      <c r="F764" t="inlineStr"/>
       <c r="G764" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17618,9 +17606,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D765" t="inlineStr"/>
-      <c r="E765" t="inlineStr"/>
-      <c r="F765" t="inlineStr"/>
       <c r="G765" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17643,9 +17628,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D766" t="inlineStr"/>
-      <c r="E766" t="inlineStr"/>
-      <c r="F766" t="inlineStr"/>
       <c r="G766" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17668,9 +17650,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D767" t="inlineStr"/>
-      <c r="E767" t="inlineStr"/>
-      <c r="F767" t="inlineStr"/>
       <c r="G767" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17693,9 +17672,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D768" t="inlineStr"/>
-      <c r="E768" t="inlineStr"/>
-      <c r="F768" t="inlineStr"/>
       <c r="G768" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17718,9 +17694,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D769" t="inlineStr"/>
-      <c r="E769" t="inlineStr"/>
-      <c r="F769" t="inlineStr"/>
       <c r="G769" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17743,9 +17716,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D770" t="inlineStr"/>
-      <c r="E770" t="inlineStr"/>
-      <c r="F770" t="inlineStr"/>
       <c r="G770" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17768,9 +17738,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D771" t="inlineStr"/>
-      <c r="E771" t="inlineStr"/>
-      <c r="F771" t="inlineStr"/>
       <c r="G771" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17793,9 +17760,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D772" t="inlineStr"/>
-      <c r="E772" t="inlineStr"/>
-      <c r="F772" t="inlineStr"/>
       <c r="G772" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17818,9 +17782,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D773" t="inlineStr"/>
-      <c r="E773" t="inlineStr"/>
-      <c r="F773" t="inlineStr"/>
       <c r="G773" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17843,9 +17804,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D774" t="inlineStr"/>
-      <c r="E774" t="inlineStr"/>
-      <c r="F774" t="inlineStr"/>
       <c r="G774" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17868,10 +17826,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D775" t="inlineStr"/>
-      <c r="E775" t="inlineStr"/>
-      <c r="F775" t="inlineStr"/>
       <c r="G775" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B776" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C776" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D776" t="inlineStr"/>
+      <c r="E776" t="inlineStr"/>
+      <c r="F776" t="inlineStr"/>
+      <c r="G776" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B777" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C777" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D777" t="inlineStr"/>
+      <c r="E777" t="inlineStr"/>
+      <c r="F777" t="inlineStr"/>
+      <c r="G777" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B778" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C778" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D778" t="inlineStr"/>
+      <c r="E778" t="inlineStr"/>
+      <c r="F778" t="inlineStr"/>
+      <c r="G778" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B779" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C779" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D779" t="inlineStr"/>
+      <c r="E779" t="inlineStr"/>
+      <c r="F779" t="inlineStr"/>
+      <c r="G779" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B780" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C780" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D780" t="inlineStr"/>
+      <c r="E780" t="inlineStr"/>
+      <c r="F780" t="inlineStr"/>
+      <c r="G780" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B781" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C781" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D781" t="inlineStr"/>
+      <c r="E781" t="inlineStr"/>
+      <c r="F781" t="inlineStr"/>
+      <c r="G781" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B782" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C782" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D782" t="inlineStr"/>
+      <c r="E782" t="inlineStr"/>
+      <c r="F782" t="inlineStr"/>
+      <c r="G782" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B783" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C783" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D783" t="inlineStr"/>
+      <c r="E783" t="inlineStr"/>
+      <c r="F783" t="inlineStr"/>
+      <c r="G783" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B784" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C784" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D784" t="inlineStr"/>
+      <c r="E784" t="inlineStr"/>
+      <c r="F784" t="inlineStr"/>
+      <c r="G784" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B785" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C785" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D785" t="inlineStr"/>
+      <c r="E785" t="inlineStr"/>
+      <c r="F785" t="inlineStr"/>
+      <c r="G785" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B786" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C786" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D786" t="inlineStr"/>
+      <c r="E786" t="inlineStr"/>
+      <c r="F786" t="inlineStr"/>
+      <c r="G786" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B787" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C787" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D787" t="inlineStr"/>
+      <c r="E787" t="inlineStr"/>
+      <c r="F787" t="inlineStr"/>
+      <c r="G787" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B788" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C788" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D788" t="inlineStr"/>
+      <c r="E788" t="inlineStr"/>
+      <c r="F788" t="inlineStr"/>
+      <c r="G788" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B789" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C789" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D789" t="inlineStr"/>
+      <c r="E789" t="inlineStr"/>
+      <c r="F789" t="inlineStr"/>
+      <c r="G789" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B790" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C790" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D790" t="inlineStr"/>
+      <c r="E790" t="inlineStr"/>
+      <c r="F790" t="inlineStr"/>
+      <c r="G790" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-10-08
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G790"/>
+  <dimension ref="A1:G805"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17848,9 +17848,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D776" t="inlineStr"/>
-      <c r="E776" t="inlineStr"/>
-      <c r="F776" t="inlineStr"/>
       <c r="G776" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17873,9 +17870,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D777" t="inlineStr"/>
-      <c r="E777" t="inlineStr"/>
-      <c r="F777" t="inlineStr"/>
       <c r="G777" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17898,9 +17892,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D778" t="inlineStr"/>
-      <c r="E778" t="inlineStr"/>
-      <c r="F778" t="inlineStr"/>
       <c r="G778" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17923,9 +17914,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D779" t="inlineStr"/>
-      <c r="E779" t="inlineStr"/>
-      <c r="F779" t="inlineStr"/>
       <c r="G779" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17948,9 +17936,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D780" t="inlineStr"/>
-      <c r="E780" t="inlineStr"/>
-      <c r="F780" t="inlineStr"/>
       <c r="G780" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17973,9 +17958,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D781" t="inlineStr"/>
-      <c r="E781" t="inlineStr"/>
-      <c r="F781" t="inlineStr"/>
       <c r="G781" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -17998,9 +17980,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D782" t="inlineStr"/>
-      <c r="E782" t="inlineStr"/>
-      <c r="F782" t="inlineStr"/>
       <c r="G782" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18023,9 +18002,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D783" t="inlineStr"/>
-      <c r="E783" t="inlineStr"/>
-      <c r="F783" t="inlineStr"/>
       <c r="G783" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18048,9 +18024,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D784" t="inlineStr"/>
-      <c r="E784" t="inlineStr"/>
-      <c r="F784" t="inlineStr"/>
       <c r="G784" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18073,9 +18046,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D785" t="inlineStr"/>
-      <c r="E785" t="inlineStr"/>
-      <c r="F785" t="inlineStr"/>
       <c r="G785" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18098,9 +18068,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D786" t="inlineStr"/>
-      <c r="E786" t="inlineStr"/>
-      <c r="F786" t="inlineStr"/>
       <c r="G786" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18123,9 +18090,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D787" t="inlineStr"/>
-      <c r="E787" t="inlineStr"/>
-      <c r="F787" t="inlineStr"/>
       <c r="G787" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18148,9 +18112,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D788" t="inlineStr"/>
-      <c r="E788" t="inlineStr"/>
-      <c r="F788" t="inlineStr"/>
       <c r="G788" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18173,9 +18134,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D789" t="inlineStr"/>
-      <c r="E789" t="inlineStr"/>
-      <c r="F789" t="inlineStr"/>
       <c r="G789" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18198,10 +18156,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D790" t="inlineStr"/>
-      <c r="E790" t="inlineStr"/>
-      <c r="F790" t="inlineStr"/>
       <c r="G790" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B791" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C791" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D791" t="inlineStr"/>
+      <c r="E791" t="inlineStr"/>
+      <c r="F791" t="inlineStr"/>
+      <c r="G791" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B792" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C792" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D792" t="inlineStr"/>
+      <c r="E792" t="inlineStr"/>
+      <c r="F792" t="inlineStr"/>
+      <c r="G792" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B793" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C793" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D793" t="inlineStr"/>
+      <c r="E793" t="inlineStr"/>
+      <c r="F793" t="inlineStr"/>
+      <c r="G793" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B794" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C794" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D794" t="inlineStr"/>
+      <c r="E794" t="inlineStr"/>
+      <c r="F794" t="inlineStr"/>
+      <c r="G794" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B795" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C795" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D795" t="inlineStr"/>
+      <c r="E795" t="inlineStr"/>
+      <c r="F795" t="inlineStr"/>
+      <c r="G795" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B796" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C796" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D796" t="inlineStr"/>
+      <c r="E796" t="inlineStr"/>
+      <c r="F796" t="inlineStr"/>
+      <c r="G796" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B797" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C797" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D797" t="inlineStr"/>
+      <c r="E797" t="inlineStr"/>
+      <c r="F797" t="inlineStr"/>
+      <c r="G797" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B798" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C798" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D798" t="inlineStr"/>
+      <c r="E798" t="inlineStr"/>
+      <c r="F798" t="inlineStr"/>
+      <c r="G798" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B799" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C799" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D799" t="inlineStr"/>
+      <c r="E799" t="inlineStr"/>
+      <c r="F799" t="inlineStr"/>
+      <c r="G799" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B800" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C800" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D800" t="inlineStr"/>
+      <c r="E800" t="inlineStr"/>
+      <c r="F800" t="inlineStr"/>
+      <c r="G800" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B801" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C801" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D801" t="inlineStr"/>
+      <c r="E801" t="inlineStr"/>
+      <c r="F801" t="inlineStr"/>
+      <c r="G801" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B802" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C802" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D802" t="inlineStr"/>
+      <c r="E802" t="inlineStr"/>
+      <c r="F802" t="inlineStr"/>
+      <c r="G802" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B803" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C803" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D803" t="inlineStr"/>
+      <c r="E803" t="inlineStr"/>
+      <c r="F803" t="inlineStr"/>
+      <c r="G803" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B804" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C804" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D804" t="inlineStr"/>
+      <c r="E804" t="inlineStr"/>
+      <c r="F804" t="inlineStr"/>
+      <c r="G804" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B805" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C805" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D805" t="inlineStr"/>
+      <c r="E805" t="inlineStr"/>
+      <c r="F805" t="inlineStr"/>
+      <c r="G805" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-10-09
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G805"/>
+  <dimension ref="A1:G820"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18178,9 +18178,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D791" t="inlineStr"/>
-      <c r="E791" t="inlineStr"/>
-      <c r="F791" t="inlineStr"/>
       <c r="G791" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18203,9 +18200,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D792" t="inlineStr"/>
-      <c r="E792" t="inlineStr"/>
-      <c r="F792" t="inlineStr"/>
       <c r="G792" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18228,9 +18222,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D793" t="inlineStr"/>
-      <c r="E793" t="inlineStr"/>
-      <c r="F793" t="inlineStr"/>
       <c r="G793" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18253,9 +18244,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D794" t="inlineStr"/>
-      <c r="E794" t="inlineStr"/>
-      <c r="F794" t="inlineStr"/>
       <c r="G794" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18278,9 +18266,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D795" t="inlineStr"/>
-      <c r="E795" t="inlineStr"/>
-      <c r="F795" t="inlineStr"/>
       <c r="G795" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18303,9 +18288,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D796" t="inlineStr"/>
-      <c r="E796" t="inlineStr"/>
-      <c r="F796" t="inlineStr"/>
       <c r="G796" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18328,9 +18310,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D797" t="inlineStr"/>
-      <c r="E797" t="inlineStr"/>
-      <c r="F797" t="inlineStr"/>
       <c r="G797" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18353,9 +18332,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D798" t="inlineStr"/>
-      <c r="E798" t="inlineStr"/>
-      <c r="F798" t="inlineStr"/>
       <c r="G798" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18378,9 +18354,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D799" t="inlineStr"/>
-      <c r="E799" t="inlineStr"/>
-      <c r="F799" t="inlineStr"/>
       <c r="G799" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18403,9 +18376,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D800" t="inlineStr"/>
-      <c r="E800" t="inlineStr"/>
-      <c r="F800" t="inlineStr"/>
       <c r="G800" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18428,9 +18398,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D801" t="inlineStr"/>
-      <c r="E801" t="inlineStr"/>
-      <c r="F801" t="inlineStr"/>
       <c r="G801" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18453,9 +18420,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D802" t="inlineStr"/>
-      <c r="E802" t="inlineStr"/>
-      <c r="F802" t="inlineStr"/>
       <c r="G802" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18478,9 +18442,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D803" t="inlineStr"/>
-      <c r="E803" t="inlineStr"/>
-      <c r="F803" t="inlineStr"/>
       <c r="G803" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18503,9 +18464,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D804" t="inlineStr"/>
-      <c r="E804" t="inlineStr"/>
-      <c r="F804" t="inlineStr"/>
       <c r="G804" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18528,10 +18486,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D805" t="inlineStr"/>
-      <c r="E805" t="inlineStr"/>
-      <c r="F805" t="inlineStr"/>
       <c r="G805" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B806" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C806" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D806" t="inlineStr"/>
+      <c r="E806" t="inlineStr"/>
+      <c r="F806" t="inlineStr"/>
+      <c r="G806" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B807" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C807" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D807" t="inlineStr"/>
+      <c r="E807" t="inlineStr"/>
+      <c r="F807" t="inlineStr"/>
+      <c r="G807" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B808" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C808" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D808" t="inlineStr"/>
+      <c r="E808" t="inlineStr"/>
+      <c r="F808" t="inlineStr"/>
+      <c r="G808" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B809" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C809" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D809" t="inlineStr"/>
+      <c r="E809" t="inlineStr"/>
+      <c r="F809" t="inlineStr"/>
+      <c r="G809" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B810" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C810" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D810" t="inlineStr"/>
+      <c r="E810" t="inlineStr"/>
+      <c r="F810" t="inlineStr"/>
+      <c r="G810" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B811" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C811" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D811" t="inlineStr"/>
+      <c r="E811" t="inlineStr"/>
+      <c r="F811" t="inlineStr"/>
+      <c r="G811" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B812" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C812" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D812" t="inlineStr"/>
+      <c r="E812" t="inlineStr"/>
+      <c r="F812" t="inlineStr"/>
+      <c r="G812" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B813" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C813" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D813" t="inlineStr"/>
+      <c r="E813" t="inlineStr"/>
+      <c r="F813" t="inlineStr"/>
+      <c r="G813" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B814" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C814" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D814" t="inlineStr"/>
+      <c r="E814" t="inlineStr"/>
+      <c r="F814" t="inlineStr"/>
+      <c r="G814" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B815" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C815" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D815" t="inlineStr"/>
+      <c r="E815" t="inlineStr"/>
+      <c r="F815" t="inlineStr"/>
+      <c r="G815" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B816" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C816" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D816" t="inlineStr"/>
+      <c r="E816" t="inlineStr"/>
+      <c r="F816" t="inlineStr"/>
+      <c r="G816" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B817" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C817" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D817" t="inlineStr"/>
+      <c r="E817" t="inlineStr"/>
+      <c r="F817" t="inlineStr"/>
+      <c r="G817" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B818" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C818" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D818" t="inlineStr"/>
+      <c r="E818" t="inlineStr"/>
+      <c r="F818" t="inlineStr"/>
+      <c r="G818" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B819" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C819" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D819" t="inlineStr"/>
+      <c r="E819" t="inlineStr"/>
+      <c r="F819" t="inlineStr"/>
+      <c r="G819" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B820" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C820" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D820" t="inlineStr"/>
+      <c r="E820" t="inlineStr"/>
+      <c r="F820" t="inlineStr"/>
+      <c r="G820" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-10-10
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G820"/>
+  <dimension ref="A1:G835"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18508,9 +18508,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D806" t="inlineStr"/>
-      <c r="E806" t="inlineStr"/>
-      <c r="F806" t="inlineStr"/>
       <c r="G806" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18533,9 +18530,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D807" t="inlineStr"/>
-      <c r="E807" t="inlineStr"/>
-      <c r="F807" t="inlineStr"/>
       <c r="G807" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18558,9 +18552,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D808" t="inlineStr"/>
-      <c r="E808" t="inlineStr"/>
-      <c r="F808" t="inlineStr"/>
       <c r="G808" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18583,9 +18574,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D809" t="inlineStr"/>
-      <c r="E809" t="inlineStr"/>
-      <c r="F809" t="inlineStr"/>
       <c r="G809" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18608,9 +18596,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D810" t="inlineStr"/>
-      <c r="E810" t="inlineStr"/>
-      <c r="F810" t="inlineStr"/>
       <c r="G810" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18633,9 +18618,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D811" t="inlineStr"/>
-      <c r="E811" t="inlineStr"/>
-      <c r="F811" t="inlineStr"/>
       <c r="G811" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18658,9 +18640,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D812" t="inlineStr"/>
-      <c r="E812" t="inlineStr"/>
-      <c r="F812" t="inlineStr"/>
       <c r="G812" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18683,9 +18662,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D813" t="inlineStr"/>
-      <c r="E813" t="inlineStr"/>
-      <c r="F813" t="inlineStr"/>
       <c r="G813" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18708,9 +18684,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D814" t="inlineStr"/>
-      <c r="E814" t="inlineStr"/>
-      <c r="F814" t="inlineStr"/>
       <c r="G814" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18733,9 +18706,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D815" t="inlineStr"/>
-      <c r="E815" t="inlineStr"/>
-      <c r="F815" t="inlineStr"/>
       <c r="G815" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18758,9 +18728,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D816" t="inlineStr"/>
-      <c r="E816" t="inlineStr"/>
-      <c r="F816" t="inlineStr"/>
       <c r="G816" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18783,9 +18750,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D817" t="inlineStr"/>
-      <c r="E817" t="inlineStr"/>
-      <c r="F817" t="inlineStr"/>
       <c r="G817" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18808,9 +18772,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D818" t="inlineStr"/>
-      <c r="E818" t="inlineStr"/>
-      <c r="F818" t="inlineStr"/>
       <c r="G818" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18833,9 +18794,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D819" t="inlineStr"/>
-      <c r="E819" t="inlineStr"/>
-      <c r="F819" t="inlineStr"/>
       <c r="G819" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18858,10 +18816,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D820" t="inlineStr"/>
-      <c r="E820" t="inlineStr"/>
-      <c r="F820" t="inlineStr"/>
       <c r="G820" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B821" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C821" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D821" t="inlineStr"/>
+      <c r="E821" t="inlineStr"/>
+      <c r="F821" t="inlineStr"/>
+      <c r="G821" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B822" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C822" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D822" t="inlineStr"/>
+      <c r="E822" t="inlineStr"/>
+      <c r="F822" t="inlineStr"/>
+      <c r="G822" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B823" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C823" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D823" t="inlineStr"/>
+      <c r="E823" t="inlineStr"/>
+      <c r="F823" t="inlineStr"/>
+      <c r="G823" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B824" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C824" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D824" t="inlineStr"/>
+      <c r="E824" t="inlineStr"/>
+      <c r="F824" t="inlineStr"/>
+      <c r="G824" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B825" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C825" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D825" t="inlineStr"/>
+      <c r="E825" t="inlineStr"/>
+      <c r="F825" t="inlineStr"/>
+      <c r="G825" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B826" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C826" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D826" t="inlineStr"/>
+      <c r="E826" t="inlineStr"/>
+      <c r="F826" t="inlineStr"/>
+      <c r="G826" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B827" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C827" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D827" t="inlineStr"/>
+      <c r="E827" t="inlineStr"/>
+      <c r="F827" t="inlineStr"/>
+      <c r="G827" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B828" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C828" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D828" t="inlineStr"/>
+      <c r="E828" t="inlineStr"/>
+      <c r="F828" t="inlineStr"/>
+      <c r="G828" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B829" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C829" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D829" t="inlineStr"/>
+      <c r="E829" t="inlineStr"/>
+      <c r="F829" t="inlineStr"/>
+      <c r="G829" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B830" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C830" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D830" t="inlineStr"/>
+      <c r="E830" t="inlineStr"/>
+      <c r="F830" t="inlineStr"/>
+      <c r="G830" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B831" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C831" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D831" t="inlineStr"/>
+      <c r="E831" t="inlineStr"/>
+      <c r="F831" t="inlineStr"/>
+      <c r="G831" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B832" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C832" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D832" t="inlineStr"/>
+      <c r="E832" t="inlineStr"/>
+      <c r="F832" t="inlineStr"/>
+      <c r="G832" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B833" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C833" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D833" t="inlineStr"/>
+      <c r="E833" t="inlineStr"/>
+      <c r="F833" t="inlineStr"/>
+      <c r="G833" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B834" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C834" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D834" t="inlineStr"/>
+      <c r="E834" t="inlineStr"/>
+      <c r="F834" t="inlineStr"/>
+      <c r="G834" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B835" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C835" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D835" t="inlineStr"/>
+      <c r="E835" t="inlineStr"/>
+      <c r="F835" t="inlineStr"/>
+      <c r="G835" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-10-11
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G835"/>
+  <dimension ref="A1:G850"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18838,9 +18838,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D821" t="inlineStr"/>
-      <c r="E821" t="inlineStr"/>
-      <c r="F821" t="inlineStr"/>
       <c r="G821" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18863,9 +18860,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D822" t="inlineStr"/>
-      <c r="E822" t="inlineStr"/>
-      <c r="F822" t="inlineStr"/>
       <c r="G822" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18888,9 +18882,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D823" t="inlineStr"/>
-      <c r="E823" t="inlineStr"/>
-      <c r="F823" t="inlineStr"/>
       <c r="G823" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18913,9 +18904,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D824" t="inlineStr"/>
-      <c r="E824" t="inlineStr"/>
-      <c r="F824" t="inlineStr"/>
       <c r="G824" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18938,9 +18926,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D825" t="inlineStr"/>
-      <c r="E825" t="inlineStr"/>
-      <c r="F825" t="inlineStr"/>
       <c r="G825" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18963,9 +18948,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D826" t="inlineStr"/>
-      <c r="E826" t="inlineStr"/>
-      <c r="F826" t="inlineStr"/>
       <c r="G826" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -18988,9 +18970,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D827" t="inlineStr"/>
-      <c r="E827" t="inlineStr"/>
-      <c r="F827" t="inlineStr"/>
       <c r="G827" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19013,9 +18992,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D828" t="inlineStr"/>
-      <c r="E828" t="inlineStr"/>
-      <c r="F828" t="inlineStr"/>
       <c r="G828" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19038,9 +19014,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D829" t="inlineStr"/>
-      <c r="E829" t="inlineStr"/>
-      <c r="F829" t="inlineStr"/>
       <c r="G829" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19063,9 +19036,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D830" t="inlineStr"/>
-      <c r="E830" t="inlineStr"/>
-      <c r="F830" t="inlineStr"/>
       <c r="G830" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19088,9 +19058,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D831" t="inlineStr"/>
-      <c r="E831" t="inlineStr"/>
-      <c r="F831" t="inlineStr"/>
       <c r="G831" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19113,9 +19080,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D832" t="inlineStr"/>
-      <c r="E832" t="inlineStr"/>
-      <c r="F832" t="inlineStr"/>
       <c r="G832" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19138,9 +19102,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D833" t="inlineStr"/>
-      <c r="E833" t="inlineStr"/>
-      <c r="F833" t="inlineStr"/>
       <c r="G833" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19163,9 +19124,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D834" t="inlineStr"/>
-      <c r="E834" t="inlineStr"/>
-      <c r="F834" t="inlineStr"/>
       <c r="G834" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19188,10 +19146,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D835" t="inlineStr"/>
-      <c r="E835" t="inlineStr"/>
-      <c r="F835" t="inlineStr"/>
       <c r="G835" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B836" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C836" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D836" t="inlineStr"/>
+      <c r="E836" t="inlineStr"/>
+      <c r="F836" t="inlineStr"/>
+      <c r="G836" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B837" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C837" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D837" t="inlineStr"/>
+      <c r="E837" t="inlineStr"/>
+      <c r="F837" t="inlineStr"/>
+      <c r="G837" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B838" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C838" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D838" t="inlineStr"/>
+      <c r="E838" t="inlineStr"/>
+      <c r="F838" t="inlineStr"/>
+      <c r="G838" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B839" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C839" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D839" t="inlineStr"/>
+      <c r="E839" t="inlineStr"/>
+      <c r="F839" t="inlineStr"/>
+      <c r="G839" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B840" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C840" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D840" t="inlineStr"/>
+      <c r="E840" t="inlineStr"/>
+      <c r="F840" t="inlineStr"/>
+      <c r="G840" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B841" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C841" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D841" t="inlineStr"/>
+      <c r="E841" t="inlineStr"/>
+      <c r="F841" t="inlineStr"/>
+      <c r="G841" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B842" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C842" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D842" t="inlineStr"/>
+      <c r="E842" t="inlineStr"/>
+      <c r="F842" t="inlineStr"/>
+      <c r="G842" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B843" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C843" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D843" t="inlineStr"/>
+      <c r="E843" t="inlineStr"/>
+      <c r="F843" t="inlineStr"/>
+      <c r="G843" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B844" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C844" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D844" t="inlineStr"/>
+      <c r="E844" t="inlineStr"/>
+      <c r="F844" t="inlineStr"/>
+      <c r="G844" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B845" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C845" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D845" t="inlineStr"/>
+      <c r="E845" t="inlineStr"/>
+      <c r="F845" t="inlineStr"/>
+      <c r="G845" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B846" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C846" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D846" t="inlineStr"/>
+      <c r="E846" t="inlineStr"/>
+      <c r="F846" t="inlineStr"/>
+      <c r="G846" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B847" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C847" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D847" t="inlineStr"/>
+      <c r="E847" t="inlineStr"/>
+      <c r="F847" t="inlineStr"/>
+      <c r="G847" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B848" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C848" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D848" t="inlineStr"/>
+      <c r="E848" t="inlineStr"/>
+      <c r="F848" t="inlineStr"/>
+      <c r="G848" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B849" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C849" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D849" t="inlineStr"/>
+      <c r="E849" t="inlineStr"/>
+      <c r="F849" t="inlineStr"/>
+      <c r="G849" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B850" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C850" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D850" t="inlineStr"/>
+      <c r="E850" t="inlineStr"/>
+      <c r="F850" t="inlineStr"/>
+      <c r="G850" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-10-12
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G850"/>
+  <dimension ref="A1:G865"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19168,9 +19168,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D836" t="inlineStr"/>
-      <c r="E836" t="inlineStr"/>
-      <c r="F836" t="inlineStr"/>
       <c r="G836" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19193,9 +19190,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D837" t="inlineStr"/>
-      <c r="E837" t="inlineStr"/>
-      <c r="F837" t="inlineStr"/>
       <c r="G837" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19218,9 +19212,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D838" t="inlineStr"/>
-      <c r="E838" t="inlineStr"/>
-      <c r="F838" t="inlineStr"/>
       <c r="G838" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19243,9 +19234,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D839" t="inlineStr"/>
-      <c r="E839" t="inlineStr"/>
-      <c r="F839" t="inlineStr"/>
       <c r="G839" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19268,9 +19256,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D840" t="inlineStr"/>
-      <c r="E840" t="inlineStr"/>
-      <c r="F840" t="inlineStr"/>
       <c r="G840" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19293,9 +19278,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D841" t="inlineStr"/>
-      <c r="E841" t="inlineStr"/>
-      <c r="F841" t="inlineStr"/>
       <c r="G841" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19318,9 +19300,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D842" t="inlineStr"/>
-      <c r="E842" t="inlineStr"/>
-      <c r="F842" t="inlineStr"/>
       <c r="G842" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19343,9 +19322,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D843" t="inlineStr"/>
-      <c r="E843" t="inlineStr"/>
-      <c r="F843" t="inlineStr"/>
       <c r="G843" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19368,9 +19344,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D844" t="inlineStr"/>
-      <c r="E844" t="inlineStr"/>
-      <c r="F844" t="inlineStr"/>
       <c r="G844" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19393,9 +19366,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D845" t="inlineStr"/>
-      <c r="E845" t="inlineStr"/>
-      <c r="F845" t="inlineStr"/>
       <c r="G845" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19418,9 +19388,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D846" t="inlineStr"/>
-      <c r="E846" t="inlineStr"/>
-      <c r="F846" t="inlineStr"/>
       <c r="G846" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19443,9 +19410,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D847" t="inlineStr"/>
-      <c r="E847" t="inlineStr"/>
-      <c r="F847" t="inlineStr"/>
       <c r="G847" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19468,9 +19432,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D848" t="inlineStr"/>
-      <c r="E848" t="inlineStr"/>
-      <c r="F848" t="inlineStr"/>
       <c r="G848" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19493,9 +19454,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D849" t="inlineStr"/>
-      <c r="E849" t="inlineStr"/>
-      <c r="F849" t="inlineStr"/>
       <c r="G849" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19518,10 +19476,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D850" t="inlineStr"/>
-      <c r="E850" t="inlineStr"/>
-      <c r="F850" t="inlineStr"/>
       <c r="G850" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B851" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C851" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D851" t="inlineStr"/>
+      <c r="E851" t="inlineStr"/>
+      <c r="F851" t="inlineStr"/>
+      <c r="G851" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B852" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C852" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D852" t="inlineStr"/>
+      <c r="E852" t="inlineStr"/>
+      <c r="F852" t="inlineStr"/>
+      <c r="G852" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B853" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C853" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D853" t="inlineStr"/>
+      <c r="E853" t="inlineStr"/>
+      <c r="F853" t="inlineStr"/>
+      <c r="G853" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B854" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C854" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D854" t="inlineStr"/>
+      <c r="E854" t="inlineStr"/>
+      <c r="F854" t="inlineStr"/>
+      <c r="G854" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B855" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C855" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D855" t="inlineStr"/>
+      <c r="E855" t="inlineStr"/>
+      <c r="F855" t="inlineStr"/>
+      <c r="G855" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C856" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D856" t="inlineStr"/>
+      <c r="E856" t="inlineStr"/>
+      <c r="F856" t="inlineStr"/>
+      <c r="G856" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B857" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C857" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D857" t="inlineStr"/>
+      <c r="E857" t="inlineStr"/>
+      <c r="F857" t="inlineStr"/>
+      <c r="G857" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B858" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C858" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D858" t="inlineStr"/>
+      <c r="E858" t="inlineStr"/>
+      <c r="F858" t="inlineStr"/>
+      <c r="G858" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B859" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C859" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D859" t="inlineStr"/>
+      <c r="E859" t="inlineStr"/>
+      <c r="F859" t="inlineStr"/>
+      <c r="G859" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B860" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C860" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D860" t="inlineStr"/>
+      <c r="E860" t="inlineStr"/>
+      <c r="F860" t="inlineStr"/>
+      <c r="G860" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B861" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C861" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D861" t="inlineStr"/>
+      <c r="E861" t="inlineStr"/>
+      <c r="F861" t="inlineStr"/>
+      <c r="G861" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B862" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C862" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D862" t="inlineStr"/>
+      <c r="E862" t="inlineStr"/>
+      <c r="F862" t="inlineStr"/>
+      <c r="G862" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B863" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C863" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D863" t="inlineStr"/>
+      <c r="E863" t="inlineStr"/>
+      <c r="F863" t="inlineStr"/>
+      <c r="G863" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B864" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C864" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D864" t="inlineStr"/>
+      <c r="E864" t="inlineStr"/>
+      <c r="F864" t="inlineStr"/>
+      <c r="G864" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B865" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C865" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D865" t="inlineStr"/>
+      <c r="E865" t="inlineStr"/>
+      <c r="F865" t="inlineStr"/>
+      <c r="G865" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-10-13
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G865"/>
+  <dimension ref="A1:G880"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19498,9 +19498,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D851" t="inlineStr"/>
-      <c r="E851" t="inlineStr"/>
-      <c r="F851" t="inlineStr"/>
       <c r="G851" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19523,9 +19520,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D852" t="inlineStr"/>
-      <c r="E852" t="inlineStr"/>
-      <c r="F852" t="inlineStr"/>
       <c r="G852" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19548,9 +19542,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D853" t="inlineStr"/>
-      <c r="E853" t="inlineStr"/>
-      <c r="F853" t="inlineStr"/>
       <c r="G853" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19573,9 +19564,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D854" t="inlineStr"/>
-      <c r="E854" t="inlineStr"/>
-      <c r="F854" t="inlineStr"/>
       <c r="G854" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19598,9 +19586,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D855" t="inlineStr"/>
-      <c r="E855" t="inlineStr"/>
-      <c r="F855" t="inlineStr"/>
       <c r="G855" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19623,9 +19608,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D856" t="inlineStr"/>
-      <c r="E856" t="inlineStr"/>
-      <c r="F856" t="inlineStr"/>
       <c r="G856" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19648,9 +19630,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D857" t="inlineStr"/>
-      <c r="E857" t="inlineStr"/>
-      <c r="F857" t="inlineStr"/>
       <c r="G857" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19673,9 +19652,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D858" t="inlineStr"/>
-      <c r="E858" t="inlineStr"/>
-      <c r="F858" t="inlineStr"/>
       <c r="G858" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19698,9 +19674,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D859" t="inlineStr"/>
-      <c r="E859" t="inlineStr"/>
-      <c r="F859" t="inlineStr"/>
       <c r="G859" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19723,9 +19696,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D860" t="inlineStr"/>
-      <c r="E860" t="inlineStr"/>
-      <c r="F860" t="inlineStr"/>
       <c r="G860" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19748,9 +19718,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D861" t="inlineStr"/>
-      <c r="E861" t="inlineStr"/>
-      <c r="F861" t="inlineStr"/>
       <c r="G861" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19773,9 +19740,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D862" t="inlineStr"/>
-      <c r="E862" t="inlineStr"/>
-      <c r="F862" t="inlineStr"/>
       <c r="G862" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19798,9 +19762,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D863" t="inlineStr"/>
-      <c r="E863" t="inlineStr"/>
-      <c r="F863" t="inlineStr"/>
       <c r="G863" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19823,9 +19784,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D864" t="inlineStr"/>
-      <c r="E864" t="inlineStr"/>
-      <c r="F864" t="inlineStr"/>
       <c r="G864" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19848,10 +19806,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D865" t="inlineStr"/>
-      <c r="E865" t="inlineStr"/>
-      <c r="F865" t="inlineStr"/>
       <c r="G865" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B866" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C866" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D866" t="inlineStr"/>
+      <c r="E866" t="inlineStr"/>
+      <c r="F866" t="inlineStr"/>
+      <c r="G866" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B867" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C867" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D867" t="inlineStr"/>
+      <c r="E867" t="inlineStr"/>
+      <c r="F867" t="inlineStr"/>
+      <c r="G867" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B868" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C868" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D868" t="inlineStr"/>
+      <c r="E868" t="inlineStr"/>
+      <c r="F868" t="inlineStr"/>
+      <c r="G868" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B869" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C869" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D869" t="inlineStr"/>
+      <c r="E869" t="inlineStr"/>
+      <c r="F869" t="inlineStr"/>
+      <c r="G869" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B870" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C870" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D870" t="inlineStr"/>
+      <c r="E870" t="inlineStr"/>
+      <c r="F870" t="inlineStr"/>
+      <c r="G870" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B871" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C871" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D871" t="inlineStr"/>
+      <c r="E871" t="inlineStr"/>
+      <c r="F871" t="inlineStr"/>
+      <c r="G871" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B872" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C872" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D872" t="inlineStr"/>
+      <c r="E872" t="inlineStr"/>
+      <c r="F872" t="inlineStr"/>
+      <c r="G872" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B873" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C873" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D873" t="inlineStr"/>
+      <c r="E873" t="inlineStr"/>
+      <c r="F873" t="inlineStr"/>
+      <c r="G873" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B874" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C874" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D874" t="inlineStr"/>
+      <c r="E874" t="inlineStr"/>
+      <c r="F874" t="inlineStr"/>
+      <c r="G874" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B875" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C875" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D875" t="inlineStr"/>
+      <c r="E875" t="inlineStr"/>
+      <c r="F875" t="inlineStr"/>
+      <c r="G875" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B876" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C876" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D876" t="inlineStr"/>
+      <c r="E876" t="inlineStr"/>
+      <c r="F876" t="inlineStr"/>
+      <c r="G876" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B877" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C877" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D877" t="inlineStr"/>
+      <c r="E877" t="inlineStr"/>
+      <c r="F877" t="inlineStr"/>
+      <c r="G877" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B878" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C878" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D878" t="inlineStr"/>
+      <c r="E878" t="inlineStr"/>
+      <c r="F878" t="inlineStr"/>
+      <c r="G878" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B879" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C879" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D879" t="inlineStr"/>
+      <c r="E879" t="inlineStr"/>
+      <c r="F879" t="inlineStr"/>
+      <c r="G879" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B880" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C880" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D880" t="inlineStr"/>
+      <c r="E880" t="inlineStr"/>
+      <c r="F880" t="inlineStr"/>
+      <c r="G880" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-10-14
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G880"/>
+  <dimension ref="A1:G895"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19828,9 +19828,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D866" t="inlineStr"/>
-      <c r="E866" t="inlineStr"/>
-      <c r="F866" t="inlineStr"/>
       <c r="G866" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19853,9 +19850,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D867" t="inlineStr"/>
-      <c r="E867" t="inlineStr"/>
-      <c r="F867" t="inlineStr"/>
       <c r="G867" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19878,9 +19872,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D868" t="inlineStr"/>
-      <c r="E868" t="inlineStr"/>
-      <c r="F868" t="inlineStr"/>
       <c r="G868" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19903,9 +19894,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D869" t="inlineStr"/>
-      <c r="E869" t="inlineStr"/>
-      <c r="F869" t="inlineStr"/>
       <c r="G869" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19928,9 +19916,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D870" t="inlineStr"/>
-      <c r="E870" t="inlineStr"/>
-      <c r="F870" t="inlineStr"/>
       <c r="G870" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19953,9 +19938,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D871" t="inlineStr"/>
-      <c r="E871" t="inlineStr"/>
-      <c r="F871" t="inlineStr"/>
       <c r="G871" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -19978,9 +19960,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D872" t="inlineStr"/>
-      <c r="E872" t="inlineStr"/>
-      <c r="F872" t="inlineStr"/>
       <c r="G872" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20003,9 +19982,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D873" t="inlineStr"/>
-      <c r="E873" t="inlineStr"/>
-      <c r="F873" t="inlineStr"/>
       <c r="G873" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20028,9 +20004,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D874" t="inlineStr"/>
-      <c r="E874" t="inlineStr"/>
-      <c r="F874" t="inlineStr"/>
       <c r="G874" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20053,9 +20026,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D875" t="inlineStr"/>
-      <c r="E875" t="inlineStr"/>
-      <c r="F875" t="inlineStr"/>
       <c r="G875" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20078,9 +20048,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D876" t="inlineStr"/>
-      <c r="E876" t="inlineStr"/>
-      <c r="F876" t="inlineStr"/>
       <c r="G876" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20103,9 +20070,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D877" t="inlineStr"/>
-      <c r="E877" t="inlineStr"/>
-      <c r="F877" t="inlineStr"/>
       <c r="G877" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20128,9 +20092,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D878" t="inlineStr"/>
-      <c r="E878" t="inlineStr"/>
-      <c r="F878" t="inlineStr"/>
       <c r="G878" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20153,9 +20114,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D879" t="inlineStr"/>
-      <c r="E879" t="inlineStr"/>
-      <c r="F879" t="inlineStr"/>
       <c r="G879" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20178,10 +20136,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D880" t="inlineStr"/>
-      <c r="E880" t="inlineStr"/>
-      <c r="F880" t="inlineStr"/>
       <c r="G880" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B881" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C881" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D881" t="inlineStr"/>
+      <c r="E881" t="inlineStr"/>
+      <c r="F881" t="inlineStr"/>
+      <c r="G881" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B882" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C882" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D882" t="inlineStr"/>
+      <c r="E882" t="inlineStr"/>
+      <c r="F882" t="inlineStr"/>
+      <c r="G882" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B883" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C883" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D883" t="inlineStr"/>
+      <c r="E883" t="inlineStr"/>
+      <c r="F883" t="inlineStr"/>
+      <c r="G883" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B884" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C884" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D884" t="inlineStr"/>
+      <c r="E884" t="inlineStr"/>
+      <c r="F884" t="inlineStr"/>
+      <c r="G884" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B885" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C885" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D885" t="inlineStr"/>
+      <c r="E885" t="inlineStr"/>
+      <c r="F885" t="inlineStr"/>
+      <c r="G885" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B886" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C886" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D886" t="inlineStr"/>
+      <c r="E886" t="inlineStr"/>
+      <c r="F886" t="inlineStr"/>
+      <c r="G886" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B887" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C887" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D887" t="inlineStr"/>
+      <c r="E887" t="inlineStr"/>
+      <c r="F887" t="inlineStr"/>
+      <c r="G887" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B888" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C888" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D888" t="inlineStr"/>
+      <c r="E888" t="inlineStr"/>
+      <c r="F888" t="inlineStr"/>
+      <c r="G888" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B889" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C889" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D889" t="inlineStr"/>
+      <c r="E889" t="inlineStr"/>
+      <c r="F889" t="inlineStr"/>
+      <c r="G889" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B890" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C890" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D890" t="inlineStr"/>
+      <c r="E890" t="inlineStr"/>
+      <c r="F890" t="inlineStr"/>
+      <c r="G890" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B891" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C891" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D891" t="inlineStr"/>
+      <c r="E891" t="inlineStr"/>
+      <c r="F891" t="inlineStr"/>
+      <c r="G891" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B892" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C892" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D892" t="inlineStr"/>
+      <c r="E892" t="inlineStr"/>
+      <c r="F892" t="inlineStr"/>
+      <c r="G892" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B893" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C893" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D893" t="inlineStr"/>
+      <c r="E893" t="inlineStr"/>
+      <c r="F893" t="inlineStr"/>
+      <c r="G893" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B894" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C894" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D894" t="inlineStr"/>
+      <c r="E894" t="inlineStr"/>
+      <c r="F894" t="inlineStr"/>
+      <c r="G894" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B895" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C895" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D895" t="inlineStr"/>
+      <c r="E895" t="inlineStr"/>
+      <c r="F895" t="inlineStr"/>
+      <c r="G895" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-10-15
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G895"/>
+  <dimension ref="A1:G910"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20158,9 +20158,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D881" t="inlineStr"/>
-      <c r="E881" t="inlineStr"/>
-      <c r="F881" t="inlineStr"/>
       <c r="G881" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20183,9 +20180,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D882" t="inlineStr"/>
-      <c r="E882" t="inlineStr"/>
-      <c r="F882" t="inlineStr"/>
       <c r="G882" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20208,9 +20202,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D883" t="inlineStr"/>
-      <c r="E883" t="inlineStr"/>
-      <c r="F883" t="inlineStr"/>
       <c r="G883" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20233,9 +20224,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D884" t="inlineStr"/>
-      <c r="E884" t="inlineStr"/>
-      <c r="F884" t="inlineStr"/>
       <c r="G884" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20258,9 +20246,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D885" t="inlineStr"/>
-      <c r="E885" t="inlineStr"/>
-      <c r="F885" t="inlineStr"/>
       <c r="G885" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20283,9 +20268,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D886" t="inlineStr"/>
-      <c r="E886" t="inlineStr"/>
-      <c r="F886" t="inlineStr"/>
       <c r="G886" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20308,9 +20290,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D887" t="inlineStr"/>
-      <c r="E887" t="inlineStr"/>
-      <c r="F887" t="inlineStr"/>
       <c r="G887" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20333,9 +20312,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D888" t="inlineStr"/>
-      <c r="E888" t="inlineStr"/>
-      <c r="F888" t="inlineStr"/>
       <c r="G888" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20358,9 +20334,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D889" t="inlineStr"/>
-      <c r="E889" t="inlineStr"/>
-      <c r="F889" t="inlineStr"/>
       <c r="G889" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20383,9 +20356,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D890" t="inlineStr"/>
-      <c r="E890" t="inlineStr"/>
-      <c r="F890" t="inlineStr"/>
       <c r="G890" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20408,9 +20378,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D891" t="inlineStr"/>
-      <c r="E891" t="inlineStr"/>
-      <c r="F891" t="inlineStr"/>
       <c r="G891" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20433,9 +20400,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D892" t="inlineStr"/>
-      <c r="E892" t="inlineStr"/>
-      <c r="F892" t="inlineStr"/>
       <c r="G892" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20458,9 +20422,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D893" t="inlineStr"/>
-      <c r="E893" t="inlineStr"/>
-      <c r="F893" t="inlineStr"/>
       <c r="G893" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20483,9 +20444,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D894" t="inlineStr"/>
-      <c r="E894" t="inlineStr"/>
-      <c r="F894" t="inlineStr"/>
       <c r="G894" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20508,10 +20466,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D895" t="inlineStr"/>
-      <c r="E895" t="inlineStr"/>
-      <c r="F895" t="inlineStr"/>
       <c r="G895" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B896" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C896" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D896" t="inlineStr"/>
+      <c r="E896" t="inlineStr"/>
+      <c r="F896" t="inlineStr"/>
+      <c r="G896" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B897" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C897" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D897" t="inlineStr"/>
+      <c r="E897" t="inlineStr"/>
+      <c r="F897" t="inlineStr"/>
+      <c r="G897" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B898" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C898" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D898" t="inlineStr"/>
+      <c r="E898" t="inlineStr"/>
+      <c r="F898" t="inlineStr"/>
+      <c r="G898" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B899" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C899" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D899" t="inlineStr"/>
+      <c r="E899" t="inlineStr"/>
+      <c r="F899" t="inlineStr"/>
+      <c r="G899" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B900" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C900" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D900" t="inlineStr"/>
+      <c r="E900" t="inlineStr"/>
+      <c r="F900" t="inlineStr"/>
+      <c r="G900" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B901" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C901" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D901" t="inlineStr"/>
+      <c r="E901" t="inlineStr"/>
+      <c r="F901" t="inlineStr"/>
+      <c r="G901" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B902" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C902" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D902" t="inlineStr"/>
+      <c r="E902" t="inlineStr"/>
+      <c r="F902" t="inlineStr"/>
+      <c r="G902" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="903">
+      <c r="A903" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B903" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C903" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D903" t="inlineStr"/>
+      <c r="E903" t="inlineStr"/>
+      <c r="F903" t="inlineStr"/>
+      <c r="G903" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B904" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C904" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D904" t="inlineStr"/>
+      <c r="E904" t="inlineStr"/>
+      <c r="F904" t="inlineStr"/>
+      <c r="G904" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B905" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C905" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D905" t="inlineStr"/>
+      <c r="E905" t="inlineStr"/>
+      <c r="F905" t="inlineStr"/>
+      <c r="G905" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B906" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C906" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D906" t="inlineStr"/>
+      <c r="E906" t="inlineStr"/>
+      <c r="F906" t="inlineStr"/>
+      <c r="G906" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B907" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C907" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D907" t="inlineStr"/>
+      <c r="E907" t="inlineStr"/>
+      <c r="F907" t="inlineStr"/>
+      <c r="G907" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B908" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C908" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D908" t="inlineStr"/>
+      <c r="E908" t="inlineStr"/>
+      <c r="F908" t="inlineStr"/>
+      <c r="G908" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B909" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C909" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D909" t="inlineStr"/>
+      <c r="E909" t="inlineStr"/>
+      <c r="F909" t="inlineStr"/>
+      <c r="G909" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="910">
+      <c r="A910" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B910" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C910" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D910" t="inlineStr"/>
+      <c r="E910" t="inlineStr"/>
+      <c r="F910" t="inlineStr"/>
+      <c r="G910" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-10-16
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G910"/>
+  <dimension ref="A1:G925"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20488,9 +20488,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D896" t="inlineStr"/>
-      <c r="E896" t="inlineStr"/>
-      <c r="F896" t="inlineStr"/>
       <c r="G896" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20513,9 +20510,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D897" t="inlineStr"/>
-      <c r="E897" t="inlineStr"/>
-      <c r="F897" t="inlineStr"/>
       <c r="G897" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20538,9 +20532,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D898" t="inlineStr"/>
-      <c r="E898" t="inlineStr"/>
-      <c r="F898" t="inlineStr"/>
       <c r="G898" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20563,9 +20554,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D899" t="inlineStr"/>
-      <c r="E899" t="inlineStr"/>
-      <c r="F899" t="inlineStr"/>
       <c r="G899" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20588,9 +20576,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D900" t="inlineStr"/>
-      <c r="E900" t="inlineStr"/>
-      <c r="F900" t="inlineStr"/>
       <c r="G900" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20613,9 +20598,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D901" t="inlineStr"/>
-      <c r="E901" t="inlineStr"/>
-      <c r="F901" t="inlineStr"/>
       <c r="G901" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20638,9 +20620,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D902" t="inlineStr"/>
-      <c r="E902" t="inlineStr"/>
-      <c r="F902" t="inlineStr"/>
       <c r="G902" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20663,9 +20642,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D903" t="inlineStr"/>
-      <c r="E903" t="inlineStr"/>
-      <c r="F903" t="inlineStr"/>
       <c r="G903" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20688,9 +20664,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D904" t="inlineStr"/>
-      <c r="E904" t="inlineStr"/>
-      <c r="F904" t="inlineStr"/>
       <c r="G904" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20713,9 +20686,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D905" t="inlineStr"/>
-      <c r="E905" t="inlineStr"/>
-      <c r="F905" t="inlineStr"/>
       <c r="G905" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20738,9 +20708,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D906" t="inlineStr"/>
-      <c r="E906" t="inlineStr"/>
-      <c r="F906" t="inlineStr"/>
       <c r="G906" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20763,9 +20730,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D907" t="inlineStr"/>
-      <c r="E907" t="inlineStr"/>
-      <c r="F907" t="inlineStr"/>
       <c r="G907" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20788,9 +20752,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D908" t="inlineStr"/>
-      <c r="E908" t="inlineStr"/>
-      <c r="F908" t="inlineStr"/>
       <c r="G908" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20813,9 +20774,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D909" t="inlineStr"/>
-      <c r="E909" t="inlineStr"/>
-      <c r="F909" t="inlineStr"/>
       <c r="G909" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20838,10 +20796,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D910" t="inlineStr"/>
-      <c r="E910" t="inlineStr"/>
-      <c r="F910" t="inlineStr"/>
       <c r="G910" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B911" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C911" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D911" t="inlineStr"/>
+      <c r="E911" t="inlineStr"/>
+      <c r="F911" t="inlineStr"/>
+      <c r="G911" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B912" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C912" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D912" t="inlineStr"/>
+      <c r="E912" t="inlineStr"/>
+      <c r="F912" t="inlineStr"/>
+      <c r="G912" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B913" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C913" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D913" t="inlineStr"/>
+      <c r="E913" t="inlineStr"/>
+      <c r="F913" t="inlineStr"/>
+      <c r="G913" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B914" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C914" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D914" t="inlineStr"/>
+      <c r="E914" t="inlineStr"/>
+      <c r="F914" t="inlineStr"/>
+      <c r="G914" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B915" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C915" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D915" t="inlineStr"/>
+      <c r="E915" t="inlineStr"/>
+      <c r="F915" t="inlineStr"/>
+      <c r="G915" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B916" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C916" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D916" t="inlineStr"/>
+      <c r="E916" t="inlineStr"/>
+      <c r="F916" t="inlineStr"/>
+      <c r="G916" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B917" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C917" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D917" t="inlineStr"/>
+      <c r="E917" t="inlineStr"/>
+      <c r="F917" t="inlineStr"/>
+      <c r="G917" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B918" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C918" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D918" t="inlineStr"/>
+      <c r="E918" t="inlineStr"/>
+      <c r="F918" t="inlineStr"/>
+      <c r="G918" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B919" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C919" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D919" t="inlineStr"/>
+      <c r="E919" t="inlineStr"/>
+      <c r="F919" t="inlineStr"/>
+      <c r="G919" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B920" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C920" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D920" t="inlineStr"/>
+      <c r="E920" t="inlineStr"/>
+      <c r="F920" t="inlineStr"/>
+      <c r="G920" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B921" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C921" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D921" t="inlineStr"/>
+      <c r="E921" t="inlineStr"/>
+      <c r="F921" t="inlineStr"/>
+      <c r="G921" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="922">
+      <c r="A922" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B922" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C922" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D922" t="inlineStr"/>
+      <c r="E922" t="inlineStr"/>
+      <c r="F922" t="inlineStr"/>
+      <c r="G922" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="923">
+      <c r="A923" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B923" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C923" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D923" t="inlineStr"/>
+      <c r="E923" t="inlineStr"/>
+      <c r="F923" t="inlineStr"/>
+      <c r="G923" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B924" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C924" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D924" t="inlineStr"/>
+      <c r="E924" t="inlineStr"/>
+      <c r="F924" t="inlineStr"/>
+      <c r="G924" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B925" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C925" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D925" t="inlineStr"/>
+      <c r="E925" t="inlineStr"/>
+      <c r="F925" t="inlineStr"/>
+      <c r="G925" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-10-17
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G925"/>
+  <dimension ref="A1:G940"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20818,9 +20818,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D911" t="inlineStr"/>
-      <c r="E911" t="inlineStr"/>
-      <c r="F911" t="inlineStr"/>
       <c r="G911" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20843,9 +20840,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D912" t="inlineStr"/>
-      <c r="E912" t="inlineStr"/>
-      <c r="F912" t="inlineStr"/>
       <c r="G912" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20868,9 +20862,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D913" t="inlineStr"/>
-      <c r="E913" t="inlineStr"/>
-      <c r="F913" t="inlineStr"/>
       <c r="G913" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20893,9 +20884,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D914" t="inlineStr"/>
-      <c r="E914" t="inlineStr"/>
-      <c r="F914" t="inlineStr"/>
       <c r="G914" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20918,9 +20906,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D915" t="inlineStr"/>
-      <c r="E915" t="inlineStr"/>
-      <c r="F915" t="inlineStr"/>
       <c r="G915" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20943,9 +20928,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D916" t="inlineStr"/>
-      <c r="E916" t="inlineStr"/>
-      <c r="F916" t="inlineStr"/>
       <c r="G916" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20968,9 +20950,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D917" t="inlineStr"/>
-      <c r="E917" t="inlineStr"/>
-      <c r="F917" t="inlineStr"/>
       <c r="G917" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -20993,9 +20972,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D918" t="inlineStr"/>
-      <c r="E918" t="inlineStr"/>
-      <c r="F918" t="inlineStr"/>
       <c r="G918" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21018,9 +20994,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D919" t="inlineStr"/>
-      <c r="E919" t="inlineStr"/>
-      <c r="F919" t="inlineStr"/>
       <c r="G919" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21043,9 +21016,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D920" t="inlineStr"/>
-      <c r="E920" t="inlineStr"/>
-      <c r="F920" t="inlineStr"/>
       <c r="G920" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21068,9 +21038,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D921" t="inlineStr"/>
-      <c r="E921" t="inlineStr"/>
-      <c r="F921" t="inlineStr"/>
       <c r="G921" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21093,9 +21060,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D922" t="inlineStr"/>
-      <c r="E922" t="inlineStr"/>
-      <c r="F922" t="inlineStr"/>
       <c r="G922" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21118,9 +21082,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D923" t="inlineStr"/>
-      <c r="E923" t="inlineStr"/>
-      <c r="F923" t="inlineStr"/>
       <c r="G923" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21143,9 +21104,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D924" t="inlineStr"/>
-      <c r="E924" t="inlineStr"/>
-      <c r="F924" t="inlineStr"/>
       <c r="G924" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21168,10 +21126,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D925" t="inlineStr"/>
-      <c r="E925" t="inlineStr"/>
-      <c r="F925" t="inlineStr"/>
       <c r="G925" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="926">
+      <c r="A926" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B926" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C926" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D926" t="inlineStr"/>
+      <c r="E926" t="inlineStr"/>
+      <c r="F926" t="inlineStr"/>
+      <c r="G926" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B927" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C927" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D927" t="inlineStr"/>
+      <c r="E927" t="inlineStr"/>
+      <c r="F927" t="inlineStr"/>
+      <c r="G927" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B928" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C928" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D928" t="inlineStr"/>
+      <c r="E928" t="inlineStr"/>
+      <c r="F928" t="inlineStr"/>
+      <c r="G928" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B929" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C929" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D929" t="inlineStr"/>
+      <c r="E929" t="inlineStr"/>
+      <c r="F929" t="inlineStr"/>
+      <c r="G929" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B930" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C930" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D930" t="inlineStr"/>
+      <c r="E930" t="inlineStr"/>
+      <c r="F930" t="inlineStr"/>
+      <c r="G930" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B931" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C931" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D931" t="inlineStr"/>
+      <c r="E931" t="inlineStr"/>
+      <c r="F931" t="inlineStr"/>
+      <c r="G931" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B932" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C932" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D932" t="inlineStr"/>
+      <c r="E932" t="inlineStr"/>
+      <c r="F932" t="inlineStr"/>
+      <c r="G932" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B933" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C933" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D933" t="inlineStr"/>
+      <c r="E933" t="inlineStr"/>
+      <c r="F933" t="inlineStr"/>
+      <c r="G933" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B934" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C934" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D934" t="inlineStr"/>
+      <c r="E934" t="inlineStr"/>
+      <c r="F934" t="inlineStr"/>
+      <c r="G934" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B935" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C935" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D935" t="inlineStr"/>
+      <c r="E935" t="inlineStr"/>
+      <c r="F935" t="inlineStr"/>
+      <c r="G935" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B936" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C936" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D936" t="inlineStr"/>
+      <c r="E936" t="inlineStr"/>
+      <c r="F936" t="inlineStr"/>
+      <c r="G936" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B937" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C937" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D937" t="inlineStr"/>
+      <c r="E937" t="inlineStr"/>
+      <c r="F937" t="inlineStr"/>
+      <c r="G937" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="938">
+      <c r="A938" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B938" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C938" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D938" t="inlineStr"/>
+      <c r="E938" t="inlineStr"/>
+      <c r="F938" t="inlineStr"/>
+      <c r="G938" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="939">
+      <c r="A939" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B939" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C939" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D939" t="inlineStr"/>
+      <c r="E939" t="inlineStr"/>
+      <c r="F939" t="inlineStr"/>
+      <c r="G939" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="940">
+      <c r="A940" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B940" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C940" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D940" t="inlineStr"/>
+      <c r="E940" t="inlineStr"/>
+      <c r="F940" t="inlineStr"/>
+      <c r="G940" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-10-18
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G940"/>
+  <dimension ref="A1:G955"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21148,9 +21148,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D926" t="inlineStr"/>
-      <c r="E926" t="inlineStr"/>
-      <c r="F926" t="inlineStr"/>
       <c r="G926" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21173,9 +21170,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D927" t="inlineStr"/>
-      <c r="E927" t="inlineStr"/>
-      <c r="F927" t="inlineStr"/>
       <c r="G927" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21198,9 +21192,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D928" t="inlineStr"/>
-      <c r="E928" t="inlineStr"/>
-      <c r="F928" t="inlineStr"/>
       <c r="G928" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21223,9 +21214,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D929" t="inlineStr"/>
-      <c r="E929" t="inlineStr"/>
-      <c r="F929" t="inlineStr"/>
       <c r="G929" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21248,9 +21236,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D930" t="inlineStr"/>
-      <c r="E930" t="inlineStr"/>
-      <c r="F930" t="inlineStr"/>
       <c r="G930" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21273,9 +21258,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D931" t="inlineStr"/>
-      <c r="E931" t="inlineStr"/>
-      <c r="F931" t="inlineStr"/>
       <c r="G931" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21298,9 +21280,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D932" t="inlineStr"/>
-      <c r="E932" t="inlineStr"/>
-      <c r="F932" t="inlineStr"/>
       <c r="G932" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21323,9 +21302,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D933" t="inlineStr"/>
-      <c r="E933" t="inlineStr"/>
-      <c r="F933" t="inlineStr"/>
       <c r="G933" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21348,9 +21324,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D934" t="inlineStr"/>
-      <c r="E934" t="inlineStr"/>
-      <c r="F934" t="inlineStr"/>
       <c r="G934" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21373,9 +21346,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D935" t="inlineStr"/>
-      <c r="E935" t="inlineStr"/>
-      <c r="F935" t="inlineStr"/>
       <c r="G935" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21398,9 +21368,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D936" t="inlineStr"/>
-      <c r="E936" t="inlineStr"/>
-      <c r="F936" t="inlineStr"/>
       <c r="G936" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21423,9 +21390,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D937" t="inlineStr"/>
-      <c r="E937" t="inlineStr"/>
-      <c r="F937" t="inlineStr"/>
       <c r="G937" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21448,9 +21412,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D938" t="inlineStr"/>
-      <c r="E938" t="inlineStr"/>
-      <c r="F938" t="inlineStr"/>
       <c r="G938" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21473,9 +21434,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D939" t="inlineStr"/>
-      <c r="E939" t="inlineStr"/>
-      <c r="F939" t="inlineStr"/>
       <c r="G939" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21498,10 +21456,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D940" t="inlineStr"/>
-      <c r="E940" t="inlineStr"/>
-      <c r="F940" t="inlineStr"/>
       <c r="G940" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="941">
+      <c r="A941" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B941" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C941" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D941" t="inlineStr"/>
+      <c r="E941" t="inlineStr"/>
+      <c r="F941" t="inlineStr"/>
+      <c r="G941" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="942">
+      <c r="A942" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B942" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C942" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D942" t="inlineStr"/>
+      <c r="E942" t="inlineStr"/>
+      <c r="F942" t="inlineStr"/>
+      <c r="G942" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="943">
+      <c r="A943" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B943" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C943" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D943" t="inlineStr"/>
+      <c r="E943" t="inlineStr"/>
+      <c r="F943" t="inlineStr"/>
+      <c r="G943" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="944">
+      <c r="A944" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B944" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C944" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D944" t="inlineStr"/>
+      <c r="E944" t="inlineStr"/>
+      <c r="F944" t="inlineStr"/>
+      <c r="G944" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="945">
+      <c r="A945" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B945" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C945" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D945" t="inlineStr"/>
+      <c r="E945" t="inlineStr"/>
+      <c r="F945" t="inlineStr"/>
+      <c r="G945" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="946">
+      <c r="A946" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B946" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C946" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D946" t="inlineStr"/>
+      <c r="E946" t="inlineStr"/>
+      <c r="F946" t="inlineStr"/>
+      <c r="G946" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="947">
+      <c r="A947" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B947" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C947" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D947" t="inlineStr"/>
+      <c r="E947" t="inlineStr"/>
+      <c r="F947" t="inlineStr"/>
+      <c r="G947" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="948">
+      <c r="A948" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B948" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C948" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D948" t="inlineStr"/>
+      <c r="E948" t="inlineStr"/>
+      <c r="F948" t="inlineStr"/>
+      <c r="G948" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="949">
+      <c r="A949" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B949" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C949" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D949" t="inlineStr"/>
+      <c r="E949" t="inlineStr"/>
+      <c r="F949" t="inlineStr"/>
+      <c r="G949" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="950">
+      <c r="A950" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B950" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C950" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D950" t="inlineStr"/>
+      <c r="E950" t="inlineStr"/>
+      <c r="F950" t="inlineStr"/>
+      <c r="G950" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="951">
+      <c r="A951" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B951" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C951" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D951" t="inlineStr"/>
+      <c r="E951" t="inlineStr"/>
+      <c r="F951" t="inlineStr"/>
+      <c r="G951" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="952">
+      <c r="A952" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B952" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C952" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D952" t="inlineStr"/>
+      <c r="E952" t="inlineStr"/>
+      <c r="F952" t="inlineStr"/>
+      <c r="G952" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B953" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C953" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D953" t="inlineStr"/>
+      <c r="E953" t="inlineStr"/>
+      <c r="F953" t="inlineStr"/>
+      <c r="G953" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="954">
+      <c r="A954" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B954" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C954" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D954" t="inlineStr"/>
+      <c r="E954" t="inlineStr"/>
+      <c r="F954" t="inlineStr"/>
+      <c r="G954" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="955">
+      <c r="A955" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B955" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C955" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D955" t="inlineStr"/>
+      <c r="E955" t="inlineStr"/>
+      <c r="F955" t="inlineStr"/>
+      <c r="G955" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-10-19
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G955"/>
+  <dimension ref="A1:G970"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21478,9 +21478,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D941" t="inlineStr"/>
-      <c r="E941" t="inlineStr"/>
-      <c r="F941" t="inlineStr"/>
       <c r="G941" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21503,9 +21500,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D942" t="inlineStr"/>
-      <c r="E942" t="inlineStr"/>
-      <c r="F942" t="inlineStr"/>
       <c r="G942" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21528,9 +21522,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D943" t="inlineStr"/>
-      <c r="E943" t="inlineStr"/>
-      <c r="F943" t="inlineStr"/>
       <c r="G943" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21553,9 +21544,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D944" t="inlineStr"/>
-      <c r="E944" t="inlineStr"/>
-      <c r="F944" t="inlineStr"/>
       <c r="G944" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21578,9 +21566,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D945" t="inlineStr"/>
-      <c r="E945" t="inlineStr"/>
-      <c r="F945" t="inlineStr"/>
       <c r="G945" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21603,9 +21588,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D946" t="inlineStr"/>
-      <c r="E946" t="inlineStr"/>
-      <c r="F946" t="inlineStr"/>
       <c r="G946" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21628,9 +21610,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D947" t="inlineStr"/>
-      <c r="E947" t="inlineStr"/>
-      <c r="F947" t="inlineStr"/>
       <c r="G947" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21653,9 +21632,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D948" t="inlineStr"/>
-      <c r="E948" t="inlineStr"/>
-      <c r="F948" t="inlineStr"/>
       <c r="G948" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21678,9 +21654,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D949" t="inlineStr"/>
-      <c r="E949" t="inlineStr"/>
-      <c r="F949" t="inlineStr"/>
       <c r="G949" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21703,9 +21676,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D950" t="inlineStr"/>
-      <c r="E950" t="inlineStr"/>
-      <c r="F950" t="inlineStr"/>
       <c r="G950" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21728,9 +21698,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D951" t="inlineStr"/>
-      <c r="E951" t="inlineStr"/>
-      <c r="F951" t="inlineStr"/>
       <c r="G951" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21753,9 +21720,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D952" t="inlineStr"/>
-      <c r="E952" t="inlineStr"/>
-      <c r="F952" t="inlineStr"/>
       <c r="G952" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21778,9 +21742,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D953" t="inlineStr"/>
-      <c r="E953" t="inlineStr"/>
-      <c r="F953" t="inlineStr"/>
       <c r="G953" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21803,9 +21764,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D954" t="inlineStr"/>
-      <c r="E954" t="inlineStr"/>
-      <c r="F954" t="inlineStr"/>
       <c r="G954" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21828,10 +21786,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D955" t="inlineStr"/>
-      <c r="E955" t="inlineStr"/>
-      <c r="F955" t="inlineStr"/>
       <c r="G955" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="956">
+      <c r="A956" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B956" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C956" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D956" t="inlineStr"/>
+      <c r="E956" t="inlineStr"/>
+      <c r="F956" t="inlineStr"/>
+      <c r="G956" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="957">
+      <c r="A957" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B957" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C957" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D957" t="inlineStr"/>
+      <c r="E957" t="inlineStr"/>
+      <c r="F957" t="inlineStr"/>
+      <c r="G957" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="958">
+      <c r="A958" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B958" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C958" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D958" t="inlineStr"/>
+      <c r="E958" t="inlineStr"/>
+      <c r="F958" t="inlineStr"/>
+      <c r="G958" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="959">
+      <c r="A959" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B959" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C959" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D959" t="inlineStr"/>
+      <c r="E959" t="inlineStr"/>
+      <c r="F959" t="inlineStr"/>
+      <c r="G959" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="960">
+      <c r="A960" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B960" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C960" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D960" t="inlineStr"/>
+      <c r="E960" t="inlineStr"/>
+      <c r="F960" t="inlineStr"/>
+      <c r="G960" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="961">
+      <c r="A961" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B961" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C961" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D961" t="inlineStr"/>
+      <c r="E961" t="inlineStr"/>
+      <c r="F961" t="inlineStr"/>
+      <c r="G961" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="962">
+      <c r="A962" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B962" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C962" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D962" t="inlineStr"/>
+      <c r="E962" t="inlineStr"/>
+      <c r="F962" t="inlineStr"/>
+      <c r="G962" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="963">
+      <c r="A963" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B963" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C963" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D963" t="inlineStr"/>
+      <c r="E963" t="inlineStr"/>
+      <c r="F963" t="inlineStr"/>
+      <c r="G963" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="964">
+      <c r="A964" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B964" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C964" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D964" t="inlineStr"/>
+      <c r="E964" t="inlineStr"/>
+      <c r="F964" t="inlineStr"/>
+      <c r="G964" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="965">
+      <c r="A965" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B965" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C965" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D965" t="inlineStr"/>
+      <c r="E965" t="inlineStr"/>
+      <c r="F965" t="inlineStr"/>
+      <c r="G965" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="966">
+      <c r="A966" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B966" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C966" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D966" t="inlineStr"/>
+      <c r="E966" t="inlineStr"/>
+      <c r="F966" t="inlineStr"/>
+      <c r="G966" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="967">
+      <c r="A967" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B967" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C967" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D967" t="inlineStr"/>
+      <c r="E967" t="inlineStr"/>
+      <c r="F967" t="inlineStr"/>
+      <c r="G967" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="968">
+      <c r="A968" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B968" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C968" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D968" t="inlineStr"/>
+      <c r="E968" t="inlineStr"/>
+      <c r="F968" t="inlineStr"/>
+      <c r="G968" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="969">
+      <c r="A969" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B969" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C969" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D969" t="inlineStr"/>
+      <c r="E969" t="inlineStr"/>
+      <c r="F969" t="inlineStr"/>
+      <c r="G969" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="970">
+      <c r="A970" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B970" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C970" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D970" t="inlineStr"/>
+      <c r="E970" t="inlineStr"/>
+      <c r="F970" t="inlineStr"/>
+      <c r="G970" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-10-20
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G970"/>
+  <dimension ref="A1:G985"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21808,9 +21808,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D956" t="inlineStr"/>
-      <c r="E956" t="inlineStr"/>
-      <c r="F956" t="inlineStr"/>
       <c r="G956" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21833,9 +21830,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D957" t="inlineStr"/>
-      <c r="E957" t="inlineStr"/>
-      <c r="F957" t="inlineStr"/>
       <c r="G957" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21858,9 +21852,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D958" t="inlineStr"/>
-      <c r="E958" t="inlineStr"/>
-      <c r="F958" t="inlineStr"/>
       <c r="G958" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21883,9 +21874,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D959" t="inlineStr"/>
-      <c r="E959" t="inlineStr"/>
-      <c r="F959" t="inlineStr"/>
       <c r="G959" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21908,9 +21896,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D960" t="inlineStr"/>
-      <c r="E960" t="inlineStr"/>
-      <c r="F960" t="inlineStr"/>
       <c r="G960" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21933,9 +21918,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D961" t="inlineStr"/>
-      <c r="E961" t="inlineStr"/>
-      <c r="F961" t="inlineStr"/>
       <c r="G961" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21958,9 +21940,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D962" t="inlineStr"/>
-      <c r="E962" t="inlineStr"/>
-      <c r="F962" t="inlineStr"/>
       <c r="G962" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -21983,9 +21962,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D963" t="inlineStr"/>
-      <c r="E963" t="inlineStr"/>
-      <c r="F963" t="inlineStr"/>
       <c r="G963" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22008,9 +21984,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D964" t="inlineStr"/>
-      <c r="E964" t="inlineStr"/>
-      <c r="F964" t="inlineStr"/>
       <c r="G964" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22033,9 +22006,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D965" t="inlineStr"/>
-      <c r="E965" t="inlineStr"/>
-      <c r="F965" t="inlineStr"/>
       <c r="G965" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22058,9 +22028,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D966" t="inlineStr"/>
-      <c r="E966" t="inlineStr"/>
-      <c r="F966" t="inlineStr"/>
       <c r="G966" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22083,9 +22050,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D967" t="inlineStr"/>
-      <c r="E967" t="inlineStr"/>
-      <c r="F967" t="inlineStr"/>
       <c r="G967" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22108,9 +22072,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D968" t="inlineStr"/>
-      <c r="E968" t="inlineStr"/>
-      <c r="F968" t="inlineStr"/>
       <c r="G968" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22133,9 +22094,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D969" t="inlineStr"/>
-      <c r="E969" t="inlineStr"/>
-      <c r="F969" t="inlineStr"/>
       <c r="G969" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22158,10 +22116,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D970" t="inlineStr"/>
-      <c r="E970" t="inlineStr"/>
-      <c r="F970" t="inlineStr"/>
       <c r="G970" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="971">
+      <c r="A971" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B971" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C971" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D971" t="inlineStr"/>
+      <c r="E971" t="inlineStr"/>
+      <c r="F971" t="inlineStr"/>
+      <c r="G971" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="972">
+      <c r="A972" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B972" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C972" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D972" t="inlineStr"/>
+      <c r="E972" t="inlineStr"/>
+      <c r="F972" t="inlineStr"/>
+      <c r="G972" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="973">
+      <c r="A973" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B973" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C973" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D973" t="inlineStr"/>
+      <c r="E973" t="inlineStr"/>
+      <c r="F973" t="inlineStr"/>
+      <c r="G973" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="974">
+      <c r="A974" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B974" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C974" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D974" t="inlineStr"/>
+      <c r="E974" t="inlineStr"/>
+      <c r="F974" t="inlineStr"/>
+      <c r="G974" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="975">
+      <c r="A975" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B975" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C975" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D975" t="inlineStr"/>
+      <c r="E975" t="inlineStr"/>
+      <c r="F975" t="inlineStr"/>
+      <c r="G975" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="976">
+      <c r="A976" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B976" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C976" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D976" t="inlineStr"/>
+      <c r="E976" t="inlineStr"/>
+      <c r="F976" t="inlineStr"/>
+      <c r="G976" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="977">
+      <c r="A977" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B977" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C977" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D977" t="inlineStr"/>
+      <c r="E977" t="inlineStr"/>
+      <c r="F977" t="inlineStr"/>
+      <c r="G977" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="978">
+      <c r="A978" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B978" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C978" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D978" t="inlineStr"/>
+      <c r="E978" t="inlineStr"/>
+      <c r="F978" t="inlineStr"/>
+      <c r="G978" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="979">
+      <c r="A979" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B979" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C979" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D979" t="inlineStr"/>
+      <c r="E979" t="inlineStr"/>
+      <c r="F979" t="inlineStr"/>
+      <c r="G979" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="980">
+      <c r="A980" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B980" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C980" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D980" t="inlineStr"/>
+      <c r="E980" t="inlineStr"/>
+      <c r="F980" t="inlineStr"/>
+      <c r="G980" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="981">
+      <c r="A981" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B981" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C981" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D981" t="inlineStr"/>
+      <c r="E981" t="inlineStr"/>
+      <c r="F981" t="inlineStr"/>
+      <c r="G981" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="982">
+      <c r="A982" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B982" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C982" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D982" t="inlineStr"/>
+      <c r="E982" t="inlineStr"/>
+      <c r="F982" t="inlineStr"/>
+      <c r="G982" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="983">
+      <c r="A983" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B983" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C983" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D983" t="inlineStr"/>
+      <c r="E983" t="inlineStr"/>
+      <c r="F983" t="inlineStr"/>
+      <c r="G983" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="984">
+      <c r="A984" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B984" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C984" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D984" t="inlineStr"/>
+      <c r="E984" t="inlineStr"/>
+      <c r="F984" t="inlineStr"/>
+      <c r="G984" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="985">
+      <c r="A985" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B985" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C985" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D985" t="inlineStr"/>
+      <c r="E985" t="inlineStr"/>
+      <c r="F985" t="inlineStr"/>
+      <c r="G985" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-10-21
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G985"/>
+  <dimension ref="A1:G1000"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22138,9 +22138,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D971" t="inlineStr"/>
-      <c r="E971" t="inlineStr"/>
-      <c r="F971" t="inlineStr"/>
       <c r="G971" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22163,9 +22160,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D972" t="inlineStr"/>
-      <c r="E972" t="inlineStr"/>
-      <c r="F972" t="inlineStr"/>
       <c r="G972" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22188,9 +22182,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D973" t="inlineStr"/>
-      <c r="E973" t="inlineStr"/>
-      <c r="F973" t="inlineStr"/>
       <c r="G973" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22213,9 +22204,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D974" t="inlineStr"/>
-      <c r="E974" t="inlineStr"/>
-      <c r="F974" t="inlineStr"/>
       <c r="G974" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22238,9 +22226,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D975" t="inlineStr"/>
-      <c r="E975" t="inlineStr"/>
-      <c r="F975" t="inlineStr"/>
       <c r="G975" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22263,9 +22248,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D976" t="inlineStr"/>
-      <c r="E976" t="inlineStr"/>
-      <c r="F976" t="inlineStr"/>
       <c r="G976" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22288,9 +22270,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D977" t="inlineStr"/>
-      <c r="E977" t="inlineStr"/>
-      <c r="F977" t="inlineStr"/>
       <c r="G977" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22313,9 +22292,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D978" t="inlineStr"/>
-      <c r="E978" t="inlineStr"/>
-      <c r="F978" t="inlineStr"/>
       <c r="G978" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22338,9 +22314,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D979" t="inlineStr"/>
-      <c r="E979" t="inlineStr"/>
-      <c r="F979" t="inlineStr"/>
       <c r="G979" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22363,9 +22336,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D980" t="inlineStr"/>
-      <c r="E980" t="inlineStr"/>
-      <c r="F980" t="inlineStr"/>
       <c r="G980" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22388,9 +22358,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D981" t="inlineStr"/>
-      <c r="E981" t="inlineStr"/>
-      <c r="F981" t="inlineStr"/>
       <c r="G981" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22413,9 +22380,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D982" t="inlineStr"/>
-      <c r="E982" t="inlineStr"/>
-      <c r="F982" t="inlineStr"/>
       <c r="G982" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22438,9 +22402,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D983" t="inlineStr"/>
-      <c r="E983" t="inlineStr"/>
-      <c r="F983" t="inlineStr"/>
       <c r="G983" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22463,9 +22424,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D984" t="inlineStr"/>
-      <c r="E984" t="inlineStr"/>
-      <c r="F984" t="inlineStr"/>
       <c r="G984" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22488,10 +22446,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D985" t="inlineStr"/>
-      <c r="E985" t="inlineStr"/>
-      <c r="F985" t="inlineStr"/>
       <c r="G985" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="986">
+      <c r="A986" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B986" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C986" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D986" t="inlineStr"/>
+      <c r="E986" t="inlineStr"/>
+      <c r="F986" t="inlineStr"/>
+      <c r="G986" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="987">
+      <c r="A987" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B987" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C987" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D987" t="inlineStr"/>
+      <c r="E987" t="inlineStr"/>
+      <c r="F987" t="inlineStr"/>
+      <c r="G987" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="988">
+      <c r="A988" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B988" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C988" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D988" t="inlineStr"/>
+      <c r="E988" t="inlineStr"/>
+      <c r="F988" t="inlineStr"/>
+      <c r="G988" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="989">
+      <c r="A989" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B989" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C989" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D989" t="inlineStr"/>
+      <c r="E989" t="inlineStr"/>
+      <c r="F989" t="inlineStr"/>
+      <c r="G989" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="990">
+      <c r="A990" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B990" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C990" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D990" t="inlineStr"/>
+      <c r="E990" t="inlineStr"/>
+      <c r="F990" t="inlineStr"/>
+      <c r="G990" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="991">
+      <c r="A991" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B991" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C991" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D991" t="inlineStr"/>
+      <c r="E991" t="inlineStr"/>
+      <c r="F991" t="inlineStr"/>
+      <c r="G991" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="992">
+      <c r="A992" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B992" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C992" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D992" t="inlineStr"/>
+      <c r="E992" t="inlineStr"/>
+      <c r="F992" t="inlineStr"/>
+      <c r="G992" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="993">
+      <c r="A993" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B993" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C993" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D993" t="inlineStr"/>
+      <c r="E993" t="inlineStr"/>
+      <c r="F993" t="inlineStr"/>
+      <c r="G993" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="994">
+      <c r="A994" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B994" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C994" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D994" t="inlineStr"/>
+      <c r="E994" t="inlineStr"/>
+      <c r="F994" t="inlineStr"/>
+      <c r="G994" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="995">
+      <c r="A995" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B995" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C995" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D995" t="inlineStr"/>
+      <c r="E995" t="inlineStr"/>
+      <c r="F995" t="inlineStr"/>
+      <c r="G995" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="996">
+      <c r="A996" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B996" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C996" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D996" t="inlineStr"/>
+      <c r="E996" t="inlineStr"/>
+      <c r="F996" t="inlineStr"/>
+      <c r="G996" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="997">
+      <c r="A997" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B997" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C997" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D997" t="inlineStr"/>
+      <c r="E997" t="inlineStr"/>
+      <c r="F997" t="inlineStr"/>
+      <c r="G997" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="998">
+      <c r="A998" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B998" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C998" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D998" t="inlineStr"/>
+      <c r="E998" t="inlineStr"/>
+      <c r="F998" t="inlineStr"/>
+      <c r="G998" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="999">
+      <c r="A999" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B999" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C999" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D999" t="inlineStr"/>
+      <c r="E999" t="inlineStr"/>
+      <c r="F999" t="inlineStr"/>
+      <c r="G999" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1000">
+      <c r="A1000" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B1000" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1000" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D1000" t="inlineStr"/>
+      <c r="E1000" t="inlineStr"/>
+      <c r="F1000" t="inlineStr"/>
+      <c r="G1000" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-10-22
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1000"/>
+  <dimension ref="A1:G1015"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22468,9 +22468,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D986" t="inlineStr"/>
-      <c r="E986" t="inlineStr"/>
-      <c r="F986" t="inlineStr"/>
       <c r="G986" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22493,9 +22490,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D987" t="inlineStr"/>
-      <c r="E987" t="inlineStr"/>
-      <c r="F987" t="inlineStr"/>
       <c r="G987" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22518,9 +22512,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D988" t="inlineStr"/>
-      <c r="E988" t="inlineStr"/>
-      <c r="F988" t="inlineStr"/>
       <c r="G988" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22543,9 +22534,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D989" t="inlineStr"/>
-      <c r="E989" t="inlineStr"/>
-      <c r="F989" t="inlineStr"/>
       <c r="G989" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22568,9 +22556,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D990" t="inlineStr"/>
-      <c r="E990" t="inlineStr"/>
-      <c r="F990" t="inlineStr"/>
       <c r="G990" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22593,9 +22578,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D991" t="inlineStr"/>
-      <c r="E991" t="inlineStr"/>
-      <c r="F991" t="inlineStr"/>
       <c r="G991" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22618,9 +22600,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D992" t="inlineStr"/>
-      <c r="E992" t="inlineStr"/>
-      <c r="F992" t="inlineStr"/>
       <c r="G992" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22643,9 +22622,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D993" t="inlineStr"/>
-      <c r="E993" t="inlineStr"/>
-      <c r="F993" t="inlineStr"/>
       <c r="G993" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22668,9 +22644,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D994" t="inlineStr"/>
-      <c r="E994" t="inlineStr"/>
-      <c r="F994" t="inlineStr"/>
       <c r="G994" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22693,9 +22666,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D995" t="inlineStr"/>
-      <c r="E995" t="inlineStr"/>
-      <c r="F995" t="inlineStr"/>
       <c r="G995" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22718,9 +22688,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D996" t="inlineStr"/>
-      <c r="E996" t="inlineStr"/>
-      <c r="F996" t="inlineStr"/>
       <c r="G996" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22743,9 +22710,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D997" t="inlineStr"/>
-      <c r="E997" t="inlineStr"/>
-      <c r="F997" t="inlineStr"/>
       <c r="G997" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22768,9 +22732,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D998" t="inlineStr"/>
-      <c r="E998" t="inlineStr"/>
-      <c r="F998" t="inlineStr"/>
       <c r="G998" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22793,9 +22754,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D999" t="inlineStr"/>
-      <c r="E999" t="inlineStr"/>
-      <c r="F999" t="inlineStr"/>
       <c r="G999" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22818,10 +22776,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D1000" t="inlineStr"/>
-      <c r="E1000" t="inlineStr"/>
-      <c r="F1000" t="inlineStr"/>
       <c r="G1000" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1001">
+      <c r="A1001" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B1001" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1001" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D1001" t="inlineStr"/>
+      <c r="E1001" t="inlineStr"/>
+      <c r="F1001" t="inlineStr"/>
+      <c r="G1001" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1002">
+      <c r="A1002" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B1002" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1002" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D1002" t="inlineStr"/>
+      <c r="E1002" t="inlineStr"/>
+      <c r="F1002" t="inlineStr"/>
+      <c r="G1002" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B1003" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1003" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D1003" t="inlineStr"/>
+      <c r="E1003" t="inlineStr"/>
+      <c r="F1003" t="inlineStr"/>
+      <c r="G1003" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1004">
+      <c r="A1004" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B1004" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1004" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D1004" t="inlineStr"/>
+      <c r="E1004" t="inlineStr"/>
+      <c r="F1004" t="inlineStr"/>
+      <c r="G1004" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1005">
+      <c r="A1005" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B1005" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1005" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D1005" t="inlineStr"/>
+      <c r="E1005" t="inlineStr"/>
+      <c r="F1005" t="inlineStr"/>
+      <c r="G1005" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1006">
+      <c r="A1006" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B1006" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1006" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D1006" t="inlineStr"/>
+      <c r="E1006" t="inlineStr"/>
+      <c r="F1006" t="inlineStr"/>
+      <c r="G1006" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1007">
+      <c r="A1007" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B1007" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1007" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D1007" t="inlineStr"/>
+      <c r="E1007" t="inlineStr"/>
+      <c r="F1007" t="inlineStr"/>
+      <c r="G1007" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1008">
+      <c r="A1008" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B1008" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1008" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D1008" t="inlineStr"/>
+      <c r="E1008" t="inlineStr"/>
+      <c r="F1008" t="inlineStr"/>
+      <c r="G1008" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B1009" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1009" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D1009" t="inlineStr"/>
+      <c r="E1009" t="inlineStr"/>
+      <c r="F1009" t="inlineStr"/>
+      <c r="G1009" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1010">
+      <c r="A1010" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B1010" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1010" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D1010" t="inlineStr"/>
+      <c r="E1010" t="inlineStr"/>
+      <c r="F1010" t="inlineStr"/>
+      <c r="G1010" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1011">
+      <c r="A1011" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B1011" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1011" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D1011" t="inlineStr"/>
+      <c r="E1011" t="inlineStr"/>
+      <c r="F1011" t="inlineStr"/>
+      <c r="G1011" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1012">
+      <c r="A1012" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B1012" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1012" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D1012" t="inlineStr"/>
+      <c r="E1012" t="inlineStr"/>
+      <c r="F1012" t="inlineStr"/>
+      <c r="G1012" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B1013" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1013" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D1013" t="inlineStr"/>
+      <c r="E1013" t="inlineStr"/>
+      <c r="F1013" t="inlineStr"/>
+      <c r="G1013" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B1014" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1014" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D1014" t="inlineStr"/>
+      <c r="E1014" t="inlineStr"/>
+      <c r="F1014" t="inlineStr"/>
+      <c r="G1014" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1015">
+      <c r="A1015" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B1015" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1015" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D1015" t="inlineStr"/>
+      <c r="E1015" t="inlineStr"/>
+      <c r="F1015" t="inlineStr"/>
+      <c r="G1015" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-10-23
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1015"/>
+  <dimension ref="A1:G1030"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22798,9 +22798,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D1001" t="inlineStr"/>
-      <c r="E1001" t="inlineStr"/>
-      <c r="F1001" t="inlineStr"/>
       <c r="G1001" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22823,9 +22820,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D1002" t="inlineStr"/>
-      <c r="E1002" t="inlineStr"/>
-      <c r="F1002" t="inlineStr"/>
       <c r="G1002" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22848,9 +22842,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D1003" t="inlineStr"/>
-      <c r="E1003" t="inlineStr"/>
-      <c r="F1003" t="inlineStr"/>
       <c r="G1003" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22873,9 +22864,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D1004" t="inlineStr"/>
-      <c r="E1004" t="inlineStr"/>
-      <c r="F1004" t="inlineStr"/>
       <c r="G1004" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22898,9 +22886,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D1005" t="inlineStr"/>
-      <c r="E1005" t="inlineStr"/>
-      <c r="F1005" t="inlineStr"/>
       <c r="G1005" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22923,9 +22908,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D1006" t="inlineStr"/>
-      <c r="E1006" t="inlineStr"/>
-      <c r="F1006" t="inlineStr"/>
       <c r="G1006" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22948,9 +22930,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D1007" t="inlineStr"/>
-      <c r="E1007" t="inlineStr"/>
-      <c r="F1007" t="inlineStr"/>
       <c r="G1007" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22973,9 +22952,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D1008" t="inlineStr"/>
-      <c r="E1008" t="inlineStr"/>
-      <c r="F1008" t="inlineStr"/>
       <c r="G1008" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -22998,9 +22974,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D1009" t="inlineStr"/>
-      <c r="E1009" t="inlineStr"/>
-      <c r="F1009" t="inlineStr"/>
       <c r="G1009" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -23023,9 +22996,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D1010" t="inlineStr"/>
-      <c r="E1010" t="inlineStr"/>
-      <c r="F1010" t="inlineStr"/>
       <c r="G1010" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -23048,9 +23018,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D1011" t="inlineStr"/>
-      <c r="E1011" t="inlineStr"/>
-      <c r="F1011" t="inlineStr"/>
       <c r="G1011" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -23073,9 +23040,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D1012" t="inlineStr"/>
-      <c r="E1012" t="inlineStr"/>
-      <c r="F1012" t="inlineStr"/>
       <c r="G1012" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -23098,9 +23062,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D1013" t="inlineStr"/>
-      <c r="E1013" t="inlineStr"/>
-      <c r="F1013" t="inlineStr"/>
       <c r="G1013" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -23123,9 +23084,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D1014" t="inlineStr"/>
-      <c r="E1014" t="inlineStr"/>
-      <c r="F1014" t="inlineStr"/>
       <c r="G1014" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -23148,10 +23106,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D1015" t="inlineStr"/>
-      <c r="E1015" t="inlineStr"/>
-      <c r="F1015" t="inlineStr"/>
       <c r="G1015" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1016">
+      <c r="A1016" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1016" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1016" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D1016" t="inlineStr"/>
+      <c r="E1016" t="inlineStr"/>
+      <c r="F1016" t="inlineStr"/>
+      <c r="G1016" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1017">
+      <c r="A1017" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1017" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1017" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D1017" t="inlineStr"/>
+      <c r="E1017" t="inlineStr"/>
+      <c r="F1017" t="inlineStr"/>
+      <c r="G1017" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1018">
+      <c r="A1018" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1018" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1018" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D1018" t="inlineStr"/>
+      <c r="E1018" t="inlineStr"/>
+      <c r="F1018" t="inlineStr"/>
+      <c r="G1018" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1019">
+      <c r="A1019" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1019" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1019" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D1019" t="inlineStr"/>
+      <c r="E1019" t="inlineStr"/>
+      <c r="F1019" t="inlineStr"/>
+      <c r="G1019" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1020">
+      <c r="A1020" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1020" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1020" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D1020" t="inlineStr"/>
+      <c r="E1020" t="inlineStr"/>
+      <c r="F1020" t="inlineStr"/>
+      <c r="G1020" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1021">
+      <c r="A1021" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1021" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1021" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D1021" t="inlineStr"/>
+      <c r="E1021" t="inlineStr"/>
+      <c r="F1021" t="inlineStr"/>
+      <c r="G1021" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1022">
+      <c r="A1022" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1022" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1022" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D1022" t="inlineStr"/>
+      <c r="E1022" t="inlineStr"/>
+      <c r="F1022" t="inlineStr"/>
+      <c r="G1022" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1023">
+      <c r="A1023" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1023" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1023" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D1023" t="inlineStr"/>
+      <c r="E1023" t="inlineStr"/>
+      <c r="F1023" t="inlineStr"/>
+      <c r="G1023" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1024">
+      <c r="A1024" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1024" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1024" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D1024" t="inlineStr"/>
+      <c r="E1024" t="inlineStr"/>
+      <c r="F1024" t="inlineStr"/>
+      <c r="G1024" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1025">
+      <c r="A1025" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1025" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1025" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D1025" t="inlineStr"/>
+      <c r="E1025" t="inlineStr"/>
+      <c r="F1025" t="inlineStr"/>
+      <c r="G1025" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1026">
+      <c r="A1026" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1026" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1026" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D1026" t="inlineStr"/>
+      <c r="E1026" t="inlineStr"/>
+      <c r="F1026" t="inlineStr"/>
+      <c r="G1026" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1027">
+      <c r="A1027" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1027" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1027" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D1027" t="inlineStr"/>
+      <c r="E1027" t="inlineStr"/>
+      <c r="F1027" t="inlineStr"/>
+      <c r="G1027" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1028">
+      <c r="A1028" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1028" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1028" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D1028" t="inlineStr"/>
+      <c r="E1028" t="inlineStr"/>
+      <c r="F1028" t="inlineStr"/>
+      <c r="G1028" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1029">
+      <c r="A1029" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1029" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1029" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D1029" t="inlineStr"/>
+      <c r="E1029" t="inlineStr"/>
+      <c r="F1029" t="inlineStr"/>
+      <c r="G1029" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1030">
+      <c r="A1030" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1030" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1030" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D1030" t="inlineStr"/>
+      <c r="E1030" t="inlineStr"/>
+      <c r="F1030" t="inlineStr"/>
+      <c r="G1030" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-10-24
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1030"/>
+  <dimension ref="A1:G1052"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23128,9 +23128,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D1016" t="inlineStr"/>
-      <c r="E1016" t="inlineStr"/>
-      <c r="F1016" t="inlineStr"/>
       <c r="G1016" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -23153,9 +23150,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D1017" t="inlineStr"/>
-      <c r="E1017" t="inlineStr"/>
-      <c r="F1017" t="inlineStr"/>
       <c r="G1017" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -23178,9 +23172,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D1018" t="inlineStr"/>
-      <c r="E1018" t="inlineStr"/>
-      <c r="F1018" t="inlineStr"/>
       <c r="G1018" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -23203,9 +23194,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D1019" t="inlineStr"/>
-      <c r="E1019" t="inlineStr"/>
-      <c r="F1019" t="inlineStr"/>
       <c r="G1019" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -23228,9 +23216,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D1020" t="inlineStr"/>
-      <c r="E1020" t="inlineStr"/>
-      <c r="F1020" t="inlineStr"/>
       <c r="G1020" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -23253,9 +23238,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D1021" t="inlineStr"/>
-      <c r="E1021" t="inlineStr"/>
-      <c r="F1021" t="inlineStr"/>
       <c r="G1021" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -23278,9 +23260,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D1022" t="inlineStr"/>
-      <c r="E1022" t="inlineStr"/>
-      <c r="F1022" t="inlineStr"/>
       <c r="G1022" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -23303,9 +23282,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D1023" t="inlineStr"/>
-      <c r="E1023" t="inlineStr"/>
-      <c r="F1023" t="inlineStr"/>
       <c r="G1023" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -23328,9 +23304,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D1024" t="inlineStr"/>
-      <c r="E1024" t="inlineStr"/>
-      <c r="F1024" t="inlineStr"/>
       <c r="G1024" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -23353,9 +23326,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D1025" t="inlineStr"/>
-      <c r="E1025" t="inlineStr"/>
-      <c r="F1025" t="inlineStr"/>
       <c r="G1025" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -23378,9 +23348,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D1026" t="inlineStr"/>
-      <c r="E1026" t="inlineStr"/>
-      <c r="F1026" t="inlineStr"/>
       <c r="G1026" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -23403,9 +23370,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D1027" t="inlineStr"/>
-      <c r="E1027" t="inlineStr"/>
-      <c r="F1027" t="inlineStr"/>
       <c r="G1027" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -23428,9 +23392,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D1028" t="inlineStr"/>
-      <c r="E1028" t="inlineStr"/>
-      <c r="F1028" t="inlineStr"/>
       <c r="G1028" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -23453,9 +23414,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D1029" t="inlineStr"/>
-      <c r="E1029" t="inlineStr"/>
-      <c r="F1029" t="inlineStr"/>
       <c r="G1029" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -23478,14 +23436,571 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D1030" t="inlineStr"/>
-      <c r="E1030" t="inlineStr"/>
-      <c r="F1030" t="inlineStr"/>
       <c r="G1030" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>
       </c>
+    </row>
+    <row r="1031">
+      <c r="A1031" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B1031" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1031" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D1031" t="inlineStr"/>
+      <c r="E1031" t="inlineStr"/>
+      <c r="F1031" t="inlineStr"/>
+      <c r="G1031" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1032">
+      <c r="A1032" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B1032" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1032" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D1032" t="inlineStr"/>
+      <c r="E1032" t="inlineStr"/>
+      <c r="F1032" t="inlineStr"/>
+      <c r="G1032" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1033">
+      <c r="A1033" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B1033" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1033" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D1033" t="inlineStr"/>
+      <c r="E1033" t="inlineStr"/>
+      <c r="F1033" t="inlineStr"/>
+      <c r="G1033" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1034">
+      <c r="A1034" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B1034" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1034" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D1034" t="inlineStr"/>
+      <c r="E1034" t="inlineStr"/>
+      <c r="F1034" t="inlineStr"/>
+      <c r="G1034" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1035">
+      <c r="A1035" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B1035" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1035" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1035" t="n">
+        <v>2131</v>
+      </c>
+      <c r="F1035" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Duplex-litros-Branca/dp/B07FXZ8TR6/ref=sr_1_1</t>
+        </is>
+      </c>
+      <c r="G1035" t="inlineStr"/>
+    </row>
+    <row r="1036">
+      <c r="A1036" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B1036" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1036" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1036" t="n">
+        <v>2564.05</v>
+      </c>
+      <c r="F1036" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Litros-Duplex-Branca/dp/B0GFB8M9MZ/ref=sr_1_2</t>
+        </is>
+      </c>
+      <c r="G1036" t="inlineStr"/>
+    </row>
+    <row r="1037">
+      <c r="A1037" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B1037" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1037" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1037" t="n">
+        <v>3199</v>
+      </c>
+      <c r="F1037" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWVJ8LR/ref=sr_1_3</t>
+        </is>
+      </c>
+      <c r="G1037" t="inlineStr"/>
+    </row>
+    <row r="1038">
+      <c r="A1038" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B1038" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1038" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D1038" t="inlineStr"/>
+      <c r="E1038" t="inlineStr"/>
+      <c r="F1038" t="inlineStr"/>
+      <c r="G1038" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1039">
+      <c r="A1039" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B1039" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1039" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D1039" t="inlineStr"/>
+      <c r="E1039" t="inlineStr"/>
+      <c r="F1039" t="inlineStr"/>
+      <c r="G1039" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1040">
+      <c r="A1040" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B1040" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1040" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D1040" t="inlineStr"/>
+      <c r="E1040" t="inlineStr"/>
+      <c r="F1040" t="inlineStr"/>
+      <c r="G1040" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='api.scraperapi.com', port=443): Read timed out. (read timeout=60)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1041">
+      <c r="A1041" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B1041" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1041" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D1041" t="inlineStr"/>
+      <c r="E1041" t="inlineStr"/>
+      <c r="F1041" t="inlineStr"/>
+      <c r="G1041" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1042">
+      <c r="A1042" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B1042" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1042" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1042" t="n">
+        <v>509</v>
+      </c>
+      <c r="F1042" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P2FLSR/ref=sr_1_5</t>
+        </is>
+      </c>
+      <c r="G1042" t="inlineStr"/>
+    </row>
+    <row r="1043">
+      <c r="A1043" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B1043" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1043" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1043" t="n">
+        <v>496.22</v>
+      </c>
+      <c r="F1043" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Efficient-23L-ME23B/dp/B0B8KWNK12/ref=sr_1_6</t>
+        </is>
+      </c>
+      <c r="G1043" t="inlineStr"/>
+    </row>
+    <row r="1044">
+      <c r="A1044" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B1044" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1044" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1044" t="n">
+        <v>518.99</v>
+      </c>
+      <c r="F1044" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P3T3VM/ref=sr_1_7</t>
+        </is>
+      </c>
+      <c r="G1044" t="inlineStr"/>
+    </row>
+    <row r="1045">
+      <c r="A1045" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B1045" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1045" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D1045" t="inlineStr"/>
+      <c r="E1045" t="inlineStr"/>
+      <c r="F1045" t="inlineStr"/>
+      <c r="G1045" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1046">
+      <c r="A1046" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B1046" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1046" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D1046" t="inlineStr"/>
+      <c r="E1046" t="inlineStr"/>
+      <c r="F1046" t="inlineStr"/>
+      <c r="G1046" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1047">
+      <c r="A1047" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B1047" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1047" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D1047" t="inlineStr"/>
+      <c r="E1047" t="inlineStr"/>
+      <c r="F1047" t="inlineStr"/>
+      <c r="G1047" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1048">
+      <c r="A1048" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B1048" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1048" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="E1048" t="n">
+        <v>1058.99</v>
+      </c>
+      <c r="F1048" t="inlineStr">
+        <is>
+          <t>https://www.magazineluiza.com.br/fogao-4-bocas-consul-inox-cfo4naruna/p/214469000/ed/fg4b/</t>
+        </is>
+      </c>
+      <c r="G1048" t="inlineStr"/>
+    </row>
+    <row r="1049">
+      <c r="A1049" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B1049" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1049" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D1049" t="inlineStr"/>
+      <c r="E1049" t="inlineStr"/>
+      <c r="F1049" t="inlineStr"/>
+      <c r="G1049" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1050">
+      <c r="A1050" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B1050" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1050" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1050" t="n">
+        <v>1325</v>
+      </c>
+      <c r="F1050" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-Consul-Bocas-CFO4NARUNA-Bivolt/dp/B07HM9JL5K/ref=sr_1_1</t>
+        </is>
+      </c>
+      <c r="G1050" t="inlineStr"/>
+    </row>
+    <row r="1051">
+      <c r="A1051" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B1051" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1051" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1051" t="n">
+        <v>1114.73</v>
+      </c>
+      <c r="F1051" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-Bocas-Consul-Vidro-Bivolt/dp/B076BC7769/ref=sr_1_2</t>
+        </is>
+      </c>
+      <c r="G1051" t="inlineStr"/>
+    </row>
+    <row r="1052">
+      <c r="A1052" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B1052" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1052" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1052" t="n">
+        <v>1044.9</v>
+      </c>
+      <c r="F1052" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-04-Bocas-FS-CF04NABUNA/dp/B07JPZN51P/ref=sr_1_3</t>
+        </is>
+      </c>
+      <c r="G1052" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Atualiza preços de 2026-10-25
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1052"/>
+  <dimension ref="A1:G1073"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23458,9 +23458,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D1031" t="inlineStr"/>
-      <c r="E1031" t="inlineStr"/>
-      <c r="F1031" t="inlineStr"/>
       <c r="G1031" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -23483,9 +23480,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D1032" t="inlineStr"/>
-      <c r="E1032" t="inlineStr"/>
-      <c r="F1032" t="inlineStr"/>
       <c r="G1032" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -23508,9 +23502,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D1033" t="inlineStr"/>
-      <c r="E1033" t="inlineStr"/>
-      <c r="F1033" t="inlineStr"/>
       <c r="G1033" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -23533,9 +23524,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D1034" t="inlineStr"/>
-      <c r="E1034" t="inlineStr"/>
-      <c r="F1034" t="inlineStr"/>
       <c r="G1034" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -23566,7 +23554,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Duplex-litros-Branca/dp/B07FXZ8TR6/ref=sr_1_1</t>
         </is>
       </c>
-      <c r="G1035" t="inlineStr"/>
     </row>
     <row r="1036">
       <c r="A1036" t="inlineStr">
@@ -23592,7 +23579,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Litros-Duplex-Branca/dp/B0GFB8M9MZ/ref=sr_1_2</t>
         </is>
       </c>
-      <c r="G1036" t="inlineStr"/>
     </row>
     <row r="1037">
       <c r="A1037" t="inlineStr">
@@ -23618,7 +23604,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWVJ8LR/ref=sr_1_3</t>
         </is>
       </c>
-      <c r="G1037" t="inlineStr"/>
     </row>
     <row r="1038">
       <c r="A1038" t="inlineStr">
@@ -23636,9 +23621,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D1038" t="inlineStr"/>
-      <c r="E1038" t="inlineStr"/>
-      <c r="F1038" t="inlineStr"/>
       <c r="G1038" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -23661,9 +23643,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D1039" t="inlineStr"/>
-      <c r="E1039" t="inlineStr"/>
-      <c r="F1039" t="inlineStr"/>
       <c r="G1039" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -23686,9 +23665,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D1040" t="inlineStr"/>
-      <c r="E1040" t="inlineStr"/>
-      <c r="F1040" t="inlineStr"/>
       <c r="G1040" t="inlineStr">
         <is>
           <t>HTTPSConnectionPool(host='api.scraperapi.com', port=443): Read timed out. (read timeout=60)</t>
@@ -23711,9 +23687,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D1041" t="inlineStr"/>
-      <c r="E1041" t="inlineStr"/>
-      <c r="F1041" t="inlineStr"/>
       <c r="G1041" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -23744,7 +23717,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P2FLSR/ref=sr_1_5</t>
         </is>
       </c>
-      <c r="G1042" t="inlineStr"/>
     </row>
     <row r="1043">
       <c r="A1043" t="inlineStr">
@@ -23770,7 +23742,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Efficient-23L-ME23B/dp/B0B8KWNK12/ref=sr_1_6</t>
         </is>
       </c>
-      <c r="G1043" t="inlineStr"/>
     </row>
     <row r="1044">
       <c r="A1044" t="inlineStr">
@@ -23796,7 +23767,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P3T3VM/ref=sr_1_7</t>
         </is>
       </c>
-      <c r="G1044" t="inlineStr"/>
     </row>
     <row r="1045">
       <c r="A1045" t="inlineStr">
@@ -23814,9 +23784,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D1045" t="inlineStr"/>
-      <c r="E1045" t="inlineStr"/>
-      <c r="F1045" t="inlineStr"/>
       <c r="G1045" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -23839,9 +23806,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D1046" t="inlineStr"/>
-      <c r="E1046" t="inlineStr"/>
-      <c r="F1046" t="inlineStr"/>
       <c r="G1046" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -23864,9 +23828,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D1047" t="inlineStr"/>
-      <c r="E1047" t="inlineStr"/>
-      <c r="F1047" t="inlineStr"/>
       <c r="G1047" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -23897,7 +23858,6 @@
           <t>https://www.magazineluiza.com.br/fogao-4-bocas-consul-inox-cfo4naruna/p/214469000/ed/fg4b/</t>
         </is>
       </c>
-      <c r="G1048" t="inlineStr"/>
     </row>
     <row r="1049">
       <c r="A1049" t="inlineStr">
@@ -23915,9 +23875,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D1049" t="inlineStr"/>
-      <c r="E1049" t="inlineStr"/>
-      <c r="F1049" t="inlineStr"/>
       <c r="G1049" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -23948,7 +23905,6 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-Consul-Bocas-CFO4NARUNA-Bivolt/dp/B07HM9JL5K/ref=sr_1_1</t>
         </is>
       </c>
-      <c r="G1050" t="inlineStr"/>
     </row>
     <row r="1051">
       <c r="A1051" t="inlineStr">
@@ -23974,7 +23930,6 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-Bocas-Consul-Vidro-Bivolt/dp/B076BC7769/ref=sr_1_2</t>
         </is>
       </c>
-      <c r="G1051" t="inlineStr"/>
     </row>
     <row r="1052">
       <c r="A1052" t="inlineStr">
@@ -24000,7 +23955,540 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-04-Bocas-FS-CF04NABUNA/dp/B07JPZN51P/ref=sr_1_3</t>
         </is>
       </c>
-      <c r="G1052" t="inlineStr"/>
+    </row>
+    <row r="1053">
+      <c r="A1053" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B1053" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1053" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D1053" t="inlineStr"/>
+      <c r="E1053" t="inlineStr"/>
+      <c r="F1053" t="inlineStr"/>
+      <c r="G1053" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1054">
+      <c r="A1054" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B1054" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1054" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D1054" t="inlineStr"/>
+      <c r="E1054" t="inlineStr"/>
+      <c r="F1054" t="inlineStr"/>
+      <c r="G1054" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1055">
+      <c r="A1055" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B1055" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1055" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D1055" t="inlineStr"/>
+      <c r="E1055" t="inlineStr"/>
+      <c r="F1055" t="inlineStr"/>
+      <c r="G1055" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1056">
+      <c r="A1056" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B1056" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1056" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D1056" t="inlineStr"/>
+      <c r="E1056" t="inlineStr"/>
+      <c r="F1056" t="inlineStr"/>
+      <c r="G1056" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1057">
+      <c r="A1057" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B1057" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1057" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1057" t="n">
+        <v>2131</v>
+      </c>
+      <c r="F1057" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Duplex-litros-Branca/dp/B07FXZ8TR6/ref=sr_1_5</t>
+        </is>
+      </c>
+      <c r="G1057" t="inlineStr"/>
+    </row>
+    <row r="1058">
+      <c r="A1058" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B1058" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1058" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1058" t="n">
+        <v>2389.59</v>
+      </c>
+      <c r="F1058" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Litros-Duplex-Branca/dp/B0GFB8M9MZ/ref=sr_1_6</t>
+        </is>
+      </c>
+      <c r="G1058" t="inlineStr"/>
+    </row>
+    <row r="1059">
+      <c r="A1059" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B1059" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1059" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1059" t="n">
+        <v>3599.1</v>
+      </c>
+      <c r="F1059" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWVJ8LR/ref=sr_1_7</t>
+        </is>
+      </c>
+      <c r="G1059" t="inlineStr"/>
+    </row>
+    <row r="1060">
+      <c r="A1060" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B1060" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1060" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D1060" t="inlineStr"/>
+      <c r="E1060" t="inlineStr"/>
+      <c r="F1060" t="inlineStr"/>
+      <c r="G1060" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1061">
+      <c r="A1061" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B1061" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1061" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D1061" t="inlineStr"/>
+      <c r="E1061" t="inlineStr"/>
+      <c r="F1061" t="inlineStr"/>
+      <c r="G1061" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1062">
+      <c r="A1062" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B1062" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1062" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D1062" t="inlineStr"/>
+      <c r="E1062" t="inlineStr"/>
+      <c r="F1062" t="inlineStr"/>
+      <c r="G1062" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1063">
+      <c r="A1063" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B1063" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1063" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D1063" t="inlineStr"/>
+      <c r="E1063" t="inlineStr"/>
+      <c r="F1063" t="inlineStr"/>
+      <c r="G1063" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1064">
+      <c r="A1064" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B1064" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1064" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1064" t="n">
+        <v>448.99</v>
+      </c>
+      <c r="F1064" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P2FLSR/ref=sr_1_5</t>
+        </is>
+      </c>
+      <c r="G1064" t="inlineStr"/>
+    </row>
+    <row r="1065">
+      <c r="A1065" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B1065" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1065" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1065" t="n">
+        <v>496.22</v>
+      </c>
+      <c r="F1065" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Efficient-23L-ME23B/dp/B0B8KWNK12/ref=sr_1_6</t>
+        </is>
+      </c>
+      <c r="G1065" t="inlineStr"/>
+    </row>
+    <row r="1066">
+      <c r="A1066" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B1066" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1066" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1066" t="n">
+        <v>511.58</v>
+      </c>
+      <c r="F1066" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Electrolux-MTO30-Fun%C3%A7%C3%A3o-Tira/dp/B083ZFFC5Q/ref=sr_1_7</t>
+        </is>
+      </c>
+      <c r="G1066" t="inlineStr"/>
+    </row>
+    <row r="1067">
+      <c r="A1067" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B1067" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1067" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D1067" t="inlineStr"/>
+      <c r="E1067" t="inlineStr"/>
+      <c r="F1067" t="inlineStr"/>
+      <c r="G1067" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1068">
+      <c r="A1068" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B1068" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1068" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D1068" t="inlineStr"/>
+      <c r="E1068" t="inlineStr"/>
+      <c r="F1068" t="inlineStr"/>
+      <c r="G1068" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1069">
+      <c r="A1069" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B1069" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1069" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D1069" t="inlineStr"/>
+      <c r="E1069" t="inlineStr"/>
+      <c r="F1069" t="inlineStr"/>
+      <c r="G1069" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1070">
+      <c r="A1070" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B1070" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1070" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D1070" t="inlineStr"/>
+      <c r="E1070" t="inlineStr"/>
+      <c r="F1070" t="inlineStr"/>
+      <c r="G1070" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1071">
+      <c r="A1071" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B1071" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1071" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1071" t="n">
+        <v>1003.25</v>
+      </c>
+      <c r="F1071" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-Consul-Bocas-CFO4NARUNA-Bivolt/dp/B07HM9JL5K/ref=sr_1_1</t>
+        </is>
+      </c>
+      <c r="G1071" t="inlineStr"/>
+    </row>
+    <row r="1072">
+      <c r="A1072" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B1072" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1072" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1072" t="n">
+        <v>1259.1</v>
+      </c>
+      <c r="F1072" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-Bocas-Consul-Vidro-Bivolt/dp/B076BC7769/ref=sr_1_2</t>
+        </is>
+      </c>
+      <c r="G1072" t="inlineStr"/>
+    </row>
+    <row r="1073">
+      <c r="A1073" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B1073" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1073" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1073" t="n">
+        <v>1044.9</v>
+      </c>
+      <c r="F1073" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-04-Bocas-FS-CF04NABUNA/dp/B07JPZN51P/ref=sr_1_3</t>
+        </is>
+      </c>
+      <c r="G1073" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Atualiza preços de 2026-10-26
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1073"/>
+  <dimension ref="A1:G1094"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23972,9 +23972,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D1053" t="inlineStr"/>
-      <c r="E1053" t="inlineStr"/>
-      <c r="F1053" t="inlineStr"/>
       <c r="G1053" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -23997,9 +23994,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D1054" t="inlineStr"/>
-      <c r="E1054" t="inlineStr"/>
-      <c r="F1054" t="inlineStr"/>
       <c r="G1054" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -24022,9 +24016,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D1055" t="inlineStr"/>
-      <c r="E1055" t="inlineStr"/>
-      <c r="F1055" t="inlineStr"/>
       <c r="G1055" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -24047,9 +24038,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D1056" t="inlineStr"/>
-      <c r="E1056" t="inlineStr"/>
-      <c r="F1056" t="inlineStr"/>
       <c r="G1056" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -24080,7 +24068,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Duplex-litros-Branca/dp/B07FXZ8TR6/ref=sr_1_5</t>
         </is>
       </c>
-      <c r="G1057" t="inlineStr"/>
     </row>
     <row r="1058">
       <c r="A1058" t="inlineStr">
@@ -24106,7 +24093,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Litros-Duplex-Branca/dp/B0GFB8M9MZ/ref=sr_1_6</t>
         </is>
       </c>
-      <c r="G1058" t="inlineStr"/>
     </row>
     <row r="1059">
       <c r="A1059" t="inlineStr">
@@ -24132,7 +24118,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWVJ8LR/ref=sr_1_7</t>
         </is>
       </c>
-      <c r="G1059" t="inlineStr"/>
     </row>
     <row r="1060">
       <c r="A1060" t="inlineStr">
@@ -24150,9 +24135,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D1060" t="inlineStr"/>
-      <c r="E1060" t="inlineStr"/>
-      <c r="F1060" t="inlineStr"/>
       <c r="G1060" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -24175,9 +24157,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D1061" t="inlineStr"/>
-      <c r="E1061" t="inlineStr"/>
-      <c r="F1061" t="inlineStr"/>
       <c r="G1061" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -24200,9 +24179,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D1062" t="inlineStr"/>
-      <c r="E1062" t="inlineStr"/>
-      <c r="F1062" t="inlineStr"/>
       <c r="G1062" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -24225,9 +24201,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D1063" t="inlineStr"/>
-      <c r="E1063" t="inlineStr"/>
-      <c r="F1063" t="inlineStr"/>
       <c r="G1063" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -24258,7 +24231,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P2FLSR/ref=sr_1_5</t>
         </is>
       </c>
-      <c r="G1064" t="inlineStr"/>
     </row>
     <row r="1065">
       <c r="A1065" t="inlineStr">
@@ -24284,7 +24256,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Efficient-23L-ME23B/dp/B0B8KWNK12/ref=sr_1_6</t>
         </is>
       </c>
-      <c r="G1065" t="inlineStr"/>
     </row>
     <row r="1066">
       <c r="A1066" t="inlineStr">
@@ -24310,7 +24281,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Electrolux-MTO30-Fun%C3%A7%C3%A3o-Tira/dp/B083ZFFC5Q/ref=sr_1_7</t>
         </is>
       </c>
-      <c r="G1066" t="inlineStr"/>
     </row>
     <row r="1067">
       <c r="A1067" t="inlineStr">
@@ -24328,9 +24298,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D1067" t="inlineStr"/>
-      <c r="E1067" t="inlineStr"/>
-      <c r="F1067" t="inlineStr"/>
       <c r="G1067" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -24353,9 +24320,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D1068" t="inlineStr"/>
-      <c r="E1068" t="inlineStr"/>
-      <c r="F1068" t="inlineStr"/>
       <c r="G1068" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -24378,9 +24342,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D1069" t="inlineStr"/>
-      <c r="E1069" t="inlineStr"/>
-      <c r="F1069" t="inlineStr"/>
       <c r="G1069" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -24403,9 +24364,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D1070" t="inlineStr"/>
-      <c r="E1070" t="inlineStr"/>
-      <c r="F1070" t="inlineStr"/>
       <c r="G1070" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -24436,7 +24394,6 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-Consul-Bocas-CFO4NARUNA-Bivolt/dp/B07HM9JL5K/ref=sr_1_1</t>
         </is>
       </c>
-      <c r="G1071" t="inlineStr"/>
     </row>
     <row r="1072">
       <c r="A1072" t="inlineStr">
@@ -24462,7 +24419,6 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-Bocas-Consul-Vidro-Bivolt/dp/B076BC7769/ref=sr_1_2</t>
         </is>
       </c>
-      <c r="G1072" t="inlineStr"/>
     </row>
     <row r="1073">
       <c r="A1073" t="inlineStr">
@@ -24488,7 +24444,540 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-04-Bocas-FS-CF04NABUNA/dp/B07JPZN51P/ref=sr_1_3</t>
         </is>
       </c>
-      <c r="G1073" t="inlineStr"/>
+    </row>
+    <row r="1074">
+      <c r="A1074" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B1074" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1074" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D1074" t="inlineStr"/>
+      <c r="E1074" t="inlineStr"/>
+      <c r="F1074" t="inlineStr"/>
+      <c r="G1074" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1075">
+      <c r="A1075" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B1075" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1075" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D1075" t="inlineStr"/>
+      <c r="E1075" t="inlineStr"/>
+      <c r="F1075" t="inlineStr"/>
+      <c r="G1075" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1076">
+      <c r="A1076" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B1076" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1076" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D1076" t="inlineStr"/>
+      <c r="E1076" t="inlineStr"/>
+      <c r="F1076" t="inlineStr"/>
+      <c r="G1076" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1077">
+      <c r="A1077" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B1077" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1077" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D1077" t="inlineStr"/>
+      <c r="E1077" t="inlineStr"/>
+      <c r="F1077" t="inlineStr"/>
+      <c r="G1077" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1078">
+      <c r="A1078" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B1078" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1078" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1078" t="n">
+        <v>2131</v>
+      </c>
+      <c r="F1078" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Duplex-litros-Branca/dp/B07FXZ8TR6/ref=sr_1_5</t>
+        </is>
+      </c>
+      <c r="G1078" t="inlineStr"/>
+    </row>
+    <row r="1079">
+      <c r="A1079" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B1079" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1079" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1079" t="n">
+        <v>2706.55</v>
+      </c>
+      <c r="F1079" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-BRM46MK-Duplex-Extrafrio-Brastemp/dp/B0GL3Q3PTG/ref=sr_1_6</t>
+        </is>
+      </c>
+      <c r="G1079" t="inlineStr"/>
+    </row>
+    <row r="1080">
+      <c r="A1080" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B1080" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1080" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1080" t="n">
+        <v>1240</v>
+      </c>
+      <c r="F1080" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Refrigerador-Brastemp-Duplex-Litros/dp/B07ND4BB3C/ref=sr_1_7</t>
+        </is>
+      </c>
+      <c r="G1080" t="inlineStr"/>
+    </row>
+    <row r="1081">
+      <c r="A1081" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B1081" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1081" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D1081" t="inlineStr"/>
+      <c r="E1081" t="inlineStr"/>
+      <c r="F1081" t="inlineStr"/>
+      <c r="G1081" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1082">
+      <c r="A1082" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B1082" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1082" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D1082" t="inlineStr"/>
+      <c r="E1082" t="inlineStr"/>
+      <c r="F1082" t="inlineStr"/>
+      <c r="G1082" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1083">
+      <c r="A1083" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B1083" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1083" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D1083" t="inlineStr"/>
+      <c r="E1083" t="inlineStr"/>
+      <c r="F1083" t="inlineStr"/>
+      <c r="G1083" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1084">
+      <c r="A1084" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B1084" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1084" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D1084" t="inlineStr"/>
+      <c r="E1084" t="inlineStr"/>
+      <c r="F1084" t="inlineStr"/>
+      <c r="G1084" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1085">
+      <c r="A1085" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B1085" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1085" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1085" t="n">
+        <v>438.99</v>
+      </c>
+      <c r="F1085" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P2FLSR/ref=sr_1_5_mod_primary_new</t>
+        </is>
+      </c>
+      <c r="G1085" t="inlineStr"/>
+    </row>
+    <row r="1086">
+      <c r="A1086" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B1086" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1086" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1086" t="n">
+        <v>438.99</v>
+      </c>
+      <c r="F1086" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P2FLSR/ref=sr_1_5_mod_new</t>
+        </is>
+      </c>
+      <c r="G1086" t="inlineStr"/>
+    </row>
+    <row r="1087">
+      <c r="A1087" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B1087" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1087" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1087" t="n">
+        <v>384.3</v>
+      </c>
+      <c r="F1087" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P3T3VM/ref=sr_1_6</t>
+        </is>
+      </c>
+      <c r="G1087" t="inlineStr"/>
+    </row>
+    <row r="1088">
+      <c r="A1088" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B1088" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1088" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D1088" t="inlineStr"/>
+      <c r="E1088" t="inlineStr"/>
+      <c r="F1088" t="inlineStr"/>
+      <c r="G1088" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1089">
+      <c r="A1089" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B1089" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1089" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D1089" t="inlineStr"/>
+      <c r="E1089" t="inlineStr"/>
+      <c r="F1089" t="inlineStr"/>
+      <c r="G1089" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1090">
+      <c r="A1090" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B1090" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1090" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D1090" t="inlineStr"/>
+      <c r="E1090" t="inlineStr"/>
+      <c r="F1090" t="inlineStr"/>
+      <c r="G1090" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1091">
+      <c r="A1091" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B1091" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1091" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D1091" t="inlineStr"/>
+      <c r="E1091" t="inlineStr"/>
+      <c r="F1091" t="inlineStr"/>
+      <c r="G1091" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1092">
+      <c r="A1092" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B1092" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1092" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1092" t="n">
+        <v>1003.25</v>
+      </c>
+      <c r="F1092" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-Consul-Bocas-CFO4NARUNA-Bivolt/dp/B07HM9JL5K/ref=sr_1_5</t>
+        </is>
+      </c>
+      <c r="G1092" t="inlineStr"/>
+    </row>
+    <row r="1093">
+      <c r="A1093" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B1093" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1093" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1093" t="n">
+        <v>1114.73</v>
+      </c>
+      <c r="F1093" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-Bocas-Consul-Vidro-Bivolt/dp/B076BC7769/ref=sr_1_6</t>
+        </is>
+      </c>
+      <c r="G1093" t="inlineStr"/>
+    </row>
+    <row r="1094">
+      <c r="A1094" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B1094" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1094" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1094" t="n">
+        <v>1044.9</v>
+      </c>
+      <c r="F1094" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-04-Bocas-FS-CF04NABUNA/dp/B07JPZN51P/ref=sr_1_7</t>
+        </is>
+      </c>
+      <c r="G1094" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Atualiza preços de 2026-10-27
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1094"/>
+  <dimension ref="A1:G1115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24461,9 +24461,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D1074" t="inlineStr"/>
-      <c r="E1074" t="inlineStr"/>
-      <c r="F1074" t="inlineStr"/>
       <c r="G1074" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -24486,9 +24483,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D1075" t="inlineStr"/>
-      <c r="E1075" t="inlineStr"/>
-      <c r="F1075" t="inlineStr"/>
       <c r="G1075" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -24511,9 +24505,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D1076" t="inlineStr"/>
-      <c r="E1076" t="inlineStr"/>
-      <c r="F1076" t="inlineStr"/>
       <c r="G1076" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -24536,9 +24527,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D1077" t="inlineStr"/>
-      <c r="E1077" t="inlineStr"/>
-      <c r="F1077" t="inlineStr"/>
       <c r="G1077" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -24569,7 +24557,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Duplex-litros-Branca/dp/B07FXZ8TR6/ref=sr_1_5</t>
         </is>
       </c>
-      <c r="G1078" t="inlineStr"/>
     </row>
     <row r="1079">
       <c r="A1079" t="inlineStr">
@@ -24595,7 +24582,6 @@
           <t>https://www.amazon.com.br/Geladeira-BRM46MK-Duplex-Extrafrio-Brastemp/dp/B0GL3Q3PTG/ref=sr_1_6</t>
         </is>
       </c>
-      <c r="G1079" t="inlineStr"/>
     </row>
     <row r="1080">
       <c r="A1080" t="inlineStr">
@@ -24621,7 +24607,6 @@
           <t>https://www.amazon.com.br/Geladeira-Refrigerador-Brastemp-Duplex-Litros/dp/B07ND4BB3C/ref=sr_1_7</t>
         </is>
       </c>
-      <c r="G1080" t="inlineStr"/>
     </row>
     <row r="1081">
       <c r="A1081" t="inlineStr">
@@ -24639,9 +24624,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D1081" t="inlineStr"/>
-      <c r="E1081" t="inlineStr"/>
-      <c r="F1081" t="inlineStr"/>
       <c r="G1081" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -24664,9 +24646,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D1082" t="inlineStr"/>
-      <c r="E1082" t="inlineStr"/>
-      <c r="F1082" t="inlineStr"/>
       <c r="G1082" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -24689,9 +24668,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D1083" t="inlineStr"/>
-      <c r="E1083" t="inlineStr"/>
-      <c r="F1083" t="inlineStr"/>
       <c r="G1083" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -24714,9 +24690,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D1084" t="inlineStr"/>
-      <c r="E1084" t="inlineStr"/>
-      <c r="F1084" t="inlineStr"/>
       <c r="G1084" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -24747,7 +24720,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P2FLSR/ref=sr_1_5_mod_primary_new</t>
         </is>
       </c>
-      <c r="G1085" t="inlineStr"/>
     </row>
     <row r="1086">
       <c r="A1086" t="inlineStr">
@@ -24773,7 +24745,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P2FLSR/ref=sr_1_5_mod_new</t>
         </is>
       </c>
-      <c r="G1086" t="inlineStr"/>
     </row>
     <row r="1087">
       <c r="A1087" t="inlineStr">
@@ -24799,7 +24770,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P3T3VM/ref=sr_1_6</t>
         </is>
       </c>
-      <c r="G1087" t="inlineStr"/>
     </row>
     <row r="1088">
       <c r="A1088" t="inlineStr">
@@ -24817,9 +24787,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D1088" t="inlineStr"/>
-      <c r="E1088" t="inlineStr"/>
-      <c r="F1088" t="inlineStr"/>
       <c r="G1088" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -24842,9 +24809,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D1089" t="inlineStr"/>
-      <c r="E1089" t="inlineStr"/>
-      <c r="F1089" t="inlineStr"/>
       <c r="G1089" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -24867,9 +24831,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D1090" t="inlineStr"/>
-      <c r="E1090" t="inlineStr"/>
-      <c r="F1090" t="inlineStr"/>
       <c r="G1090" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -24892,9 +24853,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D1091" t="inlineStr"/>
-      <c r="E1091" t="inlineStr"/>
-      <c r="F1091" t="inlineStr"/>
       <c r="G1091" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -24925,7 +24883,6 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-Consul-Bocas-CFO4NARUNA-Bivolt/dp/B07HM9JL5K/ref=sr_1_5</t>
         </is>
       </c>
-      <c r="G1092" t="inlineStr"/>
     </row>
     <row r="1093">
       <c r="A1093" t="inlineStr">
@@ -24951,7 +24908,6 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-Bocas-Consul-Vidro-Bivolt/dp/B076BC7769/ref=sr_1_6</t>
         </is>
       </c>
-      <c r="G1093" t="inlineStr"/>
     </row>
     <row r="1094">
       <c r="A1094" t="inlineStr">
@@ -24977,7 +24933,540 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-04-Bocas-FS-CF04NABUNA/dp/B07JPZN51P/ref=sr_1_7</t>
         </is>
       </c>
-      <c r="G1094" t="inlineStr"/>
+    </row>
+    <row r="1095">
+      <c r="A1095" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1095" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1095" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D1095" t="inlineStr"/>
+      <c r="E1095" t="inlineStr"/>
+      <c r="F1095" t="inlineStr"/>
+      <c r="G1095" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1096">
+      <c r="A1096" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1096" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1096" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D1096" t="inlineStr"/>
+      <c r="E1096" t="inlineStr"/>
+      <c r="F1096" t="inlineStr"/>
+      <c r="G1096" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1097">
+      <c r="A1097" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1097" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1097" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D1097" t="inlineStr"/>
+      <c r="E1097" t="inlineStr"/>
+      <c r="F1097" t="inlineStr"/>
+      <c r="G1097" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1098">
+      <c r="A1098" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1098" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1098" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D1098" t="inlineStr"/>
+      <c r="E1098" t="inlineStr"/>
+      <c r="F1098" t="inlineStr"/>
+      <c r="G1098" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1099">
+      <c r="A1099" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1099" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1099" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1099" t="n">
+        <v>2776.67</v>
+      </c>
+      <c r="F1099" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Duplex-litros-Branca/dp/B07FXZ8TR6/ref=sr_1_1</t>
+        </is>
+      </c>
+      <c r="G1099" t="inlineStr"/>
+    </row>
+    <row r="1100">
+      <c r="A1100" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1100" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1100" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1100" t="n">
+        <v>2630.55</v>
+      </c>
+      <c r="F1100" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-BRM46MK-Duplex-Extrafrio-Brastemp/dp/B0GL3Q3PTG/ref=sr_1_2</t>
+        </is>
+      </c>
+      <c r="G1100" t="inlineStr"/>
+    </row>
+    <row r="1101">
+      <c r="A1101" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1101" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1101" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1101" t="n">
+        <v>2564.05</v>
+      </c>
+      <c r="F1101" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Litros-Duplex-Branca/dp/B0GFB8M9MZ/ref=sr_1_3</t>
+        </is>
+      </c>
+      <c r="G1101" t="inlineStr"/>
+    </row>
+    <row r="1102">
+      <c r="A1102" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1102" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1102" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D1102" t="inlineStr"/>
+      <c r="E1102" t="inlineStr"/>
+      <c r="F1102" t="inlineStr"/>
+      <c r="G1102" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1103">
+      <c r="A1103" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1103" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1103" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D1103" t="inlineStr"/>
+      <c r="E1103" t="inlineStr"/>
+      <c r="F1103" t="inlineStr"/>
+      <c r="G1103" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1104">
+      <c r="A1104" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1104" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1104" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D1104" t="inlineStr"/>
+      <c r="E1104" t="inlineStr"/>
+      <c r="F1104" t="inlineStr"/>
+      <c r="G1104" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1105">
+      <c r="A1105" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1105" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1105" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D1105" t="inlineStr"/>
+      <c r="E1105" t="inlineStr"/>
+      <c r="F1105" t="inlineStr"/>
+      <c r="G1105" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1106">
+      <c r="A1106" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1106" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1106" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1106" t="n">
+        <v>509</v>
+      </c>
+      <c r="F1106" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P2FLSR/ref=sr_1_1</t>
+        </is>
+      </c>
+      <c r="G1106" t="inlineStr"/>
+    </row>
+    <row r="1107">
+      <c r="A1107" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1107" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1107" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1107" t="n">
+        <v>496.22</v>
+      </c>
+      <c r="F1107" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Efficient-23L-ME23B/dp/B0B8KWNK12/ref=sr_1_2</t>
+        </is>
+      </c>
+      <c r="G1107" t="inlineStr"/>
+    </row>
+    <row r="1108">
+      <c r="A1108" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1108" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1108" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1108" t="n">
+        <v>529</v>
+      </c>
+      <c r="F1108" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Electrolux-MTO30-Fun%C3%A7%C3%A3o-Tira/dp/B083ZFFC5Q/ref=sr_1_3</t>
+        </is>
+      </c>
+      <c r="G1108" t="inlineStr"/>
+    </row>
+    <row r="1109">
+      <c r="A1109" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1109" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1109" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D1109" t="inlineStr"/>
+      <c r="E1109" t="inlineStr"/>
+      <c r="F1109" t="inlineStr"/>
+      <c r="G1109" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1110">
+      <c r="A1110" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1110" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1110" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D1110" t="inlineStr"/>
+      <c r="E1110" t="inlineStr"/>
+      <c r="F1110" t="inlineStr"/>
+      <c r="G1110" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1111">
+      <c r="A1111" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1111" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1111" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D1111" t="inlineStr"/>
+      <c r="E1111" t="inlineStr"/>
+      <c r="F1111" t="inlineStr"/>
+      <c r="G1111" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1112">
+      <c r="A1112" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1112" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1112" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D1112" t="inlineStr"/>
+      <c r="E1112" t="inlineStr"/>
+      <c r="F1112" t="inlineStr"/>
+      <c r="G1112" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1113">
+      <c r="A1113" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1113" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1113" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1113" t="n">
+        <v>1234.05</v>
+      </c>
+      <c r="F1113" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-Consul-Bocas-CFO4NARUNA-Bivolt/dp/B07HM9JL5K/ref=sr_1_1</t>
+        </is>
+      </c>
+      <c r="G1113" t="inlineStr"/>
+    </row>
+    <row r="1114">
+      <c r="A1114" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1114" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1114" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1114" t="n">
+        <v>1189.15</v>
+      </c>
+      <c r="F1114" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-Bocas-Consul-Vidro-Bivolt/dp/B076BC7769/ref=sr_1_2</t>
+        </is>
+      </c>
+      <c r="G1114" t="inlineStr"/>
+    </row>
+    <row r="1115">
+      <c r="A1115" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1115" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1115" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1115" t="n">
+        <v>1044.9</v>
+      </c>
+      <c r="F1115" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-04-Bocas-FS-CF04NABUNA/dp/B07JPZN51P/ref=sr_1_3</t>
+        </is>
+      </c>
+      <c r="G1115" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Atualiza preços de 2026-10-28
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1115"/>
+  <dimension ref="A1:G1136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24950,9 +24950,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D1095" t="inlineStr"/>
-      <c r="E1095" t="inlineStr"/>
-      <c r="F1095" t="inlineStr"/>
       <c r="G1095" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -24975,9 +24972,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D1096" t="inlineStr"/>
-      <c r="E1096" t="inlineStr"/>
-      <c r="F1096" t="inlineStr"/>
       <c r="G1096" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -25000,9 +24994,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D1097" t="inlineStr"/>
-      <c r="E1097" t="inlineStr"/>
-      <c r="F1097" t="inlineStr"/>
       <c r="G1097" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -25025,9 +25016,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D1098" t="inlineStr"/>
-      <c r="E1098" t="inlineStr"/>
-      <c r="F1098" t="inlineStr"/>
       <c r="G1098" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -25058,7 +25046,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Duplex-litros-Branca/dp/B07FXZ8TR6/ref=sr_1_1</t>
         </is>
       </c>
-      <c r="G1099" t="inlineStr"/>
     </row>
     <row r="1100">
       <c r="A1100" t="inlineStr">
@@ -25084,7 +25071,6 @@
           <t>https://www.amazon.com.br/Geladeira-BRM46MK-Duplex-Extrafrio-Brastemp/dp/B0GL3Q3PTG/ref=sr_1_2</t>
         </is>
       </c>
-      <c r="G1100" t="inlineStr"/>
     </row>
     <row r="1101">
       <c r="A1101" t="inlineStr">
@@ -25110,7 +25096,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Litros-Duplex-Branca/dp/B0GFB8M9MZ/ref=sr_1_3</t>
         </is>
       </c>
-      <c r="G1101" t="inlineStr"/>
     </row>
     <row r="1102">
       <c r="A1102" t="inlineStr">
@@ -25128,9 +25113,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D1102" t="inlineStr"/>
-      <c r="E1102" t="inlineStr"/>
-      <c r="F1102" t="inlineStr"/>
       <c r="G1102" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -25153,9 +25135,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D1103" t="inlineStr"/>
-      <c r="E1103" t="inlineStr"/>
-      <c r="F1103" t="inlineStr"/>
       <c r="G1103" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -25178,9 +25157,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D1104" t="inlineStr"/>
-      <c r="E1104" t="inlineStr"/>
-      <c r="F1104" t="inlineStr"/>
       <c r="G1104" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -25203,9 +25179,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D1105" t="inlineStr"/>
-      <c r="E1105" t="inlineStr"/>
-      <c r="F1105" t="inlineStr"/>
       <c r="G1105" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -25236,7 +25209,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P2FLSR/ref=sr_1_1</t>
         </is>
       </c>
-      <c r="G1106" t="inlineStr"/>
     </row>
     <row r="1107">
       <c r="A1107" t="inlineStr">
@@ -25262,7 +25234,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Efficient-23L-ME23B/dp/B0B8KWNK12/ref=sr_1_2</t>
         </is>
       </c>
-      <c r="G1107" t="inlineStr"/>
     </row>
     <row r="1108">
       <c r="A1108" t="inlineStr">
@@ -25288,7 +25259,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Electrolux-MTO30-Fun%C3%A7%C3%A3o-Tira/dp/B083ZFFC5Q/ref=sr_1_3</t>
         </is>
       </c>
-      <c r="G1108" t="inlineStr"/>
     </row>
     <row r="1109">
       <c r="A1109" t="inlineStr">
@@ -25306,9 +25276,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D1109" t="inlineStr"/>
-      <c r="E1109" t="inlineStr"/>
-      <c r="F1109" t="inlineStr"/>
       <c r="G1109" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -25331,9 +25298,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D1110" t="inlineStr"/>
-      <c r="E1110" t="inlineStr"/>
-      <c r="F1110" t="inlineStr"/>
       <c r="G1110" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -25356,9 +25320,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D1111" t="inlineStr"/>
-      <c r="E1111" t="inlineStr"/>
-      <c r="F1111" t="inlineStr"/>
       <c r="G1111" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -25381,9 +25342,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D1112" t="inlineStr"/>
-      <c r="E1112" t="inlineStr"/>
-      <c r="F1112" t="inlineStr"/>
       <c r="G1112" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -25414,7 +25372,6 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-Consul-Bocas-CFO4NARUNA-Bivolt/dp/B07HM9JL5K/ref=sr_1_1</t>
         </is>
       </c>
-      <c r="G1113" t="inlineStr"/>
     </row>
     <row r="1114">
       <c r="A1114" t="inlineStr">
@@ -25440,7 +25397,6 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-Bocas-Consul-Vidro-Bivolt/dp/B076BC7769/ref=sr_1_2</t>
         </is>
       </c>
-      <c r="G1114" t="inlineStr"/>
     </row>
     <row r="1115">
       <c r="A1115" t="inlineStr">
@@ -25466,7 +25422,540 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-04-Bocas-FS-CF04NABUNA/dp/B07JPZN51P/ref=sr_1_3</t>
         </is>
       </c>
-      <c r="G1115" t="inlineStr"/>
+    </row>
+    <row r="1116">
+      <c r="A1116" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B1116" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1116" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D1116" t="inlineStr"/>
+      <c r="E1116" t="inlineStr"/>
+      <c r="F1116" t="inlineStr"/>
+      <c r="G1116" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1117">
+      <c r="A1117" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B1117" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1117" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D1117" t="inlineStr"/>
+      <c r="E1117" t="inlineStr"/>
+      <c r="F1117" t="inlineStr"/>
+      <c r="G1117" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1118">
+      <c r="A1118" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B1118" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1118" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D1118" t="inlineStr"/>
+      <c r="E1118" t="inlineStr"/>
+      <c r="F1118" t="inlineStr"/>
+      <c r="G1118" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1119">
+      <c r="A1119" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B1119" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1119" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D1119" t="inlineStr"/>
+      <c r="E1119" t="inlineStr"/>
+      <c r="F1119" t="inlineStr"/>
+      <c r="G1119" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1120">
+      <c r="A1120" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B1120" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1120" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1120" t="n">
+        <v>2012.61</v>
+      </c>
+      <c r="F1120" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Duplex-litros-Branca/dp/B07FXZ8TR6/ref=sr_1_5</t>
+        </is>
+      </c>
+      <c r="G1120" t="inlineStr"/>
+    </row>
+    <row r="1121">
+      <c r="A1121" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B1121" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1121" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1121" t="n">
+        <v>2564.05</v>
+      </c>
+      <c r="F1121" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Litros-Duplex-Branca/dp/B0GFB8M9MZ/ref=sr_1_6</t>
+        </is>
+      </c>
+      <c r="G1121" t="inlineStr"/>
+    </row>
+    <row r="1122">
+      <c r="A1122" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B1122" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1122" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1122" t="n">
+        <v>3399.15</v>
+      </c>
+      <c r="F1122" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWVJ8LR/ref=sr_1_7</t>
+        </is>
+      </c>
+      <c r="G1122" t="inlineStr"/>
+    </row>
+    <row r="1123">
+      <c r="A1123" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B1123" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1123" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D1123" t="inlineStr"/>
+      <c r="E1123" t="inlineStr"/>
+      <c r="F1123" t="inlineStr"/>
+      <c r="G1123" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1124">
+      <c r="A1124" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B1124" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1124" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D1124" t="inlineStr"/>
+      <c r="E1124" t="inlineStr"/>
+      <c r="F1124" t="inlineStr"/>
+      <c r="G1124" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1125">
+      <c r="A1125" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B1125" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1125" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D1125" t="inlineStr"/>
+      <c r="E1125" t="inlineStr"/>
+      <c r="F1125" t="inlineStr"/>
+      <c r="G1125" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1126">
+      <c r="A1126" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B1126" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1126" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D1126" t="inlineStr"/>
+      <c r="E1126" t="inlineStr"/>
+      <c r="F1126" t="inlineStr"/>
+      <c r="G1126" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1127">
+      <c r="A1127" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B1127" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1127" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1127" t="n">
+        <v>537.83</v>
+      </c>
+      <c r="F1127" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P2FLSR/ref=sr_1_5</t>
+        </is>
+      </c>
+      <c r="G1127" t="inlineStr"/>
+    </row>
+    <row r="1128">
+      <c r="A1128" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B1128" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1128" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1128" t="n">
+        <v>426.61</v>
+      </c>
+      <c r="F1128" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Efficient-23L-ME23B/dp/B0B8KWNK12/ref=sr_1_6</t>
+        </is>
+      </c>
+      <c r="G1128" t="inlineStr"/>
+    </row>
+    <row r="1129">
+      <c r="A1129" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B1129" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1129" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1129" t="n">
+        <v>519</v>
+      </c>
+      <c r="F1129" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P3T3VM/ref=sr_1_7</t>
+        </is>
+      </c>
+      <c r="G1129" t="inlineStr"/>
+    </row>
+    <row r="1130">
+      <c r="A1130" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B1130" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1130" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D1130" t="inlineStr"/>
+      <c r="E1130" t="inlineStr"/>
+      <c r="F1130" t="inlineStr"/>
+      <c r="G1130" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1131">
+      <c r="A1131" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B1131" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1131" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D1131" t="inlineStr"/>
+      <c r="E1131" t="inlineStr"/>
+      <c r="F1131" t="inlineStr"/>
+      <c r="G1131" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1132">
+      <c r="A1132" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B1132" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1132" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D1132" t="inlineStr"/>
+      <c r="E1132" t="inlineStr"/>
+      <c r="F1132" t="inlineStr"/>
+      <c r="G1132" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1133">
+      <c r="A1133" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B1133" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1133" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D1133" t="inlineStr"/>
+      <c r="E1133" t="inlineStr"/>
+      <c r="F1133" t="inlineStr"/>
+      <c r="G1133" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1134">
+      <c r="A1134" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B1134" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1134" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1134" t="n">
+        <v>1098</v>
+      </c>
+      <c r="F1134" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-Consul-Bocas-CFO4NARUNA-Bivolt/dp/B07HM9JL5K/ref=sr_1_1</t>
+        </is>
+      </c>
+      <c r="G1134" t="inlineStr"/>
+    </row>
+    <row r="1135">
+      <c r="A1135" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B1135" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1135" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1135" t="n">
+        <v>1259.1</v>
+      </c>
+      <c r="F1135" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-Bocas-Consul-Vidro-Bivolt/dp/B076BC7769/ref=sr_1_2</t>
+        </is>
+      </c>
+      <c r="G1135" t="inlineStr"/>
+    </row>
+    <row r="1136">
+      <c r="A1136" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B1136" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1136" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1136" t="n">
+        <v>1044.9</v>
+      </c>
+      <c r="F1136" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-04-Bocas-FS-CF04NABUNA/dp/B07JPZN51P/ref=sr_1_3</t>
+        </is>
+      </c>
+      <c r="G1136" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Atualiza preços de 2026-10-29
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1136"/>
+  <dimension ref="A1:G1157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25439,9 +25439,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D1116" t="inlineStr"/>
-      <c r="E1116" t="inlineStr"/>
-      <c r="F1116" t="inlineStr"/>
       <c r="G1116" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -25464,9 +25461,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D1117" t="inlineStr"/>
-      <c r="E1117" t="inlineStr"/>
-      <c r="F1117" t="inlineStr"/>
       <c r="G1117" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -25489,9 +25483,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D1118" t="inlineStr"/>
-      <c r="E1118" t="inlineStr"/>
-      <c r="F1118" t="inlineStr"/>
       <c r="G1118" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -25514,9 +25505,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D1119" t="inlineStr"/>
-      <c r="E1119" t="inlineStr"/>
-      <c r="F1119" t="inlineStr"/>
       <c r="G1119" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -25547,7 +25535,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Duplex-litros-Branca/dp/B07FXZ8TR6/ref=sr_1_5</t>
         </is>
       </c>
-      <c r="G1120" t="inlineStr"/>
     </row>
     <row r="1121">
       <c r="A1121" t="inlineStr">
@@ -25573,7 +25560,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Litros-Duplex-Branca/dp/B0GFB8M9MZ/ref=sr_1_6</t>
         </is>
       </c>
-      <c r="G1121" t="inlineStr"/>
     </row>
     <row r="1122">
       <c r="A1122" t="inlineStr">
@@ -25599,7 +25585,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWVJ8LR/ref=sr_1_7</t>
         </is>
       </c>
-      <c r="G1122" t="inlineStr"/>
     </row>
     <row r="1123">
       <c r="A1123" t="inlineStr">
@@ -25617,9 +25602,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D1123" t="inlineStr"/>
-      <c r="E1123" t="inlineStr"/>
-      <c r="F1123" t="inlineStr"/>
       <c r="G1123" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -25642,9 +25624,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D1124" t="inlineStr"/>
-      <c r="E1124" t="inlineStr"/>
-      <c r="F1124" t="inlineStr"/>
       <c r="G1124" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -25667,9 +25646,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D1125" t="inlineStr"/>
-      <c r="E1125" t="inlineStr"/>
-      <c r="F1125" t="inlineStr"/>
       <c r="G1125" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -25692,9 +25668,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D1126" t="inlineStr"/>
-      <c r="E1126" t="inlineStr"/>
-      <c r="F1126" t="inlineStr"/>
       <c r="G1126" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -25725,7 +25698,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P2FLSR/ref=sr_1_5</t>
         </is>
       </c>
-      <c r="G1127" t="inlineStr"/>
     </row>
     <row r="1128">
       <c r="A1128" t="inlineStr">
@@ -25751,7 +25723,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Efficient-23L-ME23B/dp/B0B8KWNK12/ref=sr_1_6</t>
         </is>
       </c>
-      <c r="G1128" t="inlineStr"/>
     </row>
     <row r="1129">
       <c r="A1129" t="inlineStr">
@@ -25777,7 +25748,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P3T3VM/ref=sr_1_7</t>
         </is>
       </c>
-      <c r="G1129" t="inlineStr"/>
     </row>
     <row r="1130">
       <c r="A1130" t="inlineStr">
@@ -25795,9 +25765,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D1130" t="inlineStr"/>
-      <c r="E1130" t="inlineStr"/>
-      <c r="F1130" t="inlineStr"/>
       <c r="G1130" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -25820,9 +25787,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D1131" t="inlineStr"/>
-      <c r="E1131" t="inlineStr"/>
-      <c r="F1131" t="inlineStr"/>
       <c r="G1131" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -25845,9 +25809,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D1132" t="inlineStr"/>
-      <c r="E1132" t="inlineStr"/>
-      <c r="F1132" t="inlineStr"/>
       <c r="G1132" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -25870,9 +25831,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D1133" t="inlineStr"/>
-      <c r="E1133" t="inlineStr"/>
-      <c r="F1133" t="inlineStr"/>
       <c r="G1133" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -25903,7 +25861,6 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-Consul-Bocas-CFO4NARUNA-Bivolt/dp/B07HM9JL5K/ref=sr_1_1</t>
         </is>
       </c>
-      <c r="G1134" t="inlineStr"/>
     </row>
     <row r="1135">
       <c r="A1135" t="inlineStr">
@@ -25929,7 +25886,6 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-Bocas-Consul-Vidro-Bivolt/dp/B076BC7769/ref=sr_1_2</t>
         </is>
       </c>
-      <c r="G1135" t="inlineStr"/>
     </row>
     <row r="1136">
       <c r="A1136" t="inlineStr">
@@ -25955,7 +25911,540 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-04-Bocas-FS-CF04NABUNA/dp/B07JPZN51P/ref=sr_1_3</t>
         </is>
       </c>
-      <c r="G1136" t="inlineStr"/>
+    </row>
+    <row r="1137">
+      <c r="A1137" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B1137" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1137" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D1137" t="inlineStr"/>
+      <c r="E1137" t="inlineStr"/>
+      <c r="F1137" t="inlineStr"/>
+      <c r="G1137" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1138">
+      <c r="A1138" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B1138" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1138" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D1138" t="inlineStr"/>
+      <c r="E1138" t="inlineStr"/>
+      <c r="F1138" t="inlineStr"/>
+      <c r="G1138" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1139">
+      <c r="A1139" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B1139" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1139" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D1139" t="inlineStr"/>
+      <c r="E1139" t="inlineStr"/>
+      <c r="F1139" t="inlineStr"/>
+      <c r="G1139" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1140">
+      <c r="A1140" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B1140" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1140" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D1140" t="inlineStr"/>
+      <c r="E1140" t="inlineStr"/>
+      <c r="F1140" t="inlineStr"/>
+      <c r="G1140" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1141">
+      <c r="A1141" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B1141" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1141" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1141" t="n">
+        <v>2012.61</v>
+      </c>
+      <c r="F1141" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Duplex-litros-Branca/dp/B07FXZ8TR6/ref=sr_1_1</t>
+        </is>
+      </c>
+      <c r="G1141" t="inlineStr"/>
+    </row>
+    <row r="1142">
+      <c r="A1142" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B1142" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1142" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1142" t="n">
+        <v>999</v>
+      </c>
+      <c r="F1142" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Refrigerador-Brastemp-Duplex-Litros/dp/B07ND4BB3C/ref=sr_1_2</t>
+        </is>
+      </c>
+      <c r="G1142" t="inlineStr"/>
+    </row>
+    <row r="1143">
+      <c r="A1143" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B1143" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1143" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1143" t="n">
+        <v>2735.77</v>
+      </c>
+      <c r="F1143" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-BRM46MK-Duplex-Extrafrio-Brastemp/dp/B0GL3Q3PTG/ref=sr_1_3</t>
+        </is>
+      </c>
+      <c r="G1143" t="inlineStr"/>
+    </row>
+    <row r="1144">
+      <c r="A1144" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B1144" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1144" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D1144" t="inlineStr"/>
+      <c r="E1144" t="inlineStr"/>
+      <c r="F1144" t="inlineStr"/>
+      <c r="G1144" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1145">
+      <c r="A1145" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B1145" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1145" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D1145" t="inlineStr"/>
+      <c r="E1145" t="inlineStr"/>
+      <c r="F1145" t="inlineStr"/>
+      <c r="G1145" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1146">
+      <c r="A1146" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B1146" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1146" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D1146" t="inlineStr"/>
+      <c r="E1146" t="inlineStr"/>
+      <c r="F1146" t="inlineStr"/>
+      <c r="G1146" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1147">
+      <c r="A1147" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B1147" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1147" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D1147" t="inlineStr"/>
+      <c r="E1147" t="inlineStr"/>
+      <c r="F1147" t="inlineStr"/>
+      <c r="G1147" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1148">
+      <c r="A1148" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B1148" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1148" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1148" t="n">
+        <v>518.73</v>
+      </c>
+      <c r="F1148" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P2FLSR/ref=sr_1_1</t>
+        </is>
+      </c>
+      <c r="G1148" t="inlineStr"/>
+    </row>
+    <row r="1149">
+      <c r="A1149" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B1149" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1149" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1149" t="n">
+        <v>509</v>
+      </c>
+      <c r="F1149" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P3T3VM/ref=sr_1_2</t>
+        </is>
+      </c>
+      <c r="G1149" t="inlineStr"/>
+    </row>
+    <row r="1150">
+      <c r="A1150" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B1150" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1150" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1150" t="n">
+        <v>496.23</v>
+      </c>
+      <c r="F1150" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Efficient-23L-ME23B/dp/B0B8KWNK12/ref=sr_1_3</t>
+        </is>
+      </c>
+      <c r="G1150" t="inlineStr"/>
+    </row>
+    <row r="1151">
+      <c r="A1151" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B1151" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1151" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D1151" t="inlineStr"/>
+      <c r="E1151" t="inlineStr"/>
+      <c r="F1151" t="inlineStr"/>
+      <c r="G1151" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1152">
+      <c r="A1152" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B1152" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1152" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D1152" t="inlineStr"/>
+      <c r="E1152" t="inlineStr"/>
+      <c r="F1152" t="inlineStr"/>
+      <c r="G1152" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1153">
+      <c r="A1153" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B1153" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1153" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D1153" t="inlineStr"/>
+      <c r="E1153" t="inlineStr"/>
+      <c r="F1153" t="inlineStr"/>
+      <c r="G1153" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1154">
+      <c r="A1154" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B1154" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1154" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D1154" t="inlineStr"/>
+      <c r="E1154" t="inlineStr"/>
+      <c r="F1154" t="inlineStr"/>
+      <c r="G1154" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1155">
+      <c r="A1155" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B1155" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1155" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1155" t="n">
+        <v>1037</v>
+      </c>
+      <c r="F1155" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-Consul-Bocas-CFO4NARUNA-Bivolt/dp/B07HM9JL5K/ref=sr_1_1</t>
+        </is>
+      </c>
+      <c r="G1155" t="inlineStr"/>
+    </row>
+    <row r="1156">
+      <c r="A1156" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B1156" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1156" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1156" t="n">
+        <v>1453</v>
+      </c>
+      <c r="F1156" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-Bocas-Consul-Vidro-Bivolt/dp/B076BC7769/ref=sr_1_2</t>
+        </is>
+      </c>
+      <c r="G1156" t="inlineStr"/>
+    </row>
+    <row r="1157">
+      <c r="A1157" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B1157" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1157" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1157" t="n">
+        <v>1163.65</v>
+      </c>
+      <c r="F1157" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-04-Bocas-FS-CF04NABUNA/dp/B07JPZN51P/ref=sr_1_3</t>
+        </is>
+      </c>
+      <c r="G1157" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Atualiza preços de 2026-10-30
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1157"/>
+  <dimension ref="A1:G1178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25928,9 +25928,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D1137" t="inlineStr"/>
-      <c r="E1137" t="inlineStr"/>
-      <c r="F1137" t="inlineStr"/>
       <c r="G1137" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -25953,9 +25950,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D1138" t="inlineStr"/>
-      <c r="E1138" t="inlineStr"/>
-      <c r="F1138" t="inlineStr"/>
       <c r="G1138" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -25978,9 +25972,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D1139" t="inlineStr"/>
-      <c r="E1139" t="inlineStr"/>
-      <c r="F1139" t="inlineStr"/>
       <c r="G1139" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -26003,9 +25994,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D1140" t="inlineStr"/>
-      <c r="E1140" t="inlineStr"/>
-      <c r="F1140" t="inlineStr"/>
       <c r="G1140" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -26036,7 +26024,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Duplex-litros-Branca/dp/B07FXZ8TR6/ref=sr_1_1</t>
         </is>
       </c>
-      <c r="G1141" t="inlineStr"/>
     </row>
     <row r="1142">
       <c r="A1142" t="inlineStr">
@@ -26062,7 +26049,6 @@
           <t>https://www.amazon.com.br/Geladeira-Refrigerador-Brastemp-Duplex-Litros/dp/B07ND4BB3C/ref=sr_1_2</t>
         </is>
       </c>
-      <c r="G1142" t="inlineStr"/>
     </row>
     <row r="1143">
       <c r="A1143" t="inlineStr">
@@ -26088,7 +26074,6 @@
           <t>https://www.amazon.com.br/Geladeira-BRM46MK-Duplex-Extrafrio-Brastemp/dp/B0GL3Q3PTG/ref=sr_1_3</t>
         </is>
       </c>
-      <c r="G1143" t="inlineStr"/>
     </row>
     <row r="1144">
       <c r="A1144" t="inlineStr">
@@ -26106,9 +26091,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D1144" t="inlineStr"/>
-      <c r="E1144" t="inlineStr"/>
-      <c r="F1144" t="inlineStr"/>
       <c r="G1144" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -26131,9 +26113,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D1145" t="inlineStr"/>
-      <c r="E1145" t="inlineStr"/>
-      <c r="F1145" t="inlineStr"/>
       <c r="G1145" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -26156,9 +26135,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D1146" t="inlineStr"/>
-      <c r="E1146" t="inlineStr"/>
-      <c r="F1146" t="inlineStr"/>
       <c r="G1146" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -26181,9 +26157,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D1147" t="inlineStr"/>
-      <c r="E1147" t="inlineStr"/>
-      <c r="F1147" t="inlineStr"/>
       <c r="G1147" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -26214,7 +26187,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P2FLSR/ref=sr_1_1</t>
         </is>
       </c>
-      <c r="G1148" t="inlineStr"/>
     </row>
     <row r="1149">
       <c r="A1149" t="inlineStr">
@@ -26240,7 +26212,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P3T3VM/ref=sr_1_2</t>
         </is>
       </c>
-      <c r="G1149" t="inlineStr"/>
     </row>
     <row r="1150">
       <c r="A1150" t="inlineStr">
@@ -26266,7 +26237,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Efficient-23L-ME23B/dp/B0B8KWNK12/ref=sr_1_3</t>
         </is>
       </c>
-      <c r="G1150" t="inlineStr"/>
     </row>
     <row r="1151">
       <c r="A1151" t="inlineStr">
@@ -26284,9 +26254,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D1151" t="inlineStr"/>
-      <c r="E1151" t="inlineStr"/>
-      <c r="F1151" t="inlineStr"/>
       <c r="G1151" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -26309,9 +26276,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D1152" t="inlineStr"/>
-      <c r="E1152" t="inlineStr"/>
-      <c r="F1152" t="inlineStr"/>
       <c r="G1152" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -26334,9 +26298,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D1153" t="inlineStr"/>
-      <c r="E1153" t="inlineStr"/>
-      <c r="F1153" t="inlineStr"/>
       <c r="G1153" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -26359,9 +26320,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D1154" t="inlineStr"/>
-      <c r="E1154" t="inlineStr"/>
-      <c r="F1154" t="inlineStr"/>
       <c r="G1154" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -26392,7 +26350,6 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-Consul-Bocas-CFO4NARUNA-Bivolt/dp/B07HM9JL5K/ref=sr_1_1</t>
         </is>
       </c>
-      <c r="G1155" t="inlineStr"/>
     </row>
     <row r="1156">
       <c r="A1156" t="inlineStr">
@@ -26418,7 +26375,6 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-Bocas-Consul-Vidro-Bivolt/dp/B076BC7769/ref=sr_1_2</t>
         </is>
       </c>
-      <c r="G1156" t="inlineStr"/>
     </row>
     <row r="1157">
       <c r="A1157" t="inlineStr">
@@ -26444,7 +26400,540 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-04-Bocas-FS-CF04NABUNA/dp/B07JPZN51P/ref=sr_1_3</t>
         </is>
       </c>
-      <c r="G1157" t="inlineStr"/>
+    </row>
+    <row r="1158">
+      <c r="A1158" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1158" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1158" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D1158" t="inlineStr"/>
+      <c r="E1158" t="inlineStr"/>
+      <c r="F1158" t="inlineStr"/>
+      <c r="G1158" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1159">
+      <c r="A1159" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1159" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1159" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D1159" t="inlineStr"/>
+      <c r="E1159" t="inlineStr"/>
+      <c r="F1159" t="inlineStr"/>
+      <c r="G1159" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1160">
+      <c r="A1160" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1160" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1160" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D1160" t="inlineStr"/>
+      <c r="E1160" t="inlineStr"/>
+      <c r="F1160" t="inlineStr"/>
+      <c r="G1160" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1161">
+      <c r="A1161" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1161" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1161" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D1161" t="inlineStr"/>
+      <c r="E1161" t="inlineStr"/>
+      <c r="F1161" t="inlineStr"/>
+      <c r="G1161" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1162">
+      <c r="A1162" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1162" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1162" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1162" t="n">
+        <v>2012.61</v>
+      </c>
+      <c r="F1162" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Duplex-litros-Branca/dp/B07FXZ8TR6/ref=sr_1_1</t>
+        </is>
+      </c>
+      <c r="G1162" t="inlineStr"/>
+    </row>
+    <row r="1163">
+      <c r="A1163" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1163" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1163" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1163" t="n">
+        <v>2796.69</v>
+      </c>
+      <c r="F1163" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-BRM46MK-Duplex-Extrafrio-Brastemp/dp/B0GL3Q3PTG/ref=sr_1_2</t>
+        </is>
+      </c>
+      <c r="G1163" t="inlineStr"/>
+    </row>
+    <row r="1164">
+      <c r="A1164" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1164" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1164" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1164" t="n">
+        <v>2656.85</v>
+      </c>
+      <c r="F1164" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Litros-Duplex/dp/B0GFGNR7DQ/ref=sr_1_3</t>
+        </is>
+      </c>
+      <c r="G1164" t="inlineStr"/>
+    </row>
+    <row r="1165">
+      <c r="A1165" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1165" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1165" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D1165" t="inlineStr"/>
+      <c r="E1165" t="inlineStr"/>
+      <c r="F1165" t="inlineStr"/>
+      <c r="G1165" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1166">
+      <c r="A1166" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1166" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1166" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D1166" t="inlineStr"/>
+      <c r="E1166" t="inlineStr"/>
+      <c r="F1166" t="inlineStr"/>
+      <c r="G1166" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1167">
+      <c r="A1167" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1167" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1167" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D1167" t="inlineStr"/>
+      <c r="E1167" t="inlineStr"/>
+      <c r="F1167" t="inlineStr"/>
+      <c r="G1167" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1168">
+      <c r="A1168" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1168" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1168" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D1168" t="inlineStr"/>
+      <c r="E1168" t="inlineStr"/>
+      <c r="F1168" t="inlineStr"/>
+      <c r="G1168" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1169">
+      <c r="A1169" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1169" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1169" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1169" t="n">
+        <v>518.73</v>
+      </c>
+      <c r="F1169" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P2FLSR/ref=sr_1_1</t>
+        </is>
+      </c>
+      <c r="G1169" t="inlineStr"/>
+    </row>
+    <row r="1170">
+      <c r="A1170" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1170" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1170" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1170" t="n">
+        <v>519</v>
+      </c>
+      <c r="F1170" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P3T3VM/ref=sr_1_2</t>
+        </is>
+      </c>
+      <c r="G1170" t="inlineStr"/>
+    </row>
+    <row r="1171">
+      <c r="A1171" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1171" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1171" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1171" t="n">
+        <v>484.03</v>
+      </c>
+      <c r="F1171" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Efficient-23L-ME23B/dp/B0B8KWNK12/ref=sr_1_3</t>
+        </is>
+      </c>
+      <c r="G1171" t="inlineStr"/>
+    </row>
+    <row r="1172">
+      <c r="A1172" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1172" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1172" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D1172" t="inlineStr"/>
+      <c r="E1172" t="inlineStr"/>
+      <c r="F1172" t="inlineStr"/>
+      <c r="G1172" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1173">
+      <c r="A1173" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1173" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1173" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D1173" t="inlineStr"/>
+      <c r="E1173" t="inlineStr"/>
+      <c r="F1173" t="inlineStr"/>
+      <c r="G1173" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1174">
+      <c r="A1174" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1174" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1174" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D1174" t="inlineStr"/>
+      <c r="E1174" t="inlineStr"/>
+      <c r="F1174" t="inlineStr"/>
+      <c r="G1174" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1175">
+      <c r="A1175" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1175" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1175" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D1175" t="inlineStr"/>
+      <c r="E1175" t="inlineStr"/>
+      <c r="F1175" t="inlineStr"/>
+      <c r="G1175" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1176">
+      <c r="A1176" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1176" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1176" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1176" t="n">
+        <v>1037</v>
+      </c>
+      <c r="F1176" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-Consul-Bocas-CFO4NARUNA-Bivolt/dp/B07HM9JL5K/ref=sr_1_1</t>
+        </is>
+      </c>
+      <c r="G1176" t="inlineStr"/>
+    </row>
+    <row r="1177">
+      <c r="A1177" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1177" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1177" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1177" t="n">
+        <v>1443</v>
+      </c>
+      <c r="F1177" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-Bocas-Consul-Vidro-Bivolt/dp/B076BC7769/ref=sr_1_2</t>
+        </is>
+      </c>
+      <c r="G1177" t="inlineStr"/>
+    </row>
+    <row r="1178">
+      <c r="A1178" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1178" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1178" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1178" t="n">
+        <v>901.55</v>
+      </c>
+      <c r="F1178" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Consul-Fog%C3%A3o-bocas-Preto-esmaltada/dp/B0FM83JTS7/ref=sr_1_3</t>
+        </is>
+      </c>
+      <c r="G1178" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Atualiza preços de 2026-10-31
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1178"/>
+  <dimension ref="A1:G1199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26417,9 +26417,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D1158" t="inlineStr"/>
-      <c r="E1158" t="inlineStr"/>
-      <c r="F1158" t="inlineStr"/>
       <c r="G1158" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -26442,9 +26439,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D1159" t="inlineStr"/>
-      <c r="E1159" t="inlineStr"/>
-      <c r="F1159" t="inlineStr"/>
       <c r="G1159" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -26467,9 +26461,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D1160" t="inlineStr"/>
-      <c r="E1160" t="inlineStr"/>
-      <c r="F1160" t="inlineStr"/>
       <c r="G1160" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -26492,9 +26483,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D1161" t="inlineStr"/>
-      <c r="E1161" t="inlineStr"/>
-      <c r="F1161" t="inlineStr"/>
       <c r="G1161" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -26525,7 +26513,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Duplex-litros-Branca/dp/B07FXZ8TR6/ref=sr_1_1</t>
         </is>
       </c>
-      <c r="G1162" t="inlineStr"/>
     </row>
     <row r="1163">
       <c r="A1163" t="inlineStr">
@@ -26551,7 +26538,6 @@
           <t>https://www.amazon.com.br/Geladeira-BRM46MK-Duplex-Extrafrio-Brastemp/dp/B0GL3Q3PTG/ref=sr_1_2</t>
         </is>
       </c>
-      <c r="G1163" t="inlineStr"/>
     </row>
     <row r="1164">
       <c r="A1164" t="inlineStr">
@@ -26577,7 +26563,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Litros-Duplex/dp/B0GFGNR7DQ/ref=sr_1_3</t>
         </is>
       </c>
-      <c r="G1164" t="inlineStr"/>
     </row>
     <row r="1165">
       <c r="A1165" t="inlineStr">
@@ -26595,9 +26580,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D1165" t="inlineStr"/>
-      <c r="E1165" t="inlineStr"/>
-      <c r="F1165" t="inlineStr"/>
       <c r="G1165" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -26620,9 +26602,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D1166" t="inlineStr"/>
-      <c r="E1166" t="inlineStr"/>
-      <c r="F1166" t="inlineStr"/>
       <c r="G1166" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -26645,9 +26624,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D1167" t="inlineStr"/>
-      <c r="E1167" t="inlineStr"/>
-      <c r="F1167" t="inlineStr"/>
       <c r="G1167" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -26670,9 +26646,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D1168" t="inlineStr"/>
-      <c r="E1168" t="inlineStr"/>
-      <c r="F1168" t="inlineStr"/>
       <c r="G1168" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -26703,7 +26676,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P2FLSR/ref=sr_1_1</t>
         </is>
       </c>
-      <c r="G1169" t="inlineStr"/>
     </row>
     <row r="1170">
       <c r="A1170" t="inlineStr">
@@ -26729,7 +26701,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P3T3VM/ref=sr_1_2</t>
         </is>
       </c>
-      <c r="G1170" t="inlineStr"/>
     </row>
     <row r="1171">
       <c r="A1171" t="inlineStr">
@@ -26755,7 +26726,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Efficient-23L-ME23B/dp/B0B8KWNK12/ref=sr_1_3</t>
         </is>
       </c>
-      <c r="G1171" t="inlineStr"/>
     </row>
     <row r="1172">
       <c r="A1172" t="inlineStr">
@@ -26773,9 +26743,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D1172" t="inlineStr"/>
-      <c r="E1172" t="inlineStr"/>
-      <c r="F1172" t="inlineStr"/>
       <c r="G1172" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -26798,9 +26765,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D1173" t="inlineStr"/>
-      <c r="E1173" t="inlineStr"/>
-      <c r="F1173" t="inlineStr"/>
       <c r="G1173" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -26823,9 +26787,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D1174" t="inlineStr"/>
-      <c r="E1174" t="inlineStr"/>
-      <c r="F1174" t="inlineStr"/>
       <c r="G1174" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -26848,9 +26809,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D1175" t="inlineStr"/>
-      <c r="E1175" t="inlineStr"/>
-      <c r="F1175" t="inlineStr"/>
       <c r="G1175" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -26881,7 +26839,6 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-Consul-Bocas-CFO4NARUNA-Bivolt/dp/B07HM9JL5K/ref=sr_1_1</t>
         </is>
       </c>
-      <c r="G1176" t="inlineStr"/>
     </row>
     <row r="1177">
       <c r="A1177" t="inlineStr">
@@ -26907,7 +26864,6 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-Bocas-Consul-Vidro-Bivolt/dp/B076BC7769/ref=sr_1_2</t>
         </is>
       </c>
-      <c r="G1177" t="inlineStr"/>
     </row>
     <row r="1178">
       <c r="A1178" t="inlineStr">
@@ -26933,7 +26889,540 @@
           <t>https://www.amazon.com.br/Consul-Fog%C3%A3o-bocas-Preto-esmaltada/dp/B0FM83JTS7/ref=sr_1_3</t>
         </is>
       </c>
-      <c r="G1178" t="inlineStr"/>
+    </row>
+    <row r="1179">
+      <c r="A1179" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1179" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1179" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D1179" t="inlineStr"/>
+      <c r="E1179" t="inlineStr"/>
+      <c r="F1179" t="inlineStr"/>
+      <c r="G1179" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1180">
+      <c r="A1180" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1180" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1180" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D1180" t="inlineStr"/>
+      <c r="E1180" t="inlineStr"/>
+      <c r="F1180" t="inlineStr"/>
+      <c r="G1180" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1181">
+      <c r="A1181" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1181" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1181" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D1181" t="inlineStr"/>
+      <c r="E1181" t="inlineStr"/>
+      <c r="F1181" t="inlineStr"/>
+      <c r="G1181" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1182">
+      <c r="A1182" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1182" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1182" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D1182" t="inlineStr"/>
+      <c r="E1182" t="inlineStr"/>
+      <c r="F1182" t="inlineStr"/>
+      <c r="G1182" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1183">
+      <c r="A1183" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1183" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1183" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1183" t="n">
+        <v>2012.61</v>
+      </c>
+      <c r="F1183" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Duplex-litros-Branca/dp/B07FXZ8TR6/ref=sr_1_1</t>
+        </is>
+      </c>
+      <c r="G1183" t="inlineStr"/>
+    </row>
+    <row r="1184">
+      <c r="A1184" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1184" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1184" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1184" t="n">
+        <v>2940.15</v>
+      </c>
+      <c r="F1184" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWVJ8LR/ref=sr_1_2</t>
+        </is>
+      </c>
+      <c r="G1184" t="inlineStr"/>
+    </row>
+    <row r="1185">
+      <c r="A1185" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1185" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C1185" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1185" t="n">
+        <v>2564.05</v>
+      </c>
+      <c r="F1185" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Litros-Duplex-Branca/dp/B0GFB8M9MZ/ref=sr_1_3</t>
+        </is>
+      </c>
+      <c r="G1185" t="inlineStr"/>
+    </row>
+    <row r="1186">
+      <c r="A1186" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1186" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1186" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D1186" t="inlineStr"/>
+      <c r="E1186" t="inlineStr"/>
+      <c r="F1186" t="inlineStr"/>
+      <c r="G1186" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1187">
+      <c r="A1187" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1187" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1187" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D1187" t="inlineStr"/>
+      <c r="E1187" t="inlineStr"/>
+      <c r="F1187" t="inlineStr"/>
+      <c r="G1187" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1188">
+      <c r="A1188" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1188" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1188" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D1188" t="inlineStr"/>
+      <c r="E1188" t="inlineStr"/>
+      <c r="F1188" t="inlineStr"/>
+      <c r="G1188" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1189">
+      <c r="A1189" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1189" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1189" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D1189" t="inlineStr"/>
+      <c r="E1189" t="inlineStr"/>
+      <c r="F1189" t="inlineStr"/>
+      <c r="G1189" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1190">
+      <c r="A1190" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1190" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1190" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1190" t="n">
+        <v>518.77</v>
+      </c>
+      <c r="F1190" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P2FLSR/ref=sr_1_1</t>
+        </is>
+      </c>
+      <c r="G1190" t="inlineStr"/>
+    </row>
+    <row r="1191">
+      <c r="A1191" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1191" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1191" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1191" t="n">
+        <v>484.03</v>
+      </c>
+      <c r="F1191" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Efficient-23L-ME23B/dp/B0B8KWNK12/ref=sr_1_2</t>
+        </is>
+      </c>
+      <c r="G1191" t="inlineStr"/>
+    </row>
+    <row r="1192">
+      <c r="A1192" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1192" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C1192" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1192" t="n">
+        <v>519.01</v>
+      </c>
+      <c r="F1192" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P3T3VM/ref=sr_1_3</t>
+        </is>
+      </c>
+      <c r="G1192" t="inlineStr"/>
+    </row>
+    <row r="1193">
+      <c r="A1193" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1193" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1193" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D1193" t="inlineStr"/>
+      <c r="E1193" t="inlineStr"/>
+      <c r="F1193" t="inlineStr"/>
+      <c r="G1193" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1194">
+      <c r="A1194" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1194" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1194" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D1194" t="inlineStr"/>
+      <c r="E1194" t="inlineStr"/>
+      <c r="F1194" t="inlineStr"/>
+      <c r="G1194" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1195">
+      <c r="A1195" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1195" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1195" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D1195" t="inlineStr"/>
+      <c r="E1195" t="inlineStr"/>
+      <c r="F1195" t="inlineStr"/>
+      <c r="G1195" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1196">
+      <c r="A1196" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1196" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1196" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D1196" t="inlineStr"/>
+      <c r="E1196" t="inlineStr"/>
+      <c r="F1196" t="inlineStr"/>
+      <c r="G1196" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="1197">
+      <c r="A1197" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1197" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1197" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1197" t="n">
+        <v>1237.85</v>
+      </c>
+      <c r="F1197" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-Consul-Bocas-CFO4NARUNA-Bivolt/dp/B07HM9JL5K/ref=sr_1_1</t>
+        </is>
+      </c>
+      <c r="G1197" t="inlineStr"/>
+    </row>
+    <row r="1198">
+      <c r="A1198" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1198" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1198" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1198" t="n">
+        <v>1303</v>
+      </c>
+      <c r="F1198" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-Bocas-Consul-Vidro-Bivolt/dp/B076BC7769/ref=sr_1_2</t>
+        </is>
+      </c>
+      <c r="G1198" t="inlineStr"/>
+    </row>
+    <row r="1199">
+      <c r="A1199" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1199" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C1199" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E1199" t="n">
+        <v>1131</v>
+      </c>
+      <c r="F1199" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Consul-Branco-acendimento-autom%C3%A1tico-BIVOLT/dp/B076CBHKPW/ref=sr_1_3</t>
+        </is>
+      </c>
+      <c r="G1199" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>